<commit_message>
Ledger v4 verification, group 2: [DL4] comment IDs
Checked the 16 [DL4] rows against every comment on both dockets,
downloaded October 13, 2026 (960 + 214 comments, no gaps). 14 match
(12 upgraded); the analyst's docket and distinct-text counts reproduce
exactly. 2 corrected: TP-40 (example comment does not cite Loper Bright)
and NC-17 (MACPAC's September 21 letter is posted as CMS-2026-2476-0173).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jFZZ5qaUFnBNLfBGt45ve
</commit_message>
<xml_diff>
--- a/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
+++ b/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
@@ -3065,12 +3065,12 @@
       </c>
       <c r="M35" s="12" t="inlineStr">
         <is>
-          <t>Verification F-003: v4 API meta.totalElements = 960 (CMS-2026-1916, October 8) and 214 (CMS-2026-2476, re-confirmed October 9; the 1916 re-query hit the demo key's rate limit, so 960 rests on October 8). The 961 / 213 'corrected' view and the distinct-text counts (660; 188 / 187) come from the comment analyst's files and are not in the verification summary. The snapshot date (October 7) precedes the verification dates.</t>
+          <t>Verification F-003: v4 API meta.totalElements = 960 (CMS-2026-1916, October 8) and 214 (CMS-2026-2476, re-confirmed October 9; the 1916 re-query hit the demo key's rate limit, so 960 rests on October 8). The 961 / 213 'corrected' view and the distinct-text counts (660; 188 / 187) come from the comment analyst's files and are not in the verification summary. The snapshot date (October 7) precedes the verification dates. VERIFIED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. Result: CMS-2026-1916 960 as filed / 961 corrected, 660 distinct texts in both views; CMS-2026-2476 214 / 213, 188 / 187 distinct texts. The live API totals on October 13 are still 960 and 214, so the October 7 snapshot is unchanged.</t>
         </is>
       </c>
       <c r="N35" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — raw counts confirmed October 8–9; corrected and distinct-text counts rest on the analyst's files — NEEDS VERIFICATION [DL4] Corrected and distinct-text counts are comment-analyst output, not covered by the verification files.</t>
+          <t>verified — upgraded from verified with caveat: re-checked October 13, 2026: the API reports 960 and 214 comments; the full download reproduces 961 / 213 corrected and 660 (both views) and 188 / 187 distinct texts.</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="M37" s="12" t="inlineStr">
         <is>
-          <t>Arithmetic consistent with RM-34: 960 + 1 = 961 and 214 − 1 = 213. The letter is not identified in the note or the verification files.</t>
+          <t>Arithmetic consistent with RM-34: 960 + 1 = 961 and 214 − 1 = 213. The letter is not identified in the note or the verification files. VERIFIED October 13, 2026 (verification_v4_log.md): CMS-2026-2476-0199 is addressed to the SDP rule (RIN 0938-AV69; 'published at 91 Federal Register 30400') and its text is identical word for word to CMS-2026-1916-0958 (filed July 28, 2026). Of the other ten CMS-2452-P comments that mention CMS-2449-P or the SDP rule, all are headed CMS-2452-P letters; no CMS-2449-P comment mentions CMS-2452-P, RIN 0938-AV93 or the hold harmless threshold. Matched by script.</t>
         </is>
       </c>
       <c r="N37" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's files; the letter is not identified — NEEDS VERIFICATION [DL4] The moved letter and the corrected view are not covered by the verification files.</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: the one moved letter is CMS-2026-2476-0199, the California Behavioral Health Association's CMS-2449-P letter (RIN 0938-AV69, 91 FR 30400), word for word the same as CMS-2026-1916-0958; no other misfiled letter found.</t>
         </is>
       </c>
     </row>
@@ -10841,12 +10841,12 @@
       </c>
       <c r="M143" s="12" t="inlineStr">
         <is>
-          <t>none located — negative claim, scoped at C-4 UPDATED October 11, 2026: v17 identifies the one later reference, an individual's comment, and cites it by ID; the earlier wording ('later references restate the figure rather than reproduce it') is replaced by the single located instance. The comment ID was located by the comment analyst and is not in the verification files. Previous wording: 'Later references restate the figure rather than reproduce it'</t>
+          <t>none located — negative claim, scoped at C-4 UPDATED October 11, 2026: v17 identifies the one later reference, an individual's comment, and cites it by ID; the earlier wording ('later references restate the figure rather than reproduce it') is replaced by the single located instance. The comment ID was located by the comment analyst and is not in the verification files. Previous wording: 'Later references restate the figure rather than reproduce it' VERIFIED October 13, 2026 (verification_v4_log.md): CMS-2026-2476-0079 (an individual, no organization): 'Hospitals alone stand to lose an estimated $681 billion over a ten-year period'; no source or derivation. Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. '$681 billion' appears in no other comment or attachment in either docket.</t>
         </is>
       </c>
       <c r="N143" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — NEEDS VERIFICATION [DL4] Comment ID CMS-2026-2476-0079 is on the 'citation to add after verification' list (change map, v2 list item 7); v17 now cites it.</t>
+          <t>verified as scoped — re-checked October 13, 2026: comment CMS-2026-2476-0079, an individual's, restates $681 billion as a hospital loss with no source; it is the only comment in either docket with $681 billion.</t>
         </is>
       </c>
     </row>
@@ -12281,12 +12281,12 @@
       </c>
       <c r="M163" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-004); the letters were not re-read in the verification files. The $183B match is arithmetic against SB-09. The verification summary notes CBO's $182.7B is its estimate of the law as enacted (July 21, 2025 table headed 'As enacted on July 4, 2025'), so a 'pre-enactment' label for $183B does not describe it. TP-18 is one of these comments (-0029).</t>
+          <t>Located by the comment analyst (F-004); the letters were not re-read in the verification files. The $183B match is arithmetic against SB-09. The verification summary notes CBO's $182.7B is its estimate of the law as enacted (July 21, 2025 table headed 'As enacted on July 4, 2025'), so a 'pre-enactment' label for $183B does not describe it. TP-18 is one of these comments (-0029). VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026); matched by script. -0201 (Arizona AHCCCS) p. 1: 'roughly $183 billion to $191 billion in federal savings'; -0029 (Georgetown CCF) p. 1: $191.1 billion in reduced federal spending (CBO); -0097, -0187, -0195 (same text): 'pre-enactment estimates … $183 billion of reductions'; -0126 (Pennsylvania DHS) p. 1: '$183 billion reduction in federal deficits'; -0089 (HAP) p. 1: '$183 billion associated with the statutory changes'.</t>
         </is>
       </c>
       <c r="N163" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's findings; letters not re-read — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-004).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: each cited comment gives CBO's Section 71115 figure as stated ($191.1 billion or $183 billion, under different labels; -0201 as a range); the $183B/$182.7B match is [I] arithmetic (SB-09).</t>
         </is>
       </c>
     </row>
@@ -12353,12 +12353,12 @@
       </c>
       <c r="M164" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-016); keyword counts are approximate by the note's own statement (App. I). Not re-checked in the verification files.</t>
+          <t>Located by the comment analyst (F-016); keyword counts are approximate by the note's own statement (App. I). Not re-checked in the verification files. VERIFIED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. Patterns from count_themes.py ('$510' or '$510.1' followed by 'billion' or 'B'; '$149' or '$149.4' likewise). Exact '149.4' alone: 73 comments, 49 distinct. Examples: -0902 (Lee County Community Hospital) p. 1 cites $510.1 billion and CBO's $149.4 billion; -0128 (AAFP) p. 5 cites about $510 billion against CBO; -0756 (Allegheny Health Network) p. 2 cites $510 billion and $149.4 billion.</t>
         </is>
       </c>
       <c r="N164" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's keyword counts; approximate — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-016).</t>
+          <t>verified with caveat — upgraded from single-source; keyword counts stay approximate: re-checked October 13, 2026: with the analyst's patterns, $510 billion is in 124 CMS-2449-P comments (88 distinct texts) and $149 billion in 87 (63 distinct), in both views; the three examples match.</t>
         </is>
       </c>
     </row>
@@ -13865,12 +13865,12 @@
       </c>
       <c r="M185" s="12" t="inlineStr">
         <is>
-          <t>Pin cite recorded from the note. The letter was not re-read for this ledger. Replaces TP-16, which described this as the letter's 'central argument' UPDATED October 11, 2026: v17 moves the FAH point to App. F, cites the comment ID and p. 2 (the earlier pin cite was p. 1), and states what FAH asked for (the rate for the cap test). The comment ID and page were located by the analyst (F-019) and are on the 'citation to add after verification' list. The letter was not re-read for this ledger. Previous wording: 'The Federation of American Hospitals, in its July 21 comment letter on the SDP rule, argued that CMS should account for the provider taxes that partly finance SDPs'</t>
+          <t>Pin cite recorded from the note. The letter was not re-read for this ledger. Replaces TP-16, which described this as the letter's 'central argument' UPDATED October 11, 2026: v17 moves the FAH point to App. F, cites the comment ID and p. 2 (the earlier pin cite was p. 1), and states what FAH asked for (the rate for the cap test). The comment ID and page were located by the analyst (F-019) and are on the 'citation to add after verification' list. The letter was not re-read for this ledger. Previous wording: 'The Federation of American Hospitals, in its July 21 comment letter on the SDP rule, argued that CMS should account for the provider taxes that partly finance SDPs' VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026). FAH's p. 2 asks CMS to 'calculate the total payment rate to reflect the actual effect of SDPs on provider payment, including by accounting for the provider taxes that partially finance them'; pp. 8–9 develop the point. Matched by script.</t>
         </is>
       </c>
       <c r="N185" s="12" t="inlineStr">
         <is>
-          <t>single-source - pin cite located by the comment analyst; letter not re-read — NEEDS VERIFICATION [DL4] Comment CMS-2026-1916-0676, p. 2 is on the 'citation to add after verification' list (change map, v2 list item 1).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: comment CMS-2026-1916-0676 (Federation of American Hospitals), p. 2 of 45, asks CMS to calculate the total payment rate accounting for the provider taxes that partly finance SDPs.</t>
         </is>
       </c>
     </row>
@@ -14441,12 +14441,12 @@
       </c>
       <c r="M193" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-013); the letters were not re-read in the verification files. Bears on TP-24: most commenters describe the $220.3B as a payment cut, but none reaches $56.6B.</t>
+          <t>Located by the comment analyst (F-013); the letters were not re-read in the verification files. Bears on TP-24: most commenters describe the $220.3B as a payment cut, but none reaches $56.6B. VERIFIED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. '220.3' appears in -0049 (ACOG) p. 2, -0085 (PAR) p. 1, -0190 (NJHA) pp. 2, 7, -0201 (Arizona AHCCCS) p. 1 and -0212 p. 6; -0212 p. 6: 'Netting the tax savings against the payment reduction, CMS projects a net transfer away from providers of approximately $220.3 billion.' '56.6' appears in no CMS-2452-P comment.</t>
         </is>
       </c>
       <c r="N193" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's findings; letters not re-read — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-013).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: exactly five CMS-2452-P comments (five distinct texts, both views) cite $220.3 billion; -0049, -0085, -0190 and -0201 as a payment cut, -0212 as net of lower taxes; none has $56.6 billion.</t>
         </is>
       </c>
     </row>
@@ -14585,12 +14585,12 @@
       </c>
       <c r="M195" s="12" t="inlineStr">
         <is>
-          <t>Verification summary (F-024): the court ruling could not be read (courtlistener.com refused; govinfo's court-opinion search found no match); CHAT's 'permanently enjoined' description is secondary. Round 3 item 6 found no source for 'set aside'. The case caption is unverifiable. See RM-26.</t>
+          <t>Verification summary (F-024): the court ruling could not be read (courtlistener.com refused; govinfo's court-opinion search found no match); CHAT's 'permanently enjoined' description is secondary. Round 3 item 6 found no source for 'set aside'. The case caption is unverifiable. See RM-26. VERIFIED October 13, 2026, comment limb (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026). CHAT says at p. 13 that a federal district court in Texas 'has permanently enjoined CMS from imposing this interpretation on Texas', citing Texas v. Centers for Medicare &amp; Medicaid Svcs., 805 F. Supp. 3d 734 (E.D. Tex. 2025) (n. 22), and at p. 14 refers to CMS's Fifth Circuit appeal on Texas LPPFs. The ruling itself was not read (courtlistener.com refused).</t>
         </is>
       </c>
       <c r="N195" s="12" t="inlineStr">
         <is>
-          <t>single-source — CHAT's description; the ruling was not read — NEEDS VERIFICATION [DL4] Comment CMS-2026-2476-0114, pp. 13–14 is on the 'citation to add after verification' list (change map, v2 list item 7: F-024).</t>
+          <t>single-source — CHAT's description; the ruling was not read; re-checked October 13, 2026: comment CMS-2026-2476-0114, pp. 13–14 of 14, matches (permanent injunction; 805 F. Supp. 3d 734).</t>
         </is>
       </c>
     </row>
@@ -14657,12 +14657,12 @@
       </c>
       <c r="M196" s="12" t="inlineStr">
         <is>
-          <t>The CMS limb is the wording recorded at CE-48 (R1012; range sentence at CE-31). The commenter limb was located by the analyst (F-009) and not re-read in the verification files.</t>
+          <t>The CMS limb is the wording recorded at CE-48 (R1012; range sentence at CE-31). The commenter limb was located by the analyst (F-009) and not re-read in the verification files. VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026). MHA p. 10: CMS 'assumes that 65 percent of state directed payment spending is financed with provider taxes'. 91 FR 46592 (govinfo PDF): 55 to 75 percent 'of SDP spending'; 65 percent as 'the percentage of SDPs funded through provider taxes'. Both matched by script.</t>
         </is>
       </c>
       <c r="N196" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — CMS wording confirmed (CE-48); commenter's wording located only — NEEDS VERIFICATION [DL4] Comment CMS-2026-2476-0204, p. 10 is on the 'citation to add after verification' list (change map, v2 list item 7: F-009).</t>
+          <t>verified — upgraded from verified with caveat: re-checked October 13, 2026: comment CMS-2026-2476-0204 (Minnesota Hospital Association), p. 10, gives the 65 percent as a share of SDP spending; CMS's wording at 91 FR 46592 also matches.</t>
         </is>
       </c>
     </row>
@@ -14729,12 +14729,12 @@
       </c>
       <c r="M197" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-020). The verification summary notes F-020 'was not re-checked or edited'. The CMS figures themselves are at CE-03.</t>
+          <t>Located by the comment analyst (F-020). The verification summary notes F-020 'was not re-checked or edited'. The CMS figures themselves are at CE-03. VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026); matched by script. Table 20 (91 FR 30452, page image) has no total row; its ten cells sum to 264.7, and CMS's text gives $264.4 billion.</t>
         </is>
       </c>
       <c r="N197" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's finding; letters not re-read — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-020).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: comments CMS-2026-1916-0417 p. 6, -0509 p. 38 and -0648 p. 3 each give the state figure as $264.4 billion; Table 20's cells sum to $264.7 billion.</t>
         </is>
       </c>
     </row>
@@ -14801,12 +14801,12 @@
       </c>
       <c r="M198" s="12" t="inlineStr">
         <is>
-          <t>CMS's figures are confirmed (verification summary, F-010: $90.9B at 91 FR 46593, −$136.1B at 46594). The commenters' letters were not re-read; the last two readings are the note's [I] interpretation ('appears to').</t>
+          <t>CMS's figures are confirmed (verification summary, F-010: $90.9B at 91 FR 46593, −$136.1B at 46594). The commenters' letters were not re-read; the last two readings are the note's [I] interpretation ('appears to'). VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026); matched by script. -0145 p. 3: $90.9 billion federal after the SDP interaction; p. 4: $136.1 billion provider reduction in the high-impact scenario. -0093 p. 8: $90.9 billion. -0101 (AHIP) p. 1: 'CMS estimates that the reduction would be $154.9 billion after accounting for separate changes'; at 91 FR 46592 the $154.9 billion is how much smaller federal reductions are, not what is left. -0091 (BCBSA) p. 27: $9.1 billion to $90.9 billion, omitting the $191.8 billion high-savings figure.</t>
         </is>
       </c>
       <c r="N198" s="12" t="inlineStr">
         <is>
-          <t>single-source — CMS figures confirmed (F-010); the commenters' letters were not re-read — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-010, F-017).</t>
+          <t>verified with caveat — upgraded from single-source; the last two readings remain [I] ('appears to'): re-checked October 13, 2026: comments CMS-2026-2476-0145 pp. 3–4, -0093 p. 8, -0101 p. 1 and -0091 p. 27 say what the row describes.</t>
         </is>
       </c>
     </row>
@@ -14873,12 +14873,12 @@
       </c>
       <c r="M199" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-026); not re-read in the verification files. Round 3 item 5 could not confirm that Ohio's Medicaid agency (comment 1916-0209) makes the same argument (its comment centres on crisis-service reconciliation), so v17 names Virginia alone.</t>
+          <t>Located by the comment analyst (F-026); not re-read in the verification files. Round 3 item 5 could not confirm that Ohio's Medicaid agency (comment 1916-0209) makes the same argument (its comment centres on crisis-service reconciliation), so v17 names Virginia alone. VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026). Virginia DMAS, p. 3, heading 'CMS Should Not Default Payment Limits to State Plan Rates for Services Without a Medicare Equivalent'; matched by script. (The default it objects to is for services with no Medicare rate, not the cost-paid hospitals at RM-18.)</t>
         </is>
       </c>
       <c r="N199" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's finding; letter not re-read — NEEDS VERIFICATION [DL4] Comment CMS-2026-1916-0755, p. 3 is on the 'citation to add after verification' list (change map, v2 list item 7: F-026).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: comment CMS-2026-1916-0755 (Virginia Department of Medical Assistance Services), p. 3 of 5, matches.</t>
         </is>
       </c>
     </row>
@@ -14945,12 +14945,12 @@
       </c>
       <c r="M200" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-021); not re-read in the verification files. ASPE's estimates are at TP-10 to TP-14.</t>
+          <t>Located by the comment analyst (F-021); not re-read in the verification files. ASPE's estimates are at TP-10 to TP-14. VERIFIED October 13, 2026 (verification_v4_log.md): regulations.gov (API and attachment, downloaded October 13, 2026). Paragon 'strongly support[s] the proposed rule’s core provisions' (p. 1) and at p. 2 cites ASPE's finding that the reforms reduce non-Medicaid prices by up to 3.5 percent ($502 billion to $875 billion over 2025–2034), n. 3 citing ASPE, August 12, 2026. Matched by script.</t>
         </is>
       </c>
       <c r="N200" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's finding; letter not re-read — NEEDS VERIFICATION [DL4] Comment CMS-2026-2476-0130, p. 2 is on the 'citation to add after verification' list (change map, v2 list item 7: F-021).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: comment CMS-2026-2476-0130 (Paragon Health Institute), which supports the rule, cites ASPE's August 12, 2026 estimates at p. 2.</t>
         </is>
       </c>
     </row>
@@ -15017,12 +15017,12 @@
       </c>
       <c r="M201" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-018); keyword counts are approximate by the note's own statement. Not re-read in the verification files.</t>
+          <t>Located by the comment analyst (F-018); keyword counts are approximate by the note's own statement. Not re-read in the verification files. VERIFIED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. Pattern from count_themes.py ('net_of_tax') and a wider one give the same 12 comments, 9 distinct texts (about 11 / about 8 in v17). AHA p. 11 urges 'a net-of-tax methodology'; SCDHHS p. 3 asks CMS to 'calculate the Medicaid rate ceiling net of provider taxes'; -0369, -0476, -0808, -0437, -0424 and -0787 carry the heading 'Medicaid Reimbursement Should be Calculated Net of Provider Taxes'.</t>
         </is>
       </c>
       <c r="N201" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's findings; approximate keyword count — NEEDS VERIFICATION [DL4] Comment IDs on the 'citation to add after verification' list (change map, v2 list item 7: F-018).</t>
+          <t>verified with caveat — upgraded from single-source; keyword count stays approximate: re-checked October 13, 2026: AHA (-0928 p. 11), South Carolina DHHS (-0923 p. 3) and the six templates ask CMS to net provider taxes; the count is 12 comments, 9 distinct texts, in both views.</t>
         </is>
       </c>
     </row>
@@ -15233,12 +15233,12 @@
       </c>
       <c r="M204" s="12" t="inlineStr">
         <is>
-          <t>Located by the comment analyst (F-028); keyword counts are approximate. Not re-read in the verification files. The related negative (no comment reports a filed suit) is at NC-20.</t>
+          <t>Located by the comment analyst (F-028); keyword counts are approximate. Not re-read in the verification files. The related negative (no comment reports a filed suit) is at NC-20. CORRECTED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. 'Loper Bright' appears nowhere in CMS-2026-1916-0407 (Legal Action Center and 39 co-signers), which argues statutory authority and reasoned decision-making. Comments that do cite it include CMS-2026-1916-0288 (Premier Inc.), p. 2, and -0392 (CVS Health), p. 4. Counts: 44 / 23 (CMS-2449-P) and 11 / 9 (CMS-2452-P), as filed and corrected, against v17's about 40 / about 20 and about 11 / about 8.</t>
         </is>
       </c>
       <c r="N204" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment analyst's keyword counts; approximate — NEEDS VERIFICATION [DL4] Comment CMS-2026-1916-0407, p. 1 is on the 'citation to add after verification' list (change map, v2 list item 7: F-028).</t>
+          <t>corrected — the example comment CMS-2026-1916-0407 does not cite Loper Bright; at p. 1 it says: “We believe CMS has far exceeded its statutory authority to interpret and implement Public Law 119-21 (H.R. 1) and the Social Security Act”. The counts hold (re-checked October 13, 2026: Loper Bright in 44 CMS-2449-P comments, 23 distinct; 11 CMS-2452-P comments, 9 distinct). v17 must move or replace the example (see verification_v4_log.md). Base status was single-source.</t>
         </is>
       </c>
     </row>
@@ -19409,12 +19409,12 @@
       </c>
       <c r="M262" s="12" t="inlineStr">
         <is>
-          <t>Limits stated in App. G: the record is a snapshot; text search of scanned pages can miss figures printed as images; letters published only on submitters' sites are not in the docket; letters were matched by organization name. Replaces the C-4 scope (28 posted comments and seven letters on submitters' own sites; RM-22, NC-04). The comment-analyst output was not re-run in the verification files. The first sentence is tagged [E] and the 'found in none of them' limb [I] in v17.</t>
+          <t>Limits stated in App. G: the record is a snapshot; text search of scanned pages can miss figures printed as images; letters published only on submitters' sites are not in the docket; letters were matched by organization name. Replaces the C-4 scope (28 posted comments and seven letters on submitters' own sites; RM-22, NC-04). The comment-analyst output was not re-run in the verification files. The first sentence is tagged [E] and the 'found in none of them' limb [I] in v17. CORRECTED October 13, 2026 (verification_v4_log.md): Counts recomputed October 13, 2026 on the full download (CMS-2026-1916: 960 comments, 892 attachments; CMS-2026-2476: 214 comments, 202 attachments; the collector's report showed no gaps) with the analyst's own extract_comment_text.py and comment_text_utils.cluster (shingle Jaccard 0.5), and the keyword patterns in count_themes.py where one exists. CMS-2026-2476-0173 (posted September 22, 2026, inside the October 7 snapshot) is MACPAC's letter dated September 21, 2026; regulations.gov carries no organization or name for it, and the analyst's file tags it 'individual'. -0148 (Children's Hospital Association), -0116 (NAMD) and -0109 (Texas Hospital Association) are dated September 21, 2026; -0057 (California Hospital Association) is dated September 18, 2026. None of the five contains $681 billion. No posted CMS-2452-P comment names the Illinois Health and Hospital Association or the Illinois Attorney General in its organization field or opening text.</t>
         </is>
       </c>
       <c r="N262" s="12" t="inlineStr">
         <is>
-          <t>single-source — comment-analyst search; not covered by the verification files — NEEDS VERIFICATION [DL4] Comment IDs CMS-2026-2476-0079, -0148, -0116, -0109 and -0057 are on the 'citation to add after verification' list (change map, v2 list item 7: F-014, F-002); v17 now cites them.</t>
+          <t>corrected — MACPAC's September 21, 2026 letter is posted, as comment CMS-2026-2476-0173 (organization field blank): “The Medicaid and CHIP Payment and Access Commission (MACPAC) appreciates the opportunity to comment on the notice of proposed rulemaking” (p. 1). So five of the six letters are posted, not four. The $681 billion limb matches (re-checked October 13, 2026: only -0079 in either docket); no Illinois Health and Hospital Association or Illinois Attorney General letter found. v17 must change App. G (see verification_v4_log.md). Base status was single-source.</t>
         </is>
       </c>
     </row>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. Checked so far: [CM] Federal Register pinpoints; 17 of the 91 flagged rows. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 12 rows match and lose the flag (8 upgraded, for example single-source to verified); 4 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 0 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 2 rows with two tags were resolved for one tag only and keep the other tag's flag (counted above by the result for the resolved tag). No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
+          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. Checked so far: [CM] Federal Register pinpoints, [DL4] comment IDs; 33 of the 91 flagged rows. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 26 rows match and lose the flag (20 upgraded, for example single-source to verified); 6 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 0 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 2 rows with two tags were resolved for one tag only and keep the other tag's flag (counted above by the result for the resolved tag). No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ledger v4 verification, group 3: [DL3] re-check list
Checked the 60 [DL3] rows (secs. 3-5 sources first). Statute (govinfo),
Federal Register, bill status and journal sources: RM-16, RM-17, RM-28,
RM-30, NC-15, AC-07, AC-11 and AC-15 match; RM-18's statutory page is
added; AC-08 and FG-08 are corrected (the no-trend finding holds for the
average annual percent change only). 47 rows stay flagged as blocked
(KFF, POLITICO, HFMA, ASPE, GAO, reginfo.gov and others refused by the
network policy) and RM-26 as not found.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jFZZ5qaUFnBNLfBGt45ve
</commit_message>
<xml_diff>
--- a/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
+++ b/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
@@ -1337,12 +1337,12 @@
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>RE-DATED in the Sept 22, 2026 currency check: both RINs absent from the Sept 21, 2026 list. RIN 0938-AV69 confirmed on reginfo.gov as CMS-2449-P; 0938-AV93 is CMS-2452-P. The original Sept 5, 2026 check (P1 output, both RINs) is superseded as to date only. CMS-2450 (RIN 0938-AV70), a separate rule, has been under review since May 12, 2026 and is disclosed in the status box; see M-6 UPDATED October 11, 2026: v17 states no White House review status for either RIN: sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading 'Status as of [DATE]: White House review, CMS-2450 …' has no text under it. The September 21, 2026 check is therefore stale against the October 2026 draft and is not restated in the note.</t>
+          <t>RE-DATED in the Sept 22, 2026 currency check: both RINs absent from the Sept 21, 2026 list. RIN 0938-AV69 confirmed on reginfo.gov as CMS-2449-P; 0938-AV93 is CMS-2452-P. The original Sept 5, 2026 check (P1 output, both RINs) is superseded as to date only. CMS-2450 (RIN 0938-AV70), a separate rule, has been under review since May 12, 2026 and is disclosed in the status box; see M-6 UPDATED October 11, 2026: v17 states no White House review status for either RIN: sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading 'Status as of [DATE]: White House review, CMS-2450 …' has no text under it. The September 21, 2026 check is therefore stale against the October 2026 draft and is not restated in the note. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
         </is>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see C-6; perishable — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3–4; App. I); re-run the OIRA list check at the date the note fills in.</t>
+          <t>verified as scoped — see C-6; perishable — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3–4; App. I); re-run the OIRA list check at the date the note fills in. blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
-          <t>none located in the available outputs UPDATED October 11, 2026: v17 attributes the rural cutoff to the statute, states it as July 4, 2025 (the date of enactment) and adds that rural hospitals' grandfathered payments phase down from 2028 like others'. The statute's page for the rural rule is on the re-check list. Previous wording: 'Rural hospitals receive a more generous grandfathering window: approval or documented good-faith effort by date of enactment, against before May 1, 2025 for all others'</t>
+          <t>none located in the available outputs UPDATED October 11, 2026: v17 attributes the rural cutoff to the statute, states it as July 4, 2025 (the date of enactment) and adds that rural hospitals' grandfathered payments phase down from 2028 like others'. The statute's page for the rural rule is on the re-check list. Previous wording: 'Rural hospitals receive a more generous grandfathering window: approval or documented good-faith effort by date of enactment, against before May 1, 2025 for all others' VERIFIED October 13, 2026 (verification_v4_log.md): P.L. 119-21, govinfo HTML (PLAW-119publ21), § 71116(b) at 139 Stat. 303, matched by script; the Act's date line is July 4, 2025. The statute also limits grandfathering to the rating period occurring within 180 days of enactment; CMS reads that as a criterion for every grandfathered SDP (91 FR 30418), so v17's sentence is a fair simplification.</t>
         </is>
       </c>
       <c r="N17" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Statutory page for Section 71116's rural rule is on the decision-log re-check list (sec. 8; App. B).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: P.L. 119-21 § 71116(b), 139 Stat. 303, gives rural hospitals until the date of enactment (July 4, 2025) against before May 1, 2025, and the 10-point annual phase-down from 2028 applies to all grandfathered payments.</t>
         </is>
       </c>
     </row>
@@ -1841,12 +1841,12 @@
       </c>
       <c r="M18" s="12" t="inlineStr">
         <is>
-          <t>none located in the available outputs UPDATED October 11, 2026: v17 attributes the definition to the statute (Section 71116) and describes the first class as rural acute care hospitals paid under Medicare's inpatient prospective payment system; the earlier wording was 'rural (d) hospitals'. Previous wording: 'The rural definition covers rural (d) hospitals, critical access hospitals, sole community hospitals, Medicare-dependent small rural hospitals, low-volume hospitals and rural emergency hospitals'</t>
+          <t>none located in the available outputs UPDATED October 11, 2026: v17 attributes the definition to the statute (Section 71116) and describes the first class as rural acute care hospitals paid under Medicare's inpatient prospective payment system; the earlier wording was 'rural (d) hospitals'. Previous wording: 'The rural definition covers rural (d) hospitals, critical access hospitals, sole community hospitals, Medicare-dependent small rural hospitals, low-volume hospitals and rural emergency hospitals' VERIFIED October 13, 2026 (verification_v4_log.md): P.L. 119-21, govinfo HTML (PLAW-119publ21), § 71116(d)(2) at 139 Stat. 304, matched by script. The first class is a subsection (d) hospital located in, or treated as located in, a rural area or a rural census tract; v17's 'rural acute care hospitals paid under Medicare's inpatient prospective payment system' is a fair paraphrase.</t>
         </is>
       </c>
       <c r="N18" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Statutory page for the rural definition (Section 71116) is on the decision-log re-check list (sec. 8; App. B).</t>
+          <t>verified — upgraded from single-source: re-checked October 13, 2026: P.L. 119-21 § 71116(d)(2), 139 Stat. 304, lists the six classes (rural subsection (d) hospitals; critical access, sole community, Medicare-dependent small rural, low-volume and rural emergency hospitals).</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
       </c>
       <c r="M19" s="12" t="inlineStr">
         <is>
-          <t>none located in the available outputs UPDATED October 11, 2026: v17 cites 91 FR 30450 for the default and adds [I] that it 'may leave little or no room for SDPs above base rates' (AC-16). Previous wording: 'Critical access, freestanding children's and certain cancer hospitals are cost-reimbursed with no published Medicare rate, so the payment limit defaults to the State plan rate' CORRECTED October 13, 2026 (verification_v4_log.md): read 91 FR 30414 and 30450 in the CMS-2449-P, govinfo PDF (FR Doc. 2026-10292). At 30414 CMS lists CAHs, certain cancer hospitals and freestanding children's hospitals as paid by Medicare on a cost basis and proposes that the most recent Medicare cost report serve as the basis for the total published Medicare payment rate and so the SDP payment limit; it limits the state plan approved rate to providers not paid by Medicare at all, and says the payment limit for cost-paid providers would default to the State plan approved rate only under an alternative it did not propose. 91 FR 30450 (RIA) gives the general rule: the limit is the State plan approved rate where no total published Medicare payment rate exists. v17's claim that the three hospital types' cap defaults to the state plan rate, and AC-16's [I] reading built on it, do not match the proposal.</t>
+          <t>none located in the available outputs UPDATED October 11, 2026: v17 cites 91 FR 30450 for the default and adds [I] that it 'may leave little or no room for SDPs above base rates' (AC-16). Previous wording: 'Critical access, freestanding children's and certain cancer hospitals are cost-reimbursed with no published Medicare rate, so the payment limit defaults to the State plan rate' CORRECTED October 13, 2026 (verification_v4_log.md): read 91 FR 30414 and 30450 in the CMS-2449-P, govinfo PDF (FR Doc. 2026-10292). At 30414 CMS lists CAHs, certain cancer hospitals and freestanding children's hospitals as paid by Medicare on a cost basis and proposes that the most recent Medicare cost report serve as the basis for the total published Medicare payment rate and so the SDP payment limit; it limits the state plan approved rate to providers not paid by Medicare at all, and says the payment limit for cost-paid providers would default to the State plan approved rate only under an alternative it did not propose. 91 FR 30450 (RIA) gives the general rule: the limit is the State plan approved rate where no total published Medicare payment rate exists; the statute says the same at § 71116(a), 139 Stat. 303 (re-check-list part, matched by script). v17's claim that the three hospital types' cap defaults to the state plan rate, and AC-16's [I] reading built on it, do not match the proposal.</t>
         </is>
       </c>
       <c r="N19" s="12" t="inlineStr">
         <is>
-          <t>corrected — source says CMS proposes, for hospitals Medicare pays on cost: “we propose to use the most recent and complete Medicare cost report … for the purpose of establishing the prospective SDP payment limit” (91 FR 30414). The state plan rate default for these hospitals is an alternative CMS considered and did not propose (91 FR 30414); 91 FR 30450 states the general default where no Medicare rate exists. v17 must rewrite sec. 8, rural ¶2 (see verification_v4_log.md). Base status was single-source. Still open — NEEDS VERIFICATION [DL3] The cost-paid cap default also sits on the citation-to-add list with Section 71116 (change map, v2 list item 2); the statutory page is still to add.</t>
+          <t>corrected — source says CMS proposes, for hospitals Medicare pays on cost: “we propose to use the most recent and complete Medicare cost report … for the purpose of establishing the prospective SDP payment limit” (91 FR 30414). The state plan rate default for these hospitals is an alternative CMS considered and did not propose (91 FR 30414); 91 FR 30450 states the general default where no Medicare rate exists. v17 must rewrite sec. 8, rural ¶2 (see verification_v4_log.md). Base status was single-source. Re-check-list part (re-checked October 13, 2026): the statute's default to the state plan rate, where no total published Medicare rate exists, is P.L. 119-21 § 71116(a), 139 Stat. 303.</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2273,12 @@
       </c>
       <c r="M24" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-6. The agenda entry scopes CMS-2450 to program integrity and enrollment and retains state directed payments and payment and access requirements in its abstract; no official description of its SDP content exists beyond that abstract, and no source ties it to the CMS-2449-P/CMS-2452-P interaction. Two EO 12866 meetings were held, both with home-care and HCBS groups EXTERNAL VERIFICATION, September 27, 2026 (D-16): the reginfo.gov review record for RIN 0938-AV70 (rrid 1379863) shows CMS-2450 received at OIRA on 05/12/2026, matching the status box's 'since May 12, 2026' UPDATED October 11, 2026: v17 states the rule is 'under White House review since May 12, 2026' and that its agenda entry states an intent to rescind or revise parts of CMS's 2024 managed care rule, including SDP requirements (sec. 9 item 4), and gives the RIN in App. I. The May 12 date was externally verified at D-16 (September 27, 2026) but sits on the decision-log re-check list.</t>
+          <t>Monitored at M-6. The agenda entry scopes CMS-2450 to program integrity and enrollment and retains state directed payments and payment and access requirements in its abstract; no official description of its SDP content exists beyond that abstract, and no source ties it to the CMS-2449-P/CMS-2452-P interaction. Two EO 12866 meetings were held, both with home-care and HCBS groups EXTERNAL VERIFICATION, September 27, 2026 (D-16): the reginfo.gov review record for RIN 0938-AV70 (rrid 1379863) shows CMS-2450 received at OIRA on 05/12/2026, matching the status box's 'since May 12, 2026' UPDATED October 11, 2026: v17 states the rule is 'under White House review since May 12, 2026' and that its agenda entry states an intent to rescind or revise parts of CMS's 2024 managed care rule, including SDP requirements (sec. 9 item 4), and gives the RIN in App. I. The May 12 date was externally verified at D-16 (September 27, 2026) but sits on the decision-log re-check list. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov could not be fetched (www.reginfo.gov refused). The federalregister.gov API (reachable) lists no Federal Register document under RIN 0938-AV70.</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see M-6; perishable, and the rule's text remains non-public — NEEDS VERIFICATION [DL3] CMS-2450 (RIN 0938-AV70), its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I).</t>
+          <t>verified as scoped — see M-6; perishable, and the rule's text remains non-public — NEEDS VERIFICATION [DL3] CMS-2450 (RIN 0938-AV70), its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-6, the same trigger as RM-23; this row restates the agenda-entry finding as a forward-looking monitoring item, not a new claim UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Publication of CMS-2450 would materially change the exposure picture; its agenda entry states an intent to rescind or revise provisions of the 2024 managed care rule, which include requirements governing state directed payments'</t>
+          <t>Monitored at M-6, the same trigger as RM-23; this row restates the agenda-entry finding as a forward-looking monitoring item, not a new claim UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Publication of CMS-2450 would materially change the exposure picture; its agenda entry states an intent to rescind or revise provisions of the 2024 managed care rule, which include requirements governing state directed payments' BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov could not be fetched (www.reginfo.gov refused). The federalregister.gov API (reachable) lists no Federal Register document under RIN 0938-AV70.</t>
         </is>
       </c>
       <c r="N25" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see M-6; conditional on publication — NEEDS VERIFICATION [DL3] CMS-2450, its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I).</t>
+          <t>verified as scoped — see M-6; conditional on publication — NEEDS VERIFICATION [DL3] CMS-2450, its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later'</t>
+          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later' BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) articles could not be fetched: the proxy refused both hosts.</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>single-source — two outlets now cited in the note but neither re-read for this ledger; the dollar detail rests on the reference case at M-7 — NEEDS VERIFICATION [DL3] Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) are on the decision-log re-check list (sec. 9 item 5); neither was re-read for this ledger.</t>
+          <t>single-source — two outlets now cited in the note but neither re-read for this ledger; the dollar detail rests on the reference case at M-7 — NEEDS VERIFICATION [DL3] Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) are on the decision-log re-check list (sec. 9 item 5); neither was re-read for this ledger. blocked: www.texastribune.org; www.fiercehealthcare.com (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -2489,12 +2489,12 @@
       </c>
       <c r="M27" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-8. A reported December 2025 Eleventh Circuit decision upholding the 2023 bulletin, which would create a circuit split, is single-source and unverified, and is not in the note UPDATED October 11, 2026: The earlier wording ('the district court set aside the relevant 2024 rule provisions and 2023–2024 CMS bulletins in September 2025'; appeal about redistribution arrangements) is no longer a note claim: Round 3 item 6 found no source for 'set aside', the 2024 provisions, the 2023–2024 guidance or September 2025, and the [E] tag was unsupported. The note now attributes the ruling's terms to CHAT. The court ruling and the appeal could not be read (courtlistener.com blocked; govinfo has no opinion; no Fifth Circuit opinion at the court's standard paths). Previous wording: 'A decision in Fifth Circuit No. 25-40766 would materially change the exposure picture; the appeal concerns whether CMS may treat redistribution arrangements among taxed providers as hold harmless arrangements, and the district court set aside the relevant 2024 rule provisions and 2023–2024 CMS bulletins in September 2025'</t>
+          <t>Monitored at M-8. A reported December 2025 Eleventh Circuit decision upholding the 2023 bulletin, which would create a circuit split, is single-source and unverified, and is not in the note UPDATED October 11, 2026: The earlier wording ('the district court set aside the relevant 2024 rule provisions and 2023–2024 CMS bulletins in September 2025'; appeal about redistribution arrangements) is no longer a note claim: Round 3 item 6 found no source for 'set aside', the 2024 provisions, the 2023–2024 guidance or September 2025, and the [E] tag was unsupported. The note now attributes the ruling's terms to CHAT. The court ruling and the appeal could not be read (courtlistener.com blocked; govinfo has no opinion; no Fifth Circuit opinion at the court's standard paths). Previous wording: 'A decision in Fifth Circuit No. 25-40766 would materially change the exposure picture; the appeal concerns whether CMS may treat redistribution arrangements among taxed providers as hold harmless arrangements, and the district court set aside the relevant 2024 rule provisions and 2023–2024 CMS bulletins in September 2025' NOT FOUND October 13, 2026 (verification_v4_log.md): www.ca5.uscourts.gov opinion search (published and unpublished opinions and orders, 1996 to present) returns 0 results for '25-40766' and for '"local provider participation"'. That is consistent with a pending appeal but does not confirm the number or the June 24, 2026 status; the docket sheet is on PACER. courtlistener.com was refused.</t>
         </is>
       </c>
       <c r="N27" s="12" t="inlineStr">
         <is>
-          <t>single-source — CHAT's description (comment 2476-0114); case caption and appeal number rest on an unverified research note — NEEDS VERIFICATION [DL3] Fifth Circuit No. 25-40766 and its June 24, 2026 status (research note, unverified) are on the decision-log re-check list (sec. 9 item 6).</t>
+          <t>single-source — CHAT's description (comment 2476-0114); case caption and appeal number rest on an unverified research note — NEEDS VERIFICATION [DL3] Fifth Circuit No. 25-40766 and its June 24, 2026 status (research note, unverified) are on the decision-log re-check list (sec. 9 item 6). not found (re-checked October 13, 2026): the Fifth Circuit's opinion search has no opinion or order under No. 25-40766; the docket is on PACER, which was not reachable.</t>
         </is>
       </c>
     </row>
@@ -2633,12 +2633,12 @@
       </c>
       <c r="M29" s="12" t="inlineStr">
         <is>
-          <t>Replaces RM-07, whose first step ('6.0% now') the note no longer states: a state whose July 4, 2025 level was below 6.0% starts below it. Sequencing consistent with RM-08 (expansion states only) and RM-29 (NF and ICF/IID exempt). No corroborating source located in the available outputs UPDATED October 11, 2026: v17's source note changes the cite from 91 FR 46562 to 91 FR 46565, 46576, 46598, and defines the federal fiscal year by 31 U.S.C. 1102 (Citation check: confirmed). The statute pinpoint for the schedule itself (P.L. 119-21 § 71115) was not added to the note; the schedule's statutory page was not checked. VERIFIED October 13, 2026, [CM] part (verification_v4_log.md): the schedule is stated at 91 FR 46565 (preamble), 46576 (preamble) and 46598 (proposed § 433.68(f)(3)(ii)(B)(3)(i)-(v)) in the CMS-2452-P, govinfo PDF (FR Doc. 2026-14897); matched by script.</t>
+          <t>Replaces RM-07, whose first step ('6.0% now') the note no longer states: a state whose July 4, 2025 level was below 6.0% starts below it. Sequencing consistent with RM-08 (expansion states only) and RM-29 (NF and ICF/IID exempt). No corroborating source located in the available outputs UPDATED October 11, 2026: v17's source note changes the cite from 91 FR 46562 to 91 FR 46565, 46576, 46598, and defines the federal fiscal year by 31 U.S.C. 1102 (Citation check: confirmed). The statute pinpoint for the schedule itself (P.L. 119-21 § 71115) was not added to the note; the schedule's statutory page was not checked. VERIFIED October 13, 2026, [CM] part (verification_v4_log.md): the schedule is stated at 91 FR 46565 (preamble), 46576 (preamble) and 46598 (proposed § 433.68(f)(3)(ii)(B)(3)(i)-(v)) in the CMS-2452-P, govinfo PDF (FR Doc. 2026-14897); matched by script. Re-check-list part, October 13, 2026: the schedule is in the statute at P.L. 119-21 § 71115(a)(2), 139 Stat. 302 (govinfo HTML), and the new permissible class at 91 FR 46562 (SUMMARY); both matched by script.</t>
         </is>
       </c>
       <c r="N29" s="12" t="inlineStr">
         <is>
-          <t>single-source — [CM part] re-checked October 13, 2026: 91 FR 46565, 46576 and 46598 each state the schedule (5.5 percent in FFY 2028 down to 3.5 percent from FFY 2032); matches. Still open — NEEDS VERIFICATION [DL3] 91 FR 46562 for the threshold schedule and the new permissible class was left open on the change map (v2 to v3); the statutory page for the schedule is still to add.</t>
+          <t>verified — re-checked October 13, 2026: 91 FR 46565, 46576 and 46598 each state the schedule (5.5 percent in FFY 2028 down to 3.5 percent from FFY 2032); matches. Re-check-list part (re-checked October 13, 2026): the schedule's statutory page is P.L. 119-21 § 71115(a)(2), 139 Stat. 302 (new SSA § 1903(w)(4)(D)(ii)), and 91 FR 46562 states the new permissible class; both match. Upgraded from single-source: the rule and the statute agree.</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="M31" s="12" t="inlineStr">
         <is>
-          <t>Georgetown CCF's July 27, 2026 post (TP-08) is titled 'CMS Issues New Rule Again Going Beyond H.R. 1 Requirements to Further Restrict State Use of Medicaid Provider Taxes', which corroborates the general characterization. The two named provisions are not corroborated in the available outputs UPDATED October 11, 2026: v17 names the additions in its two tables. The earlier wording ('sunsetting a secondary prong of the hold harmless test') is replaced by CMS's stated change: stopping the 75/75 test from FFY2027 (RM-41). Georgetown CCF's July 27, 2026 title corroborates the general characterization (TP-08). Previous wording: 'CMS proposes provisions beyond the statute, including sunsetting a secondary prong of the hold harmless test and adding a permissible class'</t>
+          <t>Georgetown CCF's July 27, 2026 post (TP-08) is titled 'CMS Issues New Rule Again Going Beyond H.R. 1 Requirements to Further Restrict State Use of Medicaid Provider Taxes', which corroborates the general characterization. The two named provisions are not corroborated in the available outputs UPDATED October 11, 2026: v17 names the additions in its two tables. The earlier wording ('sunsetting a secondary prong of the hold harmless test') is replaced by CMS's stated change: stopping the 75/75 test from FFY2027 (RM-41). Georgetown CCF's July 27, 2026 title corroborates the general characterization (TP-08). Previous wording: 'CMS proposes provisions beyond the statute, including sunsetting a secondary prong of the hold harmless test and adding a permissible class' VERIFIED October 13, 2026 (verification_v4_log.md): read in the CMS-2452-P, govinfo PDF (FR Doc. 2026-14897) and CMS-2449-P, govinfo PDF (FR Doc. 2026-10292), matched by script. CMS itself says the WFTC legislation does not address the 75/75 test (46581) and that the extended limits cover services not listed in section 71116 (30453), so the beyond-statute reading now rests on the rules, not only on Georgetown CCF.</t>
         </is>
       </c>
       <c r="N31" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - beyond-statute characterization corroborated by Georgetown CCF; the two named provisions rest on the rule text as the note states it — NEEDS VERIFICATION [DL3] 91 FR 46562 for the new permissible class was left open on the change map (v2 to v3 'existing citations flagged for re-check').</t>
+          <t>verified — upgraded from verified with caveat: re-checked October 13, 2026: 91 FR 46562 (new permissible class; sunset of the second prong), 46581 (75/75 test discontinued for FFYs beginning on or after October 1, 2026), 30453 and 30456 match.</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="M33" s="12" t="inlineStr">
         <is>
-          <t>The observability limb [E] is the same public list checked at RM-10 and scoped at C-6. The 'imminent final action' limb is [FIRM]'s inference [I]. Trigger M-2 UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Transmission of either RIN to OMB is visible on reginfo.gov and marks the move from proposal to imminent final action'</t>
+          <t>The observability limb [E] is the same public list checked at RM-10 and scoped at C-6. The 'imminent final action' limb is [FIRM]'s inference [I]. Trigger M-2 UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Transmission of either RIN to OMB is visible on reginfo.gov and marks the move from proposal to imminent final action' BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
         </is>
       </c>
       <c r="N33" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - second limb is inference — NEEDS VERIFICATION [DL3] reginfo.gov is on the decision-log re-check list (sec. 9 items 3–4; App. I).</t>
+          <t>verified with caveat - second limb is inference — NEEDS VERIFICATION [DL3] reginfo.gov is on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="M46" s="12" t="inlineStr">
         <is>
-          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18.</t>
+          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18. BLOCKED October 13, 2026 (verification_v4_log.md): The SDP preprint form could not be fetched: the proxy refused www.medicaid.gov. Neither proposed rule reproduces the form's Section VI (searched 91 FR 30400–30466 and 46562–46599 by script), and no comment in either docket reproduces it (full-docket search).</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>single-source — the preprint form was not read in the verification files — NEEDS VERIFICATION [DL3] SDP preprint, Section VI (financing fields) is on the decision-log re-check list (sec. 7 step 3).</t>
+          <t>single-source — the preprint form was not read in the verification files — NEEDS VERIFICATION [DL3] SDP preprint, Section VI (financing fields) is on the decision-log re-check list (sec. 7 step 3). blocked: www.medicaid.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -10049,12 +10049,12 @@
       </c>
       <c r="M132" s="12" t="inlineStr">
         <is>
-          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter'</t>
+          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter' BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
         </is>
       </c>
       <c r="N132" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — single publisher, no corroborating outlet located — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified with caveat — single publisher, no corroborating outlet located — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -10121,12 +10121,12 @@
       </c>
       <c r="M133" s="12" t="inlineStr">
         <is>
-          <t>Internal: 756 + 265 − 340 = 681 exactly</t>
+          <t>Internal: 756 + 265 − 340 = 681 exactly BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
         </is>
       </c>
       <c r="N133" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -10193,12 +10193,12 @@
       </c>
       <c r="M134" s="12" t="inlineStr">
         <is>
-          <t>The note relies on this phrase to avoid attributing the figure to any hospital association</t>
+          <t>The note relies on this phrase to avoid attributing the figure to any hospital association BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
         </is>
       </c>
       <c r="N134" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -11273,12 +11273,12 @@
       </c>
       <c r="M149" s="12" t="inlineStr">
         <is>
-          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source'</t>
+          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source' BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article (www.politico.com refused) and CBO's July 21, 2025 table (www.cbo.gov answered 403) could not be fetched.</t>
         </is>
       </c>
       <c r="N149" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com; www.cbo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -12425,12 +12425,12 @@
       </c>
       <c r="M165" s="12" t="inlineStr">
         <is>
-          <t>C3 output retrieved the full article text and confirms this is the only passage containing all three figures UPDATED October 11, 2026: v17 quotes only the final fragment ('leaving a net decrease of $56.6 billion') and paraphrases the rest; the full passage remains as recorded in the Quote column. Previous wording: 'HFMA reports $220.3B, $163.7B and $56.6B in a single passage'</t>
+          <t>C3 output retrieved the full article text and confirms this is the only passage containing all three figures UPDATED October 11, 2026: v17 quotes only the final fragment ('leaving a net decrease of $56.6 billion') and paraphrases the rest; the full passage remains as recorded in the Quote column. Previous wording: 'HFMA reports $220.3B, $163.7B and $56.6B in a single passage' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched: the proxy refused www.hfma.org.</t>
         </is>
       </c>
       <c r="N165" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). The ledger's own C3 output retrieved the full text; the public-comment review did not re-check it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). The ledger's own C3 output retrieved the full text; the public-comment review did not re-check it. blocked: www.hfma.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -12641,12 +12641,12 @@
       </c>
       <c r="M168" s="12" t="inlineStr">
         <is>
-          <t>C3 output finding (b) confirms verbatim; P4 independently confirms UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'HFMA's stated baseline is a scenario with no OBBBA and no proposed rule'</t>
+          <t>C3 output finding (b) confirms verbatim; P4 independently confirms UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'HFMA's stated baseline is a scenario with no OBBBA and no proposed rule' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched: the proxy refused www.hfma.org.</t>
         </is>
       </c>
       <c r="N168" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -12929,12 +12929,12 @@
       </c>
       <c r="M172" s="12" t="inlineStr">
         <is>
-          <t>C3 output retrieved and quotes the sentence; this is the note's only external corroboration of CE-36 (formerly CE-13) UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Georgetown CCF reports the $220.3B with the qualification that it is after the reduction in taxes paid by providers'</t>
+          <t>C3 output retrieved and quotes the sentence; this is the note's only external corroboration of CE-36 (formerly CE-13) UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Georgetown CCF reports the $220.3B with the qualification that it is after the reduction in taxes paid by providers' BLOCKED October 13, 2026 (verification_v4_log.md): Georgetown CCF's July 27, 2026 post could not be fetched: the proxy refused ccf.georgetown.edu. CCF's own comment on CMS-2452-P (CMS-2026-2476-0029) is posted, but it is not the cited post.</t>
         </is>
       </c>
       <c r="N172" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] Georgetown CCF, July 27, 2026 is on the decision-log re-check list (sec. 5, HFMA paragraph).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] Georgetown CCF, July 27, 2026 is on the decision-log re-check list (sec. 5, HFMA paragraph). blocked: ccf.georgetown.edu (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13073,12 +13073,12 @@
       </c>
       <c r="M174" s="12" t="inlineStr">
         <is>
-          <t>V1 output located and verified the quote at p. 11 and confirms it is not a headline savings figure EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version of the report carries the same $891B and $875B figures as the August 12 version the note cites UPDATED October 11, 2026: v17 no longer calls the $891B a 'sensitivity-analysis estimate' or an input to the $875B benefit estimate, and does not state the $875B. The p. 11 quote and the external verification of the September 2 version stand. Previous wording: 'ASPE's $891B is a sensitivity-analysis estimate of total federal-plus-state Medicaid spending reduction from the combined provisions, used as an intermediate input to its $875B benefit estimate'</t>
+          <t>V1 output located and verified the quote at p. 11 and confirms it is not a headline savings figure EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version of the report carries the same $891B and $875B figures as the August 12 version the note cites UPDATED October 11, 2026: v17 no longer calls the $891B a 'sensitivity-analysis estimate' or an input to the $875B benefit estimate, and does not state the $875B. The p. 11 quote and the external verification of the September 2 version stand. Previous wording: 'ASPE's $891B is a sensitivity-analysis estimate of total federal-plus-state Medicaid spending reduction from the combined provisions, used as an intermediate input to its $875B benefit estimate' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N174" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13145,12 +13145,12 @@
       </c>
       <c r="M175" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms, and further establishes that the double-counting language circulating alongside this figure traces to KFF's companion brief rather than to ASPE UPDATED October 11, 2026: v17 states the point as THEIA's reading of what ASPE does not say. The earlier support (ASPE's combined federal savings 'about the size of the SDP effect alone ($510 billion) estimated by OACT') is no longer stated in v17 and remains ledger evidence. Previous wording: 'ASPE does not describe the $891B as adjusted for double counting; it notes its combined estimate is about the size of the SDP effect alone as estimated by OACT'</t>
+          <t>V1 output confirms, and further establishes that the double-counting language circulating alongside this figure traces to KFF's companion brief rather than to ASPE UPDATED October 11, 2026: v17 states the point as THEIA's reading of what ASPE does not say. The earlier support (ASPE's combined federal savings 'about the size of the SDP effect alone ($510 billion) estimated by OACT') is no longer stated in v17 and remains ledger evidence. Previous wording: 'ASPE does not describe the $891B as adjusted for double counting; it notes its combined estimate is about the size of the SDP effect alone as estimated by OACT' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N175" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13217,12 +13217,12 @@
       </c>
       <c r="M176" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms both figures and the $100–175B annual benefit once phased in EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version carries the same $502–875B and 3.5 percent figures as the August 12 version the note cites UPDATED October 11, 2026: citation and location restated to v17 (changed: cite).</t>
+          <t>V1 output confirms both figures and the $100–175B annual benefit once phased in EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version carries the same $502–875B and 3.5 percent figures as the August 12 version the note cites UPDATED October 11, 2026: citation and location restated to v17 (changed: cite). BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N176" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13289,12 +13289,12 @@
       </c>
       <c r="M177" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms the report analyzes Sections 71115–71117 and cites the proposed rules only as data inputs UPDATED October 11, 2026: v17 words the difference as statute-level scoring and different years; it no longer states the dollar basis (unstated vs real 2026) or that the report analyzes Section 71117. The V1 confirmation stands. The conclusion about THEIA's $916.9B is at TP-26. Previous wording: 'ASPE analyzes the statute rather than either proposed rule, on a different horizon and dollar basis'</t>
+          <t>V1 output confirms the report analyzes Sections 71115–71117 and cites the proposed rules only as data inputs UPDATED October 11, 2026: v17 words the difference as statute-level scoring and different years; it no longer states the dollar basis (unstated vs real 2026) or that the report analyzes Section 71117. The V1 confirmation stands. The conclusion about THEIA's $916.9B is at TP-26. Previous wording: 'ASPE analyzes the statute rather than either proposed rule, on a different horizon and dollar basis' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N177" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13361,12 +13361,12 @@
       </c>
       <c r="M178" s="12" t="inlineStr">
         <is>
-          <t>Internal: both attribute part of the effect to commercial payers, but the horizons, bases and objects of analysis differ, so no numerical reconciliation is attempted or possible</t>
+          <t>Internal: both attribute part of the effect to commercial payers, but the horizons, bases and objects of analysis differ, so no numerical reconciliation is attempted or possible BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N178" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — interpretive, not an equivalence — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified with caveat — interpretive, not an equivalence — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13433,12 +13433,12 @@
       </c>
       <c r="M179" s="12" t="inlineStr">
         <is>
-          <t>Internal: 154.9 rounds to 155. V1 output locates and quotes the KFF sentence and confirms it refers to OACT's $510B SDP estimate UPDATED September 27, 2026: the note now cites the KFF brief by title and date (August 14, 2026), the same brief as SE-01 UPDATED October 11, 2026: v17 words the first limb as KFF's report [E] and the match with CMS's $154.9B as THEIA's [I]. Previous wording: 'KFF's widely repeated $155B is the federal share of CMS's $241.9B overlap finding'</t>
+          <t>Internal: 154.9 rounds to 155. V1 output locates and quotes the KFF sentence and confirms it refers to OACT's $510B SDP estimate UPDATED September 27, 2026: the note now cites the KFF brief by title and date (August 14, 2026), the same brief as SE-01 UPDATED October 11, 2026: v17 words the first limb as KFF's report [E] and the match with CMS's $154.9B as THEIA's [I]. Previous wording: 'KFF's widely repeated $155B is the federal share of CMS's $241.9B overlap finding' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief could not be fetched (www.kff.org refused). The CMS limb matches: 91 FR 46592 gives federal spending reductions $154.9 billion less after counting the SDP rule and the $241.9 billion overlap (CMS-2452-P, govinfo PDF (FR Doc. 2026-14897), matched by script).</t>
         </is>
       </c>
       <c r="N179" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -13577,12 +13577,12 @@
       </c>
       <c r="M181" s="12" t="inlineStr">
         <is>
-          <t>This is the instance whose existence bounds NC-09: paired figures exist for at least one state, a consistent multi-state version does not. No figures are reproduced in the note, so nothing here is arithmetically checkable UPDATED September 27, 2026: the note now gives the publication's title and year (2025, while the reconciliation law was pending). Not re-read for this ledger UPDATED October 11, 2026: v17 words this as 'a state hospital association' (sec. 9 item 10) and names the Texas Hospital Association in App. F; the earlier 'for both mechanisms' qualifier is not stated. Not re-read for this ledger. Previous wording: 'The Texas Hospital Association publishes paired gross and net figures for both mechanisms'</t>
+          <t>This is the instance whose existence bounds NC-09: paired figures exist for at least one state, a consistent multi-state version does not. No figures are reproduced in the note, so nothing here is arithmetically checkable UPDATED September 27, 2026: the note now gives the publication's title and year (2025, while the reconciliation law was pending). Not re-read for this ledger UPDATED October 11, 2026: v17 words this as 'a state hospital association' (sec. 9 item 10) and names the Texas Hospital Association in App. F; the earlier 'for both mechanisms' qualifier is not stated. Not re-read for this ledger. Previous wording: 'The Texas Hospital Association publishes paired gross and net figures for both mechanisms' BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Hospital Association's 2025 publication with paired gross and net figures could not be fetched: the proxy refused www.tha.org. THA's comment on CMS-2452-P (CMS-2026-2476-0109) is posted but is not the cited publication.</t>
         </is>
       </c>
       <c r="N181" s="12" t="inlineStr">
         <is>
-          <t>single-source - existence claim only, no figures reproduced — NEEDS VERIFICATION [DL3] Texas Hospital Association paired gross and net figures, 2025, are on the decision-log re-check list (App. F; sec. 9 item 10).</t>
+          <t>single-source - existence claim only, no figures reproduced — NEEDS VERIFICATION [DL3] Texas Hospital Association paired gross and net figures, 2025, are on the decision-log re-check list (App. F; sec. 9 item 10). blocked: www.tha.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -14009,12 +14009,12 @@
       </c>
       <c r="M187" s="12" t="inlineStr">
         <is>
-          <t>HFMA wording at TP-04. CMS's 'pre-statute' baseline and the Tables 5, 9, 10 captions verified at D-16 (CE-43). Replaces TP-05. Resolves D-9 in HFMA's favour UPDATED October 11, 2026: v17 states the match as 'HFMA's July 22, 2026 article, which describes the same no-OBBBA comparison point as CMS'.</t>
+          <t>HFMA wording at TP-04. CMS's 'pre-statute' baseline and the Tables 5, 9, 10 captions verified at D-16 (CE-43). Replaces TP-05. Resolves D-9 in HFMA's favour UPDATED October 11, 2026: v17 states the match as 'HFMA's July 22, 2026 article, which describes the same no-OBBBA comparison point as CMS'. BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched (www.hfma.org refused). The CMS limb (no-OBBBA baseline, Tables 5, 9, 10) was verified at D-16 and is not affected.</t>
         </is>
       </c>
       <c r="N187" s="12" t="inlineStr">
         <is>
-          <t>verified - pre-statute baseline verified at D-16 — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified - pre-statute baseline verified at D-16 — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -14081,12 +14081,12 @@
       </c>
       <c r="M188" s="12" t="inlineStr">
         <is>
-          <t>Internal: 220.3 − 163.7 = 56.6 exactly, and CE-36 establishes that 220.3 is already net of the same 163.7. Absence of 56.6 from both RIAs at TP-07 and NC-08. Georgetown CCF's net reading at TP-08. Replaces TP-06, which stated the double subtraction as fact UPDATED October 11, 2026: v17 drops two clauses of the earlier wording: 'or it comes from a source the note did not locate' and 'the components HFMA cites are correct'. The Table 12 caption evidence is at CE-37. Previous wording: 'On the note's reading, the $56.6B is Table 12's provider line with the tax relief counted a second time, or it comes from a source the note did not locate. The components HFMA cites are correct. If the reading is right, the $56.6B understates the rule's standalone net provider reduction, which is $220.3B'</t>
+          <t>Internal: 220.3 − 163.7 = 56.6 exactly, and CE-36 establishes that 220.3 is already net of the same 163.7. Absence of 56.6 from both RIAs at TP-07 and NC-08. Georgetown CCF's net reading at TP-08. Replaces TP-06, which stated the double subtraction as fact UPDATED October 11, 2026: v17 drops two clauses of the earlier wording: 'or it comes from a source the note did not locate' and 'the components HFMA cites are correct'. The Table 12 caption evidence is at CE-37. Previous wording: 'On the note's reading, the $56.6B is Table 12's provider line with the tax relief counted a second time, or it comes from a source the note did not locate. The components HFMA cites are correct. If the reading is right, the $56.6B understates the rule's standalone net provider reduction, which is $220.3B' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched (www.hfma.org refused). The CMS figures match by script: Table 8 at 91 FR 46590 gives $163.7 billion in lower taxes paid by providers and Table 12 at 46592 a provider line of −$220.3 billion (CMS-2452-P, govinfo PDF (FR Doc. 2026-14897)); 220.3 − 163.7 = 56.6.</t>
         </is>
       </c>
       <c r="N188" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - the arithmetic closes; the note presents it as a reading — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified with caveat - the arithmetic closes; the note presents it as a reading — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -14225,12 +14225,12 @@
       </c>
       <c r="M190" s="12" t="inlineStr">
         <is>
-          <t>TP-10 for the $891B; CE-38 for the $916.9B. The note draws no inference, and the ledger draws none UPDATED October 11, 2026: v17 states the comparison as a cannot-compare conclusion; the earlier 'for scale' wording ('no inference about ASPE's treatment of overlap is drawn') is not stated. The bases are at TP-13. Previous wording: 'For scale, CMS's overlap-adjusted combined estimate is $916.9B against ASPE's $891B; the windows and dollar bases differ, so no inference about ASPE's treatment of overlap is drawn'</t>
+          <t>TP-10 for the $891B; CE-38 for the $916.9B. The note draws no inference, and the ledger draws none UPDATED October 11, 2026: v17 states the comparison as a cannot-compare conclusion; the earlier 'for scale' wording ('no inference about ASPE's treatment of overlap is drawn') is not stated. The bases are at TP-13. Previous wording: 'For scale, CMS's overlap-adjusted combined estimate is $916.9B against ASPE's $891B; the windows and dollar bases differ, so no inference about ASPE's treatment of overlap is drawn' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
         </is>
       </c>
       <c r="N190" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -14513,12 +14513,12 @@
       </c>
       <c r="M194" s="12" t="inlineStr">
         <is>
-          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18.</t>
+          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18. BLOCKED October 13, 2026 (verification_v4_log.md): GAO-24-106202 could not be fetched: the proxy refused www.gao.gov and files.gao.gov; govinfo's GAO collection does not carry it.</t>
         </is>
       </c>
       <c r="N194" s="12" t="inlineStr">
         <is>
-          <t>single-source — not re-read in the review or for this ledger — NEEDS VERIFICATION [DL3] GAO-24-106202, Table 4 is on the decision-log re-check list (sec. 2).</t>
+          <t>single-source — not re-read in the review or for this ledger — NEEDS VERIFICATION [DL3] GAO-24-106202, Table 4 is on the decision-log re-check list (sec. 2). blocked: www.gao.gov; files.gao.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15089,12 +15089,12 @@
       </c>
       <c r="M202" s="12" t="inlineStr">
         <is>
-          <t>The CMS limb is the net construction of Table 12 (CE-36). The distinction is v17's [I] reading; it keeps TP-21 and TP-37 from being read as support for a net-of-tax provider loss. Related: TP-17 (Texas Hospital Association paired figures).</t>
+          <t>The CMS limb is the net construction of Table 12 (CE-36). The distinction is v17's [I] reading; it keeps TP-21 and TP-37 from being read as support for a net-of-tax provider loss. Related: TP-17 (Texas Hospital Association paired figures). BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Hospital Association's 2025 publication with paired gross and net figures could not be fetched: the proxy refused www.tha.org. THA's comment on CMS-2452-P (CMS-2026-2476-0109) is posted but is not the cited publication.</t>
         </is>
       </c>
       <c r="N202" s="12" t="inlineStr">
         <is>
-          <t>verified as inference — NEEDS VERIFICATION [DL3] The Texas Hospital Association's paired gross and net figures (2025), which this note cites alongside CMS's netting (App. F), are on the decision-log re-check list.</t>
+          <t>verified as inference — NEEDS VERIFICATION [DL3] The Texas Hospital Association's paired gross and net figures (2025), which this note cites alongside CMS's netting (App. F), are on the decision-log re-check list. blocked: www.tha.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15305,12 +15305,12 @@
       </c>
       <c r="M205" s="12" t="inlineStr">
         <is>
-          <t>C4: 51 jurisdictions less the 14 with no hospital SDPs = 37 exactly UPDATED October 11, 2026: v17 words the count as 37 states 'including DC' that 'likely exceed the new caps' and tags it [E]. KFF's own wording is 'at least 37 states' with SDPs that 'could be reduced'; the note's 'likely exceed' is a paraphrase. The 51 less 14 arithmetic is unchanged. The KFF brief was not re-read this cycle (kff.org was unreachable in the verification files). Previous wording: 'KFF identifies 37 states with hospital SDPs likely affected by the new limits'</t>
+          <t>C4: 51 jurisdictions less the 14 with no hospital SDPs = 37 exactly UPDATED October 11, 2026: v17 words the count as 37 states 'including DC' that 'likely exceed the new caps' and tags it [E]. KFF's own wording is 'at least 37 states' with SDPs that 'could be reduced'; the note's 'likely exceed' is a paraphrase. The 51 less 14 arithmetic is unchanged. The KFF brief was not re-read this cycle (kff.org was unreachable in the verification files). Previous wording: 'KFF identifies 37 states with hospital SDPs likely affected by the new limits' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N205" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15377,12 +15377,12 @@
       </c>
       <c r="M206" s="12" t="inlineStr">
         <is>
-          <t>Internal: the note's own group dollar column sums to $60.1B. V1 output independently confirms the $78.0B denominator UPDATED October 11, 2026: v17 splits the KFF bullet in two, states that the $60 billion excludes Minnesota and Missouri, says 'one year's' spending and restores 'about $93 billion' in all federal SDP spending (change map S6.1; decision log, 'Numbers vs ledger'). The Group A-D dollar column in the v17 table is the same $60.1 billion by construction (SE-05 to SE-08). The brief was not re-read this cycle. Previous wording: 'Approximately $60B in federal hospital SDP spending sits above the new limits, out of roughly $78B federal hospital SDP spending, within roughly $93B total federal SDP spending'</t>
+          <t>Internal: the note's own group dollar column sums to $60.1B. V1 output independently confirms the $78.0B denominator UPDATED October 11, 2026: v17 splits the KFF bullet in two, states that the $60 billion excludes Minnesota and Missouri, says 'one year's' spending and restores 'about $93 billion' in all federal SDP spending (change map S6.1; decision log, 'Numbers vs ledger'). The Group A-D dollar column in the v17 table is the same $60.1 billion by construction (SE-05 to SE-08). The brief was not re-read this cycle. Previous wording: 'Approximately $60B in federal hospital SDP spending sits above the new limits, out of roughly $78B federal hospital SDP spending, within roughly $93B total federal SDP spending' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N206" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15449,12 +15449,12 @@
       </c>
       <c r="M207" s="12" t="inlineStr">
         <is>
-          <t>C4: NH 0.0910; DC 1.0000; LA 0.9995. Count of shares at or above 0.70 = 27 exactly UPDATED October 11, 2026: v17 moves this bullet from sec. 6 to App. H (change map U31, U49) and words it 'at least 70 percent in 27 states'. The 9 percent (New Hampshire) and 100 percent (Louisiana and DC) endpoints are unchanged. C4 re-derivation stands.</t>
+          <t>C4: NH 0.0910; DC 1.0000; LA 0.9995. Count of shares at or above 0.70 = 27 exactly UPDATED October 11, 2026: v17 moves this bullet from sec. 6 to App. H (change map U31, U49) and words it 'at least 70 percent in 27 states'. The 9 percent (New Hampshire) and 100 percent (Louisiana and DC) endpoints are unchanged. C4 re-derivation stands. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N207" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15521,12 +15521,12 @@
       </c>
       <c r="M208" s="12" t="inlineStr">
         <is>
-          <t>C4: exactly 28 expansion states carry hospital_tax_above_3_5 = Yes. The ambulance and MCO counts are not checkable from the available outputs UPDATED October 11, 2026: v17 words the claim '31 expansion states have a non-exempt provider tax above 3.5 percent: 28 with hospital taxes, 10 with ambulance taxes and 6 with managed care organization taxes' and moves it to sec. 6. Counts unchanged. The 'non-exempt' qualifier corresponds to the statutory exemption for nursing facility and ICF/IID taxes (RM-29).</t>
+          <t>C4: exactly 28 expansion states carry hospital_tax_above_3_5 = Yes. The ambulance and MCO counts are not checkable from the available outputs UPDATED October 11, 2026: v17 words the claim '31 expansion states have a non-exempt provider tax above 3.5 percent: 28 with hospital taxes, 10 with ambulance taxes and 6 with managed care organization taxes' and moves it to sec. 6. Counts unchanged. The 'non-exempt' qualifier corresponds to the statutory exemption for nursing facility and ICF/IID taxes (RM-29). BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N208" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified with caveat — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15593,12 +15593,12 @@
       </c>
       <c r="M209" s="12" t="inlineStr">
         <is>
-          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits'</t>
+          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N209" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15665,12 +15665,12 @@
       </c>
       <c r="M210" s="12" t="inlineStr">
         <is>
-          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B'</t>
+          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N210" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15737,12 +15737,12 @@
       </c>
       <c r="M211" s="12" t="inlineStr">
         <is>
-          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B'</t>
+          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N211" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15809,12 +15809,12 @@
       </c>
       <c r="M212" s="12" t="inlineStr">
         <is>
-          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B'</t>
+          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N212" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15881,12 +15881,12 @@
       </c>
       <c r="M213" s="12" t="inlineStr">
         <is>
-          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure'</t>
+          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N213" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -15953,12 +15953,12 @@
       </c>
       <c r="M214" s="12" t="inlineStr">
         <is>
-          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four'</t>
+          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N214" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16025,12 +16025,12 @@
       </c>
       <c r="M215" s="12" t="inlineStr">
         <is>
-          <t>C4: every non-expansion row reads "N/A - not assessed (non-expansion state)" and carries an explicit note that the tier is not evidence of lower exposure UPDATED October 11, 2026: v17 tags the first limb [E] (KFF did not assess) and the second [I] ('not evidence'), and adds that the lower threshold does not reach non-expansion states. The earlier 'Group D's tax indicators read not assessed' wording is replaced by 'KFF did not assess'. Previous wording: 'Group D's tax indicators read "not assessed," which is an absence of assessment rather than evidence of an absence of taxes above the threshold'</t>
+          <t>C4: every non-expansion row reads "N/A - not assessed (non-expansion state)" and carries an explicit note that the tier is not evidence of lower exposure UPDATED October 11, 2026: v17 tags the first limb [E] (KFF did not assess) and the second [I] ('not evidence'), and adds that the lower threshold does not reach non-expansion states. The earlier 'Group D's tax indicators read not assessed' wording is replaced by 'KFF did not assess'. Previous wording: 'Group D's tax indicators read "not assessed," which is an absence of assessment rather than evidence of an absence of taxes above the threshold' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N215" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16097,12 +16097,12 @@
       </c>
       <c r="M216" s="12" t="inlineStr">
         <is>
-          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each'</t>
+          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N216" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16169,12 +16169,12 @@
       </c>
       <c r="M217" s="12" t="inlineStr">
         <is>
-          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before.</t>
+          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N217" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16241,12 +16241,12 @@
       </c>
       <c r="M218" s="12" t="inlineStr">
         <is>
-          <t>C4: both INSUFFICIENT with a blank share. The C4 response states the point directly — "their blank is not a zero" — and distinguishes them from the 14 determined zeros UPDATED October 11, 2026: v17 states the exclusion and 'no KFF estimate' and no longer says the two states' SDPs are 'benchmarked to average commercial rates'; that limb is no longer a note claim. v17 tags the whole sentence [E], but 'belong in Group A' is THEIA Services' own grouping (SE-17); the C4 check (both INSUFFICIENT with a blank share) supports the 'no estimate' limb only. Previous wording: 'Minnesota and Missouri have hospital SDPs benchmarked to average commercial rates but no estimable above-limit figure, and are excluded from the $45.4B'</t>
+          <t>C4: both INSUFFICIENT with a blank share. The C4 response states the point directly — "their blank is not a zero" — and distinguishes them from the 14 determined zeros UPDATED October 11, 2026: v17 states the exclusion and 'no KFF estimate' and no longer says the two states' SDPs are 'benchmarked to average commercial rates'; that limb is no longer a note claim. v17 tags the whole sentence [E], but 'belong in Group A' is THEIA Services' own grouping (SE-17); the C4 check (both INSUFFICIENT with a blank share) supports the 'no estimate' limb only. Previous wording: 'Minnesota and Missouri have hospital SDPs benchmarked to average commercial rates but no estimable above-limit figure, and are excluded from the $45.4B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N218" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16385,12 +16385,12 @@
       </c>
       <c r="M220" s="12" t="inlineStr">
         <is>
-          <t>none located beyond KFF itself UPDATED October 11, 2026: CORRECTED. The previous wording had KFF's base-rate finding backwards: it said a high share above the limits partly reflects low base payment rates. The finding runs the other way: states with most SDP spending above the caps already have base rates at or near the caps, and low base rates leave more SDP spending under the caps. v17 states it that way. The first limb, 'dollars above the caps do not show which states face the largest proportional effects', replaces the earlier 'do not show proportional effects' (change map S6.2, NTC 6.14). The change map records v17's base-rate wording as 'kept as in v16' (S6.2). The correction was instructed by the note's author and matches v17's text; the KFF brief itself could not be re-read here. Previous wording: 'KFF's caveat governs the dollar column: a high share above limits partly reflects low base payment rates rather than unusually generous supplemental payments'</t>
+          <t>none located beyond KFF itself UPDATED October 11, 2026: CORRECTED. The previous wording had KFF's base-rate finding backwards: it said a high share above the limits partly reflects low base payment rates. The finding runs the other way: states with most SDP spending above the caps already have base rates at or near the caps, and low base rates leave more SDP spending under the caps. v17 states it that way. The first limb, 'dollars above the caps do not show which states face the largest proportional effects', replaces the earlier 'do not show proportional effects' (change map S6.2, NTC 6.14). The change map records v17's base-rate wording as 'kept as in v16' (S6.2). The correction was instructed by the note's author and matches v17's text; the KFF brief itself could not be re-read here. Previous wording: 'KFF's caveat governs the dollar column: a high share above limits partly reflects low base payment rates rather than unusually generous supplemental payments' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N220" s="12" t="inlineStr">
         <is>
-          <t>single-source — direction corrected to match v17; KFF brief not re-read — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>single-source — direction corrected to match v17; KFF brief not re-read — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16673,12 +16673,12 @@
       </c>
       <c r="M224" s="12" t="inlineStr">
         <is>
-          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there'</t>
+          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N224" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -16961,12 +16961,12 @@
       </c>
       <c r="M228" s="12" t="inlineStr">
         <is>
-          <t>First limb of the sentence at SE-16, split out so the base-rate direction can be tracked separately. The KFF brief was not re-read this cycle. No corroborating source located beyond KFF itself.</t>
+          <t>First limb of the sentence at SE-16, split out so the base-rate direction can be tracked separately. The KFF brief was not re-read this cycle. No corroborating source located beyond KFF itself. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N228" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -17465,12 +17465,12 @@
       </c>
       <c r="M235" s="12" t="inlineStr">
         <is>
-          <t>Internal: 11.3 + 16.8 = 28.1 exactly for 2011, but 9.06 + 19.5 = 28.6 against the reported 28.4 for 2023, a 0.2 gap consistent with the paper's own rounding. **The note reports each figure as published and does not assert the sum.** No corroborating source located. Read with AC-08 UPDATED October 11, 2026: v17 gives the figures as published ('about flat at 28.1 and 28.4') and no longer says the freestanding rise 'offset' the short-term acute-care decline; it does not state the sum of the components. The 9.06 + 19.5 = 28.6 against 28.4 point is unchanged. Previous wording: 'Total inpatient psychiatric beds across both facility types were essentially flat, 28.1 per 100,000 in 2011 against 28.4 in 2023; freestanding psychiatric hospital beds rose from 16.8 to 19.5, offsetting the short-term acute-care decline'</t>
+          <t>Internal: 11.3 + 16.8 = 28.1 exactly for 2011, but 9.06 + 19.5 = 28.6 against the reported 28.4 for 2023, a 0.2 gap consistent with the paper's own rounding. **The note reports each figure as published and does not assert the sum.** No corroborating source located. Read with AC-08 UPDATED October 11, 2026: v17 gives the figures as published ('about flat at 28.1 and 28.4') and no longer says the freestanding rise 'offset' the short-term acute-care decline; it does not state the sum of the components. The 9.06 + 19.5 = 28.6 against 28.4 point is unchanged. Previous wording: 'Total inpatient psychiatric beds across both facility types were essentially flat, 28.1 per 100,000 in 2011 against 28.4 in 2023; freestanding psychiatric hospital beds rose from 16.8 to 19.5, offsetting the short-term acute-care decline' VERIFIED October 13, 2026 (verification_v4_log.md): Lindenfeld et al., PLoS Medicine 22(7): e1004682, July 23, 2025 (doi:10.1371/journal.pmed.1004682), PMC full text PMC12310024 read through the PubMed connector; journals.plos.org, pmc.ncbi.nlm.nih.gov and europepmc.org refused the connection, so the text could not be saved and was compared by reading, not by script. Results: 28.1 and 28.4 IPBs per 100,000 across both facility types; psychiatric hospitals 16.8 to 19.5; the total 'did not change' (abstract). The paper's Results give the short-term acute care series as 11.2 to 8.9, which with 16.8 and 19.5 close to 28.0 and 28.4; the abstract's 11.3 and 9.06 (AC-11) explain the 0.2 gap noted here.</t>
         </is>
       </c>
       <c r="N235" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Lindenfeld et al., PLoS Medicine, July 2025 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it.</t>
+          <t>single-source — one study; re-checked October 13, 2026 against the PMC full text: 28.1 (2011) and 28.4 (2023) in total, 16.8 to 19.5 in psychiatric hospitals; matches (read, not script-matched).</t>
         </is>
       </c>
     </row>
@@ -17537,12 +17537,12 @@
       </c>
       <c r="M236" s="12" t="inlineStr">
         <is>
-          <t>Internal: the interval spans zero, so the short-term acute-care decline cited at AC-01 is not distinguishable from no trend at conventional significance. No corroborating source located UPDATED October 11, 2026: v17 states only the non-significance. The average annual percent change of -2.0 and its 95 percent confidence interval of -5.84 to 3.01 for short-term acute-care beds are no longer in the note; they stay true to the abstract as ledgered and are kept as ledger evidence. Previous wording: 'The average annual percent change is not statistically significant for any bed type; for short-term acute-care hospital beds it is −2.0, with a 95 percent confidence interval of −5.84 to 3.01'</t>
+          <t>Internal: the interval spans zero, so the short-term acute-care decline cited at AC-01 is not distinguishable from no trend at conventional significance. No corroborating source located UPDATED October 11, 2026: v17 states only the non-significance. The average annual percent change of -2.0 and its 95 percent confidence interval of -5.84 to 3.01 for short-term acute-care beds are no longer in the note; they stay true to the abstract as ledgered and are kept as ledger evidence. Previous wording: 'The average annual percent change is not statistically significant for any bed type; for short-term acute-care hospital beds it is −2.0, with a 95 percent confidence interval of −5.84 to 3.01' CORRECTED October 13, 2026 (verification_v4_log.md): Lindenfeld et al., PLoS Medicine 22(7): e1004682, July 23, 2025 (doi:10.1371/journal.pmed.1004682), PMC full text PMC12310024 read through the PubMed connector; journals.plos.org, pmc.ncbi.nlm.nih.gov and europepmc.org refused the connection, so the text could not be saved and was compared by reading, not by script. Fig 1 note: AAPC −2.0 (95% CI −5.84, 3.01) for STACH beds, 1.4 (−1.9, 4.9) for psychiatric hospitals, 0.34 (−2.34, 3.11) in total, all spanning zero. But Table 2 gives a year IRR of 0.97 (95% CI 0.96–0.99, p&lt;0.001) for STACH psychiatric beds, and Table 3 a significant yearly decrease in county beds per 100,000 (−153.78, p&lt;0.001). 'No statistically significant trend for any type of bed' is true of the AAPC only.</t>
         </is>
       </c>
       <c r="N236" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Lindenfeld et al., PLoS Medicine, July 2025 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it.</t>
+          <t>corrected — source says: “For all types of IPBs, the average annual percent change over the study period was not significant” (Lindenfeld et al., Results ¶1; Fig 1 note). The paper's regression and county models do find a significant yearly decline (Tables 2–3). v17 must narrow 'no statistically significant trend for any type of bed' to the average annual percent change (see verification_v4_log.md). Base status was single-source. Read via the PubMed connector, not script-matched.</t>
         </is>
       </c>
     </row>
@@ -17609,12 +17609,12 @@
       </c>
       <c r="M237" s="12" t="inlineStr">
         <is>
-          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services'</t>
+          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services' BLOCKED October 13, 2026 (verification_v4_log.md): GAO-23-105515 could not be fetched: the proxy refused www.gao.gov and files.gao.gov.</t>
         </is>
       </c>
       <c r="N237" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — NEEDS VERIFICATION [DL3] GAO-23-105515 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it.</t>
+          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — NEEDS VERIFICATION [DL3] GAO-23-105515 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: www.gao.gov; files.gao.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -17681,12 +17681,12 @@
       </c>
       <c r="M238" s="12" t="inlineStr">
         <is>
-          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period'</t>
+          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period' BLOCKED October 13, 2026 (verification_v4_log.md): Michelson, Cushing and Bucholz, 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics 179(2):208–209 (doi:10.1001/jamapediatrics.2024.5110; PMC11612914). PubMed has no abstract, the PubMed connector returned no full text, and the proxy refused jamanetwork.com, pmc.ncbi.nlm.nih.gov and europepmc.org.</t>
         </is>
       </c>
       <c r="N238" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it.</t>
+          <t>single-source — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: jamanetwork.com; pmc.ncbi.nlm.nih.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -17753,12 +17753,12 @@
       </c>
       <c r="M239" s="12" t="inlineStr">
         <is>
-          <t>This is the series behind the shift in point estimates at AC-14 (the 'migration' reading at AC-12 is superseded), and it is the series whose trend AC-08 shows is not statistically significant. Read with AC-07 and AC-08: the decline is real as a level comparison and not distinguishable from no trend as a rate UPDATED October 11, 2026: v17 gives the series in the psychiatry bullet next to the freestanding series (AC-07), with the no-trend statement (AC-08). Figures unchanged. Previous wording: 'Inpatient psychiatric beds within short-term acute-care hospitals fell from 11.3 to 9.06 per 100,000 population across 2011-2023'</t>
+          <t>This is the series behind the shift in point estimates at AC-14 (the 'migration' reading at AC-12 is superseded), and it is the series whose trend AC-08 shows is not statistically significant. Read with AC-07 and AC-08: the decline is real as a level comparison and not distinguishable from no trend as a rate UPDATED October 11, 2026: v17 gives the series in the psychiatry bullet next to the freestanding series (AC-07), with the no-trend statement (AC-08). Figures unchanged. Previous wording: 'Inpatient psychiatric beds within short-term acute-care hospitals fell from 11.3 to 9.06 per 100,000 population across 2011-2023' VERIFIED WITH CAVEAT October 13, 2026 (verification_v4_log.md): Lindenfeld et al., PLoS Medicine 22(7): e1004682, July 23, 2025 (doi:10.1371/journal.pmed.1004682), PMC full text PMC12310024 read through the PubMed connector; journals.plos.org, pmc.ncbi.nlm.nih.gov and europepmc.org refused the connection, so the text could not be saved and was compared by reading, not by script. Abstract: STACH beds 'fell from 11.3 in 2011 to 9.06 in 2023'; Results: 'from 11.2 in 2011 to 8.9 in 2023'. v17 follows the abstract. The Results figures add up with the psychiatric-hospital series to the published totals.</t>
         </is>
       </c>
       <c r="N239" s="12" t="inlineStr">
         <is>
-          <t>single-source - and see AC-08, which removes the significance — NEEDS VERIFICATION [DL3] Lindenfeld et al., PLoS Medicine, July 2025 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it.</t>
+          <t>verified with caveat — single study; re-checked October 13, 2026: the abstract gives 11.3 (2011) and 9.06 (2023), as v17 does, but the paper's Results give 11.2 and 8.9 for the same series (read, not script-matched).</t>
         </is>
       </c>
     </row>
@@ -18041,12 +18041,12 @@
       </c>
       <c r="M243" s="12" t="inlineStr">
         <is>
-          <t>The note cites no source for this sentence. The provisions named in the citation column are the ledger's identification, offered as a citation the author may add; they were not re-read for this ledger UPDATED October 11, 2026: v17 now cites the exclusion (§ 1905(a)) and the managed care exception (42 CFR 438.6(e)), where the earlier row recorded the note as uncited. The Citation check confirms § 1905(a) (closing text, clause (B)) and § 1905(i), and 42 CFR 438.6(e) ('an enrollee aged 21-64'). The exception for 'certain demonstrations' is tagged [I] in the body and App. B says it is not yet sourced. The ledger's earlier suggested citations for section 1115 demonstrations were not re-read. Previous wording: 'The IMD exclusion is a long-standing limit that predates both rules, with exceptions for managed care and certain demonstrations'</t>
+          <t>The note cites no source for this sentence. The provisions named in the citation column are the ledger's identification, offered as a citation the author may add; they were not re-read for this ledger UPDATED October 11, 2026: v17 now cites the exclusion (§ 1905(a)) and the managed care exception (42 CFR 438.6(e)), where the earlier row recorded the note as uncited. The Citation check confirms § 1905(a) (closing text, clause (B)) and § 1905(i), and 42 CFR 438.6(e) ('an enrollee aged 21-64'). The exception for 'certain demonstrations' is tagged [I] in the body and App. B says it is not yet sourced. The ledger's earlier suggested citations for section 1115 demonstrations were not re-read. Previous wording: 'The IMD exclusion is a long-standing limit that predates both rules, with exceptions for managed care and certain demonstrations' VERIFIED October 13, 2026 (verification_v4_log.md): 81 FR 27562 (Medicaid managed care final rule, FR Doc. 2016-09581, govinfo PDF) says SMDL #15-003 lets states request a section 1115(a) demonstration to receive federal matching funds for individuals residing in IMDs to treat SUD; matched by script. Lindenfeld et al. (2025) say states could apply for section 1115 waivers for mental health treatment in IMDs from 2015 (read, not script-matched). v17's App. B 'not yet sourced' can be replaced by the 81 FR 27562 cite.</t>
         </is>
       </c>
       <c r="N243" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — exclusion and managed care exception confirmed by the Citation check; the 'certain demonstrations' exception is not yet sourced — NEEDS VERIFICATION [DL3] A source for the IMD exclusion's exception for 'certain demonstrations' is on the 'citation to add after verification' list (change map, v2 list item 9; decision log, review item 4-8).</t>
+          <t>verified — upgraded from verified with caveat: re-checked October 13, 2026: a source for the demonstration exception exists: section 1115(a) demonstrations for IMD stays, under SMDL #15-003 (81 FR 27562).</t>
         </is>
       </c>
     </row>
@@ -18617,12 +18617,12 @@
       </c>
       <c r="M251" s="12" t="inlineStr">
         <is>
-          <t>Re-dated from Sept 5 to Sept 21, 2026 in the Sept 22 currency check; AV69 confirmed on reginfo.gov. See RM-10 UPDATED October 11, 2026: v17 states no OIRA review-list status for either RIN. Sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading ('Status as of [DATE]: White House review, CMS-2450, comment periods and counts, HFMA contact') has no text under it. The September 21, 2026 check is stale against the October 2026 draft and is not restated in the note. See RM-10.</t>
+          <t>Re-dated from Sept 5 to Sept 21, 2026 in the Sept 22 currency check; AV69 confirmed on reginfo.gov. See RM-10 UPDATED October 11, 2026: v17 states no OIRA review-list status for either RIN. Sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading ('Status as of [DATE]: White House review, CMS-2450, comment periods and counts, HFMA contact') has no text under it. The September 21, 2026 check is stale against the October 2026 draft and is not restated in the note. See RM-10. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
         </is>
       </c>
       <c r="N251" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped (C-6) — perishable; no longer stated in the note — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3-4; App. I); re-run the OIRA list check at the date the note fills in.</t>
+          <t>verified as scoped (C-6) — perishable; no longer stated in the note — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3-4; App. I); re-run the OIRA list check at the date the note fills in. blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -19265,12 +19265,12 @@
       </c>
       <c r="M260" s="12" t="inlineStr">
         <is>
-          <t>Litigation and bill limbs as re-checked Sept 22, 2026 (NC-05, C-5). The lobbying limb rests on TP-28. Replaces NC-05, which said opposition 'consists of comment letters' UPDATED October 11, 2026: v17 drops the opposition limb: it no longer says the formal opposition located 'is in comment letters' or that press reports describe hospitals lobbying (TP-28 is superseded). The litigation limb is tagged [I] and the bill limb [E]; the bill numbers and scope are in App. I. Both limbs are dated September 22, 2026 and are perishable; the October 7, 2026 comment review adds that no comment reports a filed suit (NC-20). Previous wording: 'As of Sept 22, 2026, no filed litigation challenging either proposed rule was located. Two bills introduced in July 2025 would repeal the underlying statutory sections, S. 2279 (Sections 71115 and 71116) and H.R. 4807 (Section 71115), and neither has advanced beyond committee referral. The formal opposition located is in comment letters; press reports describe hospitals lobbying against the rules as well'</t>
+          <t>Litigation and bill limbs as re-checked Sept 22, 2026 (NC-05, C-5). The lobbying limb rests on TP-28. Replaces NC-05, which said opposition 'consists of comment letters' UPDATED October 11, 2026: v17 drops the opposition limb: it no longer says the formal opposition located 'is in comment letters' or that press reports describe hospitals lobbying (TP-28 is superseded). The litigation limb is tagged [I] and the bill limb [E]; the bill numbers and scope are in App. I. Both limbs are dated September 22, 2026 and are perishable; the October 7, 2026 comment review adds that no comment reports a filed suit (NC-20). Previous wording: 'As of Sept 22, 2026, no filed litigation challenging either proposed rule was located. Two bills introduced in July 2025 would repeal the underlying statutory sections, S. 2279 (Sections 71115 and 71116) and H.R. 4807 (Section 71115), and neither has advanced beyond committee referral. The formal opposition located is in comment letters; press reports describe hospitals lobbying against the rules as well' VERIFIED October 13, 2026 (verification_v4_log.md): govinfo BILLSTATUS XML for S. 2279 and H.R. 4807 (119th Congress), retrieved October 13, 2026: latest action is the July 2025 referral for each; S. 2279 repeals the provider tax and SDP changes, H.R. 4807 the provider tax changes. This supports the bill limb at a later date than September 22, 2026. The litigation limb ([I]) was not re-searched: courtlistener.com was refused.</t>
         </is>
       </c>
       <c r="N260" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped (C-5) — perishable; opposition limb no longer a note claim — NEEDS VERIFICATION [DL3] S. 2279, H.R. 4807, their committee-referral status and the 'as of September 22, 2026' date are on the decision-log re-check list (sec. 9 item 7; App. I); no source in the files supports a later date.</t>
+          <t>verified as scoped (C-5) — perishable; re-checked October 13, 2026: govinfo bill status shows S. 2279 (July 15, 2025, Finance) and H.R. 4807 (July 29, 2025, Energy and Commerce) with no action after referral.</t>
         </is>
       </c>
     </row>
@@ -20129,12 +20129,12 @@
       </c>
       <c r="M272" s="12" t="inlineStr">
         <is>
-          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down'</t>
+          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
         </is>
       </c>
       <c r="N272" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it.</t>
+          <t>verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -20201,12 +20201,12 @@
       </c>
       <c r="M273" s="12" t="inlineStr">
         <is>
-          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)'</t>
+          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)' BLOCKED October 13, 2026 (verification_v4_log.md): Michelson, Cushing and Bucholz, 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics 179(2):208–209 (doi:10.1001/jamapediatrics.2024.5110; PMC11612914). PubMed has no abstract, the PubMed connector returned no full text, and the proxy refused jamanetwork.com, pmc.ncbi.nlm.nih.gov and europepmc.org.</t>
         </is>
       </c>
       <c r="N273" s="12" t="inlineStr">
         <is>
-          <t>single-source - one study (AC-10); caption only in v17 — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (sec. 8); the figure rests on AC-10.</t>
+          <t>single-source - one study (AC-10); caption only in v17 — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (sec. 8); the figure rests on AC-10. blocked: jamanetwork.com; pmc.ncbi.nlm.nih.gov (re-checked October 13, 2026).</t>
         </is>
       </c>
     </row>
@@ -20273,12 +20273,12 @@
       </c>
       <c r="M274" s="12" t="inlineStr">
         <is>
-          <t>Values at AC-07, AC-08, AC-11. Internal: 9.06 + 19.5 = 28.56, stated as 28.6, against 28.4 (AC-07) UPDATED October 11, 2026: v17 carries only the caption ('The combined total was about flat, and the authors found no statistically significant trend for any type of bed'). The confidence interval and the 28.6 against 28.4 note are not in the caption and are not note claims (AC-08); whether the artwork still shows them was not supplied. Values at AC-07, AC-08, AC-11. Internal: 9.06 + 19.5 = 28.56 (28.6) against 28.4. Previous wording: 'Figure 8. "Psychiatric beds per 100,000 by facility type, 2011 and 2023." Values: total 28.1 to 28.4; freestanding psychiatric 16.8 to 19.5; short-term acute-care 11.3 to 9.06. Note: no significant trend for any bed type (95% CI −5.84 to 3.01 for short-term beds); 2023 components sum to 28.6 against a published 28.4'</t>
+          <t>Values at AC-07, AC-08, AC-11. Internal: 9.06 + 19.5 = 28.56, stated as 28.6, against 28.4 (AC-07) UPDATED October 11, 2026: v17 carries only the caption ('The combined total was about flat, and the authors found no statistically significant trend for any type of bed'). The confidence interval and the 28.6 against 28.4 note are not in the caption and are not note claims (AC-08); whether the artwork still shows them was not supplied. Values at AC-07, AC-08, AC-11. Internal: 9.06 + 19.5 = 28.56 (28.6) against 28.4. Previous wording: 'Figure 8. "Psychiatric beds per 100,000 by facility type, 2011 and 2023." Values: total 28.1 to 28.4; freestanding psychiatric 16.8 to 19.5; short-term acute-care 11.3 to 9.06. Note: no significant trend for any bed type (95% CI −5.84 to 3.01 for short-term beds); 2023 components sum to 28.6 against a published 28.4' CORRECTED October 13, 2026 (verification_v4_log.md): see AC-08, AC-07 and AC-11; Lindenfeld et al., PLoS Medicine 22(7): e1004682, July 23, 2025 (doi:10.1371/journal.pmed.1004682), PMC full text PMC12310024 read through the PubMed connector; journals.plos.org, pmc.ncbi.nlm.nih.gov and europepmc.org refused the connection, so the text could not be saved and was compared by reading, not by script.</t>
         </is>
       </c>
       <c r="N274" s="12" t="inlineStr">
         <is>
-          <t>single-source - one study (AC-07); caption only in v17 — NEEDS VERIFICATION [DL3] Lindenfeld et al., PLoS Medicine, July 2025 is on the decision-log re-check list (sec. 8); the figure rests on AC-07, AC-08 and AC-11.</t>
+          <t>corrected — source says: “For all types of IPBs, the average annual percent change over the study period was not significant” (Lindenfeld et al., Results ¶1); the paper's regression models find a significant decline (Tables 2–3). The [Figure 8] caption's 'no statistically significant trend for any type of bed' must be narrowed (see verification_v4_log.md and AC-08). Values 28.1/28.4 and 16.8/19.5 match; 11.3/9.06 match the abstract only (AC-11). Read via the PubMed connector, not script-matched. Base status was single-source.</t>
         </is>
       </c>
     </row>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. Checked so far: [CM] Federal Register pinpoints, [DL4] comment IDs; 33 of the 91 flagged rows. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 26 rows match and lose the flag (20 upgraded, for example single-source to verified); 6 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 0 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 2 rows with two tags were resolved for one tag only and keep the other tag's flag (counted above by the result for the resolved tag). No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
+          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. Checked so far: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list; 90 of the 91 flagged rows. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 34 rows match and lose the flag (25 upgraded, for example single-source to verified); 8 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 48 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 0 rows with two tags were resolved for one tag only and keep the other tag's flag (counted above by the result for the resolved tag). No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ledger v4 verification, group 4: AC-14 and final log
AC-14: no source found that most freestanding psychiatric hospitals are
IMDs (Federal Register full-text search, four rules read on govinfo,
PubMed, Lindenfeld et al.); the row stays unresolved and flagged
'not found'. NC-19 left unchanged as instructed. Coverage note, Legend
counts and verification_v4_log.md brought to the final state: 34 match,
8 corrected, 47 blocked, 2 not found.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jFZZ5qaUFnBNLfBGt45ve
</commit_message>
<xml_diff>
--- a/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
+++ b/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
@@ -17969,12 +17969,12 @@
       </c>
       <c r="M242" s="12" t="inlineStr">
         <is>
-          <t>Shift limb supported by AC-07 and AC-11 and constrained by AC-08. The claim that most freestanding psychiatric hospitals are IMDs is uncited in the note. IMD limb at AC-15. Replaces AC-12 UPDATED October 11, 2026: v17 no longer says point estimates 'shifted from general hospitals toward freestanding psychiatric hospitals'; the two series are stated in the psychiatry bullet (AC-07, AC-11) with the no-trend statement (AC-08). The IMD sentence is tagged [I], and App. B says 'That most freestanding psychiatric hospitals are IMDs, and the exception for certain demonstrations (sec. 8), are not yet sourced.' The IMD definition and the exclusion are sourced (AC-15, AC-17). Previous wording: 'Point estimates shifted from general hospitals toward freestanding psychiatric hospitals, though the authors found no statistically significant trend for any bed type. For Medicaid adults that shift is not access-neutral: most freestanding psychiatric hospitals are institutions for mental diseases, where federal Medicaid payment for adults aged 21 to 64 is restricted'</t>
+          <t>Shift limb supported by AC-07 and AC-11 and constrained by AC-08. The claim that most freestanding psychiatric hospitals are IMDs is uncited in the note. IMD limb at AC-15. Replaces AC-12 UPDATED October 11, 2026: v17 no longer says point estimates 'shifted from general hospitals toward freestanding psychiatric hospitals'; the two series are stated in the psychiatry bullet (AC-07, AC-11) with the no-trend statement (AC-08). The IMD sentence is tagged [I], and App. B says 'That most freestanding psychiatric hospitals are IMDs, and the exception for certain demonstrations (sec. 8), are not yet sourced.' The IMD definition and the exclusion are sourced (AC-15, AC-17). Previous wording: 'Point estimates shifted from general hospitals toward freestanding psychiatric hospitals, though the authors found no statistically significant trend for any bed type. For Medicaid adults that shift is not access-neutral: most freestanding psychiatric hospitals are institutions for mental diseases, where federal Medicaid payment for adults aged 21 to 64 is restricted' NOT FOUND October 13, 2026 (verification_v4_log.md): searched the federalregister.gov full-text API for six phrasings (for example "freestanding psychiatric hospitals" with "institutions for mental diseases"; "psychiatric hospitals are IMDs"; "most psychiatric hospitals"), read the IMD passages of 69 FR 66922 (IPF PPS, 2004), 81 FR 27498 (managed care, 2016), 89 FR 23146 (FY 2025 IPF PPS proposed) and 91 FR 48514 (FY 2027 IPF PPS) on govinfo, searched PubMed (4 articles, none with PMC full text) and read Lindenfeld et al. (2025). None says it. Closest support: an IMD is a facility of more than 16 beds primarily engaged in treating mental diseases (§ 1905(i), restated at 81 FR 27561–27562), and psychiatric hospitals in Lindenfeld et al.'s sample average 108 beds (mean, not median). MACPAC (www.macpac.gov) and KFF were refused by the proxy. The claim stays [I] and unresolved.</t>
         </is>
       </c>
       <c r="N242" s="12" t="inlineStr">
         <is>
-          <t>unresolved — 'most freestanding psychiatric hospitals are IMDs' is tagged [I] and App. B says it is not yet sourced — NEEDS VERIFICATION [DL3] A source for 'most freestanding psychiatric hospitals are institutions for mental diseases' is on the 'citation to add after verification' list (change map, v2 list item 8; decision log, review item 4-8).</t>
+          <t>unresolved — 'most freestanding psychiatric hospitals are IMDs' is tagged [I] and App. B says it is not yet sourced — NEEDS VERIFICATION [DL3] A source for 'most freestanding psychiatric hospitals are institutions for mental diseases' is on the 'citation to add after verification' list (change map, v2 list item 8; decision log, review item 4-8). not found (re-checked October 13, 2026): no source located that says most freestanding psychiatric hospitals are IMDs.</t>
         </is>
       </c>
     </row>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. Checked so far: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list; 90 of the 91 flagged rows. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 34 rows match and lose the flag (25 upgraded, for example single-source to verified); 8 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 48 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 0 rows with two tags were resolved for one tag only and keep the other tag's flag (counted above by the result for the resolved tag). No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
+          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. All 91 flagged rows were checked, in order: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list, the unresolved row AC-14. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text, except four rows on one journal article read through the PubMed connector (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 34 rows match and lose the flag (25 upgraded, for example single-source to verified); 8 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 49 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ledger v4 verification: second pass on the 47 blocked rows; blank organization fields
After the network policy was opened, re-ran the 47 rows blocked in the
first pass with the same script-matching rules: 24 match, 4 corrected
(SE-09 Colorado's SDP above the caps; SE-11 KFF's survey did cover
non-expansion states; SE-16 and SE-24 KFF's hedge), 19 still blocked
(POLITICO, Fierce, JAMA, GAO, medicaid.gov and CBO refused at the site;
KFF's chart data host refused by the network policy), each with its URL.
Adds sections 4-5 to verification_v4_log.md: second-pass results, and the
32 organization letters filed with a blank organization field (no count
in article_v4.md changes).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jFZZ5qaUFnBNLfBGt45ve
</commit_message>
<xml_diff>
--- a/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
+++ b/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
@@ -1337,12 +1337,12 @@
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>RE-DATED in the Sept 22, 2026 currency check: both RINs absent from the Sept 21, 2026 list. RIN 0938-AV69 confirmed on reginfo.gov as CMS-2449-P; 0938-AV93 is CMS-2452-P. The original Sept 5, 2026 check (P1 output, both RINs) is superseded as to date only. CMS-2450 (RIN 0938-AV70), a separate rule, has been under review since May 12, 2026 and is disclosed in the status box; see M-6 UPDATED October 11, 2026: v17 states no White House review status for either RIN: sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading 'Status as of [DATE]: White House review, CMS-2450 …' has no text under it. The September 21, 2026 check is therefore stale against the October 2026 draft and is not restated in the note. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
+          <t>RE-DATED in the Sept 22, 2026 currency check: both RINs absent from the Sept 21, 2026 list. RIN 0938-AV69 confirmed on reginfo.gov as CMS-2449-P; 0938-AV93 is CMS-2452-P. The original Sept 5, 2026 check (P1 output, both RINs) is superseded as to date only. CMS-2450 (RIN 0938-AV70), a separate rule, has been under review since May 12, 2026 and is disclosed in the status box; see M-6 UPDATED October 11, 2026: v17 states no White House review status for either RIN: sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading 'Status as of [DATE]: White House review, CMS-2450 …' has no text under it. The September 21, 2026 check is therefore stale against the October 2026 draft and is not restated in the note. VERIFIED October 13, 2026, second pass (verification_v4_log.md): reginfo.gov, read October 13, 2026: the EO 12866 'rules under review' XML (RUNDATE 2026-10-13; https://www.reginfo.gov/public/do/XMLViewFileAction?f=EO_RULES_UNDER_REVIEW.xml) lists RIN 0938-AV70 (CMS-2450, received 05/12/2026) and neither 0938-AV69 nor 0938-AV93; this year's completed list shows OIRA concluded review of both proposed rules (AV69 on 2026-05-19, AV93 on 2026-07-21). Matched by script against the downloaded XML.</t>
         </is>
       </c>
       <c r="N11" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see C-6; perishable — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3–4; App. I); re-run the OIRA list check at the date the note fills in. blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
+          <t>verified as scoped — see C-6; perishable — re-checked October 13, 2026, second pass: OIRA's list of rules under review, run October 13, 2026, shows neither RIN (0938-AV69, 0938-AV93); the check can now be dated October 13, 2026.</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2273,12 @@
       </c>
       <c r="M24" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-6. The agenda entry scopes CMS-2450 to program integrity and enrollment and retains state directed payments and payment and access requirements in its abstract; no official description of its SDP content exists beyond that abstract, and no source ties it to the CMS-2449-P/CMS-2452-P interaction. Two EO 12866 meetings were held, both with home-care and HCBS groups EXTERNAL VERIFICATION, September 27, 2026 (D-16): the reginfo.gov review record for RIN 0938-AV70 (rrid 1379863) shows CMS-2450 received at OIRA on 05/12/2026, matching the status box's 'since May 12, 2026' UPDATED October 11, 2026: v17 states the rule is 'under White House review since May 12, 2026' and that its agenda entry states an intent to rescind or revise parts of CMS's 2024 managed care rule, including SDP requirements (sec. 9 item 4), and gives the RIN in App. I. The May 12 date was externally verified at D-16 (September 27, 2026) but sits on the decision-log re-check list. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov could not be fetched (www.reginfo.gov refused). The federalregister.gov API (reachable) lists no Federal Register document under RIN 0938-AV70.</t>
+          <t>Monitored at M-6. The agenda entry scopes CMS-2450 to program integrity and enrollment and retains state directed payments and payment and access requirements in its abstract; no official description of its SDP content exists beyond that abstract, and no source ties it to the CMS-2449-P/CMS-2452-P interaction. Two EO 12866 meetings were held, both with home-care and HCBS groups EXTERNAL VERIFICATION, September 27, 2026 (D-16): the reginfo.gov review record for RIN 0938-AV70 (rrid 1379863) shows CMS-2450 received at OIRA on 05/12/2026, matching the status box's 'since May 12, 2026' UPDATED October 11, 2026: v17 states the rule is 'under White House review since May 12, 2026' and that its agenda entry states an intent to rescind or revise parts of CMS's 2024 managed care rule, including SDP requirements (sec. 9 item 4), and gives the RIN in App. I. The May 12 date was externally verified at D-16 (September 27, 2026) but sits on the decision-log re-check list. VERIFIED October 13, 2026, second pass (verification_v4_log.md): reginfo.gov review record (https://www.reginfo.gov/public/do/eoDetails?rrid=1379863): RIN 0938-AV70, CMS-2450, received 05/12/2026, still 'Pending EO 12866 Regulatory Review' on October 13, 2026; agenda entry (https://www.reginfo.gov/public/do/eAgendaViewRule?pubId=202510&amp;RIN=0938-AV70): abstract covers state enrollment, 'state directed payments and other payment and access requirements', and the statement of need includes 'rescinding or revising provisions finalized in the 2024 final rules'. Matched by script.</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see M-6; perishable, and the rule's text remains non-public — NEEDS VERIFICATION [DL3] CMS-2450 (RIN 0938-AV70), its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
+          <t>verified as scoped — see M-6; perishable, and the rule's text remains non-public — re-checked October 13, 2026, second pass: reginfo.gov matches (CMS-2450, RIN 0938-AV70, received May 12, 2026, still pending; agenda entry covers SDPs and rescinding or revising 2024 provisions).</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-6, the same trigger as RM-23; this row restates the agenda-entry finding as a forward-looking monitoring item, not a new claim UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Publication of CMS-2450 would materially change the exposure picture; its agenda entry states an intent to rescind or revise provisions of the 2024 managed care rule, which include requirements governing state directed payments' BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov could not be fetched (www.reginfo.gov refused). The federalregister.gov API (reachable) lists no Federal Register document under RIN 0938-AV70.</t>
+          <t>Monitored at M-6, the same trigger as RM-23; this row restates the agenda-entry finding as a forward-looking monitoring item, not a new claim UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Publication of CMS-2450 would materially change the exposure picture; its agenda entry states an intent to rescind or revise provisions of the 2024 managed care rule, which include requirements governing state directed payments' VERIFIED October 13, 2026, second pass (verification_v4_log.md): reginfo.gov review record (https://www.reginfo.gov/public/do/eoDetails?rrid=1379863): RIN 0938-AV70, CMS-2450, received 05/12/2026, still 'Pending EO 12866 Regulatory Review' on October 13, 2026; agenda entry (https://www.reginfo.gov/public/do/eAgendaViewRule?pubId=202510&amp;RIN=0938-AV70): abstract covers state enrollment, 'state directed payments and other payment and access requirements', and the statement of need includes 'rescinding or revising provisions finalized in the 2024 final rules'. Matched by script.</t>
         </is>
       </c>
       <c r="N25" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped — see M-6; conditional on publication — NEEDS VERIFICATION [DL3] CMS-2450, its agenda entry and the May 12, 2026 review date are on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
+          <t>verified as scoped — see M-6; conditional on publication — re-checked October 13, 2026, second pass: reginfo.gov matches (as RM-23).</t>
         </is>
       </c>
     </row>
@@ -2417,12 +2417,12 @@
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later' BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) articles could not be fetched: the proxy refused both hosts.</t>
+          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): Fierce Healthcare's September 18, 2026 article (https://www.fiercehealthcare.com/providers/cms-restores-12b-frozen-supplemental-medicaid-funds) answered a Cloudflare challenge. The Texas Tribune limb matches (https://www.texastribune.org/2026/09/17/texas-medicaid-hospitals-greg-abbott-federal-impasse/, matched by script): the halt began Sept. 1, the start of Texas's fiscal year, in a dispute over how Texas raises the taxes, and about $12 billion was restored on Sept. 17 (16 days, so 'about two and a half weeks' is closer to 'about two weeks'). URL to open: https://www.fiercehealthcare.com/providers/cms-restores-12b-frozen-supplemental-medicaid-funds. Texas Tribune limb matches.</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>single-source — two outlets now cited in the note but neither re-read for this ledger; the dollar detail rests on the reference case at M-7 — NEEDS VERIFICATION [DL3] Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) are on the decision-log re-check list (sec. 9 item 5); neither was re-read for this ledger. blocked: www.texastribune.org; www.fiercehealthcare.com (re-checked October 13, 2026).</t>
+          <t>single-source — two outlets now cited in the note but neither re-read for this ledger; the dollar detail rests on the reference case at M-7 — NEEDS VERIFICATION [DL3] Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) are on the decision-log re-check list (sec. 9 item 5); neither was re-read for this ledger. blocked: www.fiercehealthcare.com (site refused); re-checked October 13, 2026, second pass. Texas Tribune limb matches.</t>
         </is>
       </c>
     </row>
@@ -2921,12 +2921,12 @@
       </c>
       <c r="M33" s="12" t="inlineStr">
         <is>
-          <t>The observability limb [E] is the same public list checked at RM-10 and scoped at C-6. The 'imminent final action' limb is [FIRM]'s inference [I]. Trigger M-2 UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Transmission of either RIN to OMB is visible on reginfo.gov and marks the move from proposal to imminent final action' BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
+          <t>The observability limb [E] is the same public list checked at RM-10 and scoped at C-6. The 'imminent final action' limb is [FIRM]'s inference [I]. Trigger M-2 UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Transmission of either RIN to OMB is visible on reginfo.gov and marks the move from proposal to imminent final action' VERIFIED October 13, 2026, second pass (verification_v4_log.md): reginfo.gov, read October 13, 2026: the EO 12866 'rules under review' XML (RUNDATE 2026-10-13; https://www.reginfo.gov/public/do/XMLViewFileAction?f=EO_RULES_UNDER_REVIEW.xml) lists RIN 0938-AV70 (CMS-2450, received 05/12/2026) and neither 0938-AV69 nor 0938-AV93; this year's completed list shows OIRA concluded review of both proposed rules (AV69 on 2026-05-19, AV93 on 2026-07-21). Matched by script against the downloaded XML.</t>
         </is>
       </c>
       <c r="N33" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - second limb is inference — NEEDS VERIFICATION [DL3] reginfo.gov is on the decision-log re-check list (sec. 9 items 3–4; App. I). blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
+          <t>verified with caveat - second limb is inference — re-checked October 13, 2026, second pass: reginfo.gov's review list shows each rule under review by RIN (it shows CMS-2450 today); the 'final rule is near' limb stays [I].</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="M46" s="12" t="inlineStr">
         <is>
-          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18. BLOCKED October 13, 2026 (verification_v4_log.md): The SDP preprint form could not be fetched: the proxy refused www.medicaid.gov. Neither proposed rule reproduces the form's Section VI (searched 91 FR 30400–30466 and 46562–46599 by script), and no comment in either docket reproduces it (full-docket search).</t>
+          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): medicaid.gov answered 'Access Denied' (Akamai, HTTP 403) for the SDP guidance page and the preprint template. URL to open: https://www.medicaid.gov/medicaid/managed-care/downloads/sdp-4386c-preprint-template.pdf.</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>single-source — the preprint form was not read in the verification files — NEEDS VERIFICATION [DL3] SDP preprint, Section VI (financing fields) is on the decision-log re-check list (sec. 7 step 3). blocked: www.medicaid.gov (re-checked October 13, 2026).</t>
+          <t>single-source — the preprint form was not read in the verification files — NEEDS VERIFICATION [DL3] SDP preprint, Section VI (financing fields) is on the decision-log re-check list (sec. 7 step 3). blocked: www.medicaid.gov (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -10049,12 +10049,12 @@
       </c>
       <c r="M132" s="12" t="inlineStr">
         <is>
-          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter' BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
+          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
         </is>
       </c>
       <c r="N132" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — single publisher, no corroborating outlet located — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
+          <t>verified with caveat — single publisher, no corroborating outlet located — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -10121,12 +10121,12 @@
       </c>
       <c r="M133" s="12" t="inlineStr">
         <is>
-          <t>Internal: 756 + 265 − 340 = 681 exactly BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
+          <t>Internal: 756 + 265 − 340 = 681 exactly BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
         </is>
       </c>
       <c r="N133" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -10193,12 +10193,12 @@
       </c>
       <c r="M134" s="12" t="inlineStr">
         <is>
-          <t>The note relies on this phrase to avoid attributing the figure to any hospital association BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article could not be fetched: the proxy refused www.politico.com.</t>
+          <t>The note relies on this phrase to avoid attributing the figure to any hospital association BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
         </is>
       </c>
       <c r="N134" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -11273,12 +11273,12 @@
       </c>
       <c r="M149" s="12" t="inlineStr">
         <is>
-          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source' BLOCKED October 13, 2026 (verification_v4_log.md): POLITICO's September 2, 2026 article (www.politico.com refused) and CBO's July 21, 2025 table (www.cbo.gov answered 403) could not be fetched.</t>
+          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge and cbo.gov a JavaScript bot check (HTTP 403). The CBO files mentioned in the request were not among the session's uploads (only the ledger md and xlsx and the v17 docx are there), so CBO's July 21, 2025 Table 7 was not read. URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch); https://www.cbo.gov/publication/61570.</t>
         </is>
       </c>
       <c r="N149" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com; www.cbo.gov (re-checked October 13, 2026).</t>
+          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com; www.cbo.gov (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -12425,12 +12425,12 @@
       </c>
       <c r="M165" s="12" t="inlineStr">
         <is>
-          <t>C3 output retrieved the full article text and confirms this is the only passage containing all three figures UPDATED October 11, 2026: v17 quotes only the final fragment ('leaving a net decrease of $56.6 billion') and paraphrases the rest; the full passage remains as recorded in the Quote column. Previous wording: 'HFMA reports $220.3B, $163.7B and $56.6B in a single passage' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched: the proxy refused www.hfma.org.</t>
+          <t>C3 output retrieved the full article text and confirms this is the only passage containing all three figures UPDATED October 11, 2026: v17 quotes only the final fragment ('leaving a net decrease of $56.6 billion') and paraphrases the rest; the full passage remains as recorded in the Quote column. Previous wording: 'HFMA reports $220.3B, $163.7B and $56.6B in a single passage' VERIFIED October 13, 2026, second pass (verification_v4_log.md): HFMA, 'Medicaid provider tax proposed rule could cut payments by $220 billion over 10 years', published July 22, 2026, updated July 23, 2026 (https://www.hfma.org/payment-reimbursement-and-managed-care/medicaid-provider-tax-proposed-rule/), matched by script. Caveat: the article now reads 'Providers would face a projected net deficit … That's because Medicaid payments …'; the ledger's Quote column ('Providers would end up with a net deficit …') does not match the current text, probably the July 22 version before the July 23 update. v17's own quotation, 'leaving a net decrease of $56.6 billion', matches.</t>
         </is>
       </c>
       <c r="N165" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). The ledger's own C3 output retrieved the full text; the public-comment review did not re-check it. blocked: www.hfma.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: HFMA matches ($220.3 billion lower payments; $163.7 billion in taxes saved; 'leaving a net decrease of $56.6 billion'); the ledger's longer quotation predates HFMA's July 23 update.</t>
         </is>
       </c>
     </row>
@@ -12641,12 +12641,12 @@
       </c>
       <c r="M168" s="12" t="inlineStr">
         <is>
-          <t>C3 output finding (b) confirms verbatim; P4 independently confirms UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'HFMA's stated baseline is a scenario with no OBBBA and no proposed rule' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched: the proxy refused www.hfma.org.</t>
+          <t>C3 output finding (b) confirms verbatim; P4 independently confirms UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'HFMA's stated baseline is a scenario with no OBBBA and no proposed rule' VERIFIED October 13, 2026, second pass (verification_v4_log.md): HFMA, 'Medicaid provider tax proposed rule could cut payments by $220 billion over 10 years', published July 22, 2026, updated July 23, 2026 (https://www.hfma.org/payment-reimbursement-and-managed-care/medicaid-provider-tax-proposed-rule/), matched by script. Caveat: the article now reads 'Providers would face a projected net deficit … That's because Medicaid payments …'; the ledger's Quote column ('Providers would end up with a net deficit …') does not match the current text, probably the July 22 version before the July 23 update. v17's own quotation, 'leaving a net decrease of $56.6 billion', matches.</t>
         </is>
       </c>
       <c r="N168" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: HFMA matches ('compared with a scenario in which there is no OBBBA and no proposed rule').</t>
         </is>
       </c>
     </row>
@@ -12929,12 +12929,12 @@
       </c>
       <c r="M172" s="12" t="inlineStr">
         <is>
-          <t>C3 output retrieved and quotes the sentence; this is the note's only external corroboration of CE-36 (formerly CE-13) UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Georgetown CCF reports the $220.3B with the qualification that it is after the reduction in taxes paid by providers' BLOCKED October 13, 2026 (verification_v4_log.md): Georgetown CCF's July 27, 2026 post could not be fetched: the proxy refused ccf.georgetown.edu. CCF's own comment on CMS-2452-P (CMS-2026-2476-0029) is posted, but it is not the cited post.</t>
+          <t>C3 output retrieved and quotes the sentence; this is the note's only external corroboration of CE-36 (formerly CE-13) UPDATED October 11, 2026: claim reworded to the note's current text (v17). Previous wording: 'Georgetown CCF reports the $220.3B with the qualification that it is after the reduction in taxes paid by providers' VERIFIED October 13, 2026, second pass (verification_v4_log.md): Georgetown CCF, 'CMS Issues New Rule Again Going Beyond H.R. 1 Requirements to Further Restrict State Use of Medicaid Provider Taxes' (https://ccf.georgetown.edu/2026/07/27/cms-issues-new-rule-again-going-beyond-h-r-1-requirements-to-further-restrict-state-use-of-medicaid-provider-taxes/), matched by script.</t>
         </is>
       </c>
       <c r="N172" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] Georgetown CCF, July 27, 2026 is on the decision-log re-check list (sec. 5, HFMA paragraph). blocked: ccf.georgetown.edu (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: Georgetown CCF's July 27, 2026 post matches.</t>
         </is>
       </c>
     </row>
@@ -13073,12 +13073,12 @@
       </c>
       <c r="M174" s="12" t="inlineStr">
         <is>
-          <t>V1 output located and verified the quote at p. 11 and confirms it is not a headline savings figure EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version of the report carries the same $891B and $875B figures as the August 12 version the note cites UPDATED October 11, 2026: v17 no longer calls the $891B a 'sensitivity-analysis estimate' or an input to the $875B benefit estimate, and does not state the $875B. The p. 11 quote and the external verification of the September 2 version stand. Previous wording: 'ASPE's $891B is a sensitivity-analysis estimate of total federal-plus-state Medicaid spending reduction from the combined provisions, used as an intermediate input to its $875B benefit estimate' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>V1 output located and verified the quote at p. 11 and confirms it is not a headline savings figure EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version of the report carries the same $891B and $875B figures as the August 12 version the note cites UPDATED October 11, 2026: v17 no longer calls the $891B a 'sensitivity-analysis estimate' or an input to the $875B benefit estimate, and does not state the $875B. The p. 11 quote and the external verification of the September 2 version stand. Previous wording: 'ASPE's $891B is a sensitivity-analysis estimate of total federal-plus-state Medicaid spending reduction from the combined provisions, used as an intermediate input to its $875B benefit estimate' VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title.</t>
         </is>
       </c>
       <c r="N174" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: ASPE matches ($891 billion total federal and state savings, 2025-2034, used to estimate benefits).</t>
         </is>
       </c>
     </row>
@@ -13145,12 +13145,12 @@
       </c>
       <c r="M175" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms, and further establishes that the double-counting language circulating alongside this figure traces to KFF's companion brief rather than to ASPE UPDATED October 11, 2026: v17 states the point as THEIA's reading of what ASPE does not say. The earlier support (ASPE's combined federal savings 'about the size of the SDP effect alone ($510 billion) estimated by OACT') is no longer stated in v17 and remains ledger evidence. Previous wording: 'ASPE does not describe the $891B as adjusted for double counting; it notes its combined estimate is about the size of the SDP effect alone as estimated by OACT' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>V1 output confirms, and further establishes that the double-counting language circulating alongside this figure traces to KFF's companion brief rather than to ASPE UPDATED October 11, 2026: v17 states the point as THEIA's reading of what ASPE does not say. The earlier support (ASPE's combined federal savings 'about the size of the SDP effect alone ($510 billion) estimated by OACT') is no longer stated in v17 and remains ledger evidence. Previous wording: 'ASPE does not describe the $891B as adjusted for double counting; it notes its combined estimate is about the size of the SDP effect alone as estimated by OACT' VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title. A full-text search of the page finds no 'overlap', 'interaction' or 'double'; the negative is therefore confirmed by search.</t>
         </is>
       </c>
       <c r="N175" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: ASPE matches (federal estimate 'about the size of the SDP effect alone ($510 billion)'; no mention of overlap or interaction anywhere in the report).</t>
         </is>
       </c>
     </row>
@@ -13217,12 +13217,12 @@
       </c>
       <c r="M176" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms both figures and the $100–175B annual benefit once phased in EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version carries the same $502–875B and 3.5 percent figures as the August 12 version the note cites UPDATED October 11, 2026: citation and location restated to v17 (changed: cite). BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>V1 output confirms both figures and the $100–175B annual benefit once phased in EXTERNAL VERIFICATION, September 27, 2026 (D-16): ASPE's September 2, 2026 version carries the same $502–875B and 3.5 percent figures as the August 12 version the note cites UPDATED October 11, 2026: citation and location restated to v17 (changed: cite). VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title.</t>
         </is>
       </c>
       <c r="N176" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: ASPE Key Points match (up to 3.5 percent lower non-Medicaid prices; $502-$875 billion to non-Medicaid payers, 2025-2034).</t>
         </is>
       </c>
     </row>
@@ -13289,12 +13289,12 @@
       </c>
       <c r="M177" s="12" t="inlineStr">
         <is>
-          <t>V1 output confirms the report analyzes Sections 71115–71117 and cites the proposed rules only as data inputs UPDATED October 11, 2026: v17 words the difference as statute-level scoring and different years; it no longer states the dollar basis (unstated vs real 2026) or that the report analyzes Section 71117. The V1 confirmation stands. The conclusion about THEIA's $916.9B is at TP-26. Previous wording: 'ASPE analyzes the statute rather than either proposed rule, on a different horizon and dollar basis' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>V1 output confirms the report analyzes Sections 71115–71117 and cites the proposed rules only as data inputs UPDATED October 11, 2026: v17 words the difference as statute-level scoring and different years; it no longer states the dollar basis (unstated vs real 2026) or that the report analyzes Section 71117. The V1 confirmation stands. The conclusion about THEIA's $916.9B is at TP-26. Previous wording: 'ASPE analyzes the statute rather than either proposed rule, on a different horizon and dollar basis' VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title.</t>
         </is>
       </c>
       <c r="N177" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: ASPE matches: its three estimates rescale RAND's and CBO's scores of the legislation over 2025-2034 (footnote xxii on RAND), not CMS's proposed rules over 2026-2035.</t>
         </is>
       </c>
     </row>
@@ -13361,12 +13361,12 @@
       </c>
       <c r="M178" s="12" t="inlineStr">
         <is>
-          <t>Internal: both attribute part of the effect to commercial payers, but the horizons, bases and objects of analysis differ, so no numerical reconciliation is attempted or possible BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>Internal: both attribute part of the effect to commercial payers, but the horizons, bases and objects of analysis differ, so no numerical reconciliation is attempted or possible VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title.</t>
         </is>
       </c>
       <c r="N178" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — interpretive, not an equivalence — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified with caveat — interpretive, not an equivalence — re-checked October 13, 2026, second pass: ASPE's price finding is confirmed; the 'counterpart' of CMS's $35.0 billion stays THEIA Services' [I] reading.</t>
         </is>
       </c>
     </row>
@@ -13433,12 +13433,12 @@
       </c>
       <c r="M179" s="12" t="inlineStr">
         <is>
-          <t>Internal: 154.9 rounds to 155. V1 output locates and quotes the KFF sentence and confirms it refers to OACT's $510B SDP estimate UPDATED September 27, 2026: the note now cites the KFF brief by title and date (August 14, 2026), the same brief as SE-01 UPDATED October 11, 2026: v17 words the first limb as KFF's report [E] and the match with CMS's $154.9B as THEIA's [I]. Previous wording: 'KFF's widely repeated $155B is the federal share of CMS's $241.9B overlap finding' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief could not be fetched (www.kff.org refused). The CMS limb matches: 91 FR 46592 gives federal spending reductions $154.9 billion less after counting the SDP rule and the $241.9 billion overlap (CMS-2452-P, govinfo PDF (FR Doc. 2026-14897), matched by script).</t>
+          <t>Internal: 154.9 rounds to 155. V1 output locates and quotes the KFF sentence and confirms it refers to OACT's $510B SDP estimate UPDATED September 27, 2026: the note now cites the KFF brief by title and date (August 14, 2026), the same brief as SE-01 UPDATED October 11, 2026: v17 words the first limb as KFF's report [E] and the match with CMS's $154.9B as THEIA's [I]. Previous wording: 'KFF's widely repeated $155B is the federal share of CMS's $241.9B overlap finding' VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script. KFF dates CMS's $510 billion as 2026-2034; CMS's own window is 2026-2035 (91 FR 30451). v17 states no window for KFF's figure, so nothing changes.</t>
         </is>
       </c>
       <c r="N179" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: KFF brief matches ($155 billion of the $510 billion 'also part of the reduced spending stemming from changes to provider tax rules'); CMS's $154.9 billion at 91 FR 46592 matched earlier.</t>
         </is>
       </c>
     </row>
@@ -13577,12 +13577,12 @@
       </c>
       <c r="M181" s="12" t="inlineStr">
         <is>
-          <t>This is the instance whose existence bounds NC-09: paired figures exist for at least one state, a consistent multi-state version does not. No figures are reproduced in the note, so nothing here is arithmetically checkable UPDATED September 27, 2026: the note now gives the publication's title and year (2025, while the reconciliation law was pending). Not re-read for this ledger UPDATED October 11, 2026: v17 words this as 'a state hospital association' (sec. 9 item 10) and names the Texas Hospital Association in App. F; the earlier 'for both mechanisms' qualifier is not stated. Not re-read for this ledger. Previous wording: 'The Texas Hospital Association publishes paired gross and net figures for both mechanisms' BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Hospital Association's 2025 publication with paired gross and net figures could not be fetched: the proxy refused www.tha.org. THA's comment on CMS-2452-P (CMS-2026-2476-0109) is posted but is not the cited publication.</t>
+          <t>This is the instance whose existence bounds NC-09: paired figures exist for at least one state, a consistent multi-state version does not. No figures are reproduced in the note, so nothing here is arithmetically checkable UPDATED September 27, 2026: the note now gives the publication's title and year (2025, while the reconciliation law was pending). Not re-read for this ledger UPDATED October 11, 2026: v17 words this as 'a state hospital association' (sec. 9 item 10) and names the Texas Hospital Association in App. F; the earlier 'for both mechanisms' qualifier is not stated. Not re-read for this ledger. Previous wording: 'The Texas Hospital Association publishes paired gross and net figures for both mechanisms' VERIFIED October 13, 2026, second pass (verification_v4_log.md): Texas Hospital Association, 'Proposed Medicaid Cuts Would Have Catastrophic Impact On Texas' (PDF created April 2025; https://www.tha.org/wp-content/uploads/2025/04/2025_Medicaid_Proposed_Cuts_Reconciliation.pdf), matched by script: each provider-tax scenario gives a gross loss to Texas Medicaid and a net loss to hospitals.</t>
         </is>
       </c>
       <c r="N181" s="12" t="inlineStr">
         <is>
-          <t>single-source - existence claim only, no figures reproduced — NEEDS VERIFICATION [DL3] Texas Hospital Association paired gross and net figures, 2025, are on the decision-log re-check list (App. F; sec. 9 item 10). blocked: www.tha.org (re-checked October 13, 2026).</t>
+          <t>single-source - existence claim only, no figures reproduced — re-checked October 13, 2026, second pass: THA's 2025 publication matches (paired gross and net figures).</t>
         </is>
       </c>
     </row>
@@ -14009,12 +14009,12 @@
       </c>
       <c r="M187" s="12" t="inlineStr">
         <is>
-          <t>HFMA wording at TP-04. CMS's 'pre-statute' baseline and the Tables 5, 9, 10 captions verified at D-16 (CE-43). Replaces TP-05. Resolves D-9 in HFMA's favour UPDATED October 11, 2026: v17 states the match as 'HFMA's July 22, 2026 article, which describes the same no-OBBBA comparison point as CMS'. BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched (www.hfma.org refused). The CMS limb (no-OBBBA baseline, Tables 5, 9, 10) was verified at D-16 and is not affected.</t>
+          <t>HFMA wording at TP-04. CMS's 'pre-statute' baseline and the Tables 5, 9, 10 captions verified at D-16 (CE-43). Replaces TP-05. Resolves D-9 in HFMA's favour UPDATED October 11, 2026: v17 states the match as 'HFMA's July 22, 2026 article, which describes the same no-OBBBA comparison point as CMS'. VERIFIED October 13, 2026, second pass (verification_v4_log.md): HFMA, 'Medicaid provider tax proposed rule could cut payments by $220 billion over 10 years', published July 22, 2026, updated July 23, 2026 (https://www.hfma.org/payment-reimbursement-and-managed-care/medicaid-provider-tax-proposed-rule/), matched by script. Caveat: the article now reads 'Providers would face a projected net deficit … That's because Medicaid payments …'; the ledger's Quote column ('Providers would end up with a net deficit …') does not match the current text, probably the July 22 version before the July 23 update. v17's own quotation, 'leaving a net decrease of $56.6 billion', matches.</t>
         </is>
       </c>
       <c r="N187" s="12" t="inlineStr">
         <is>
-          <t>verified - pre-statute baseline verified at D-16 — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
+          <t>verified - pre-statute baseline verified at D-16 — re-checked October 13, 2026, second pass: HFMA's stated baseline matches; CMS's no-OBBBA baseline was verified at D-16.</t>
         </is>
       </c>
     </row>
@@ -14081,12 +14081,12 @@
       </c>
       <c r="M188" s="12" t="inlineStr">
         <is>
-          <t>Internal: 220.3 − 163.7 = 56.6 exactly, and CE-36 establishes that 220.3 is already net of the same 163.7. Absence of 56.6 from both RIAs at TP-07 and NC-08. Georgetown CCF's net reading at TP-08. Replaces TP-06, which stated the double subtraction as fact UPDATED October 11, 2026: v17 drops two clauses of the earlier wording: 'or it comes from a source the note did not locate' and 'the components HFMA cites are correct'. The Table 12 caption evidence is at CE-37. Previous wording: 'On the note's reading, the $56.6B is Table 12's provider line with the tax relief counted a second time, or it comes from a source the note did not locate. The components HFMA cites are correct. If the reading is right, the $56.6B understates the rule's standalone net provider reduction, which is $220.3B' BLOCKED October 13, 2026 (verification_v4_log.md): HFMA's July 22, 2026 article could not be fetched (www.hfma.org refused). The CMS figures match by script: Table 8 at 91 FR 46590 gives $163.7 billion in lower taxes paid by providers and Table 12 at 46592 a provider line of −$220.3 billion (CMS-2452-P, govinfo PDF (FR Doc. 2026-14897)); 220.3 − 163.7 = 56.6.</t>
+          <t>Internal: 220.3 − 163.7 = 56.6 exactly, and CE-36 establishes that 220.3 is already net of the same 163.7. Absence of 56.6 from both RIAs at TP-07 and NC-08. Georgetown CCF's net reading at TP-08. Replaces TP-06, which stated the double subtraction as fact UPDATED October 11, 2026: v17 drops two clauses of the earlier wording: 'or it comes from a source the note did not locate' and 'the components HFMA cites are correct'. The Table 12 caption evidence is at CE-37. Previous wording: 'On the note's reading, the $56.6B is Table 12's provider line with the tax relief counted a second time, or it comes from a source the note did not locate. The components HFMA cites are correct. If the reading is right, the $56.6B understates the rule's standalone net provider reduction, which is $220.3B' VERIFIED October 13, 2026, second pass (verification_v4_log.md): HFMA, 'Medicaid provider tax proposed rule could cut payments by $220 billion over 10 years', published July 22, 2026, updated July 23, 2026 (https://www.hfma.org/payment-reimbursement-and-managed-care/medicaid-provider-tax-proposed-rule/), matched by script. Caveat: the article now reads 'Providers would face a projected net deficit … That's because Medicaid payments …'; the ledger's Quote column ('Providers would end up with a net deficit …') does not match the current text, probably the July 22 version before the July 23 update. v17's own quotation, 'leaving a net decrease of $56.6 billion', matches.</t>
         </is>
       </c>
       <c r="N188" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - the arithmetic closes; the note presents it as a reading — NEEDS VERIFICATION [DL3] HFMA, July 22, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.hfma.org (re-checked October 13, 2026).</t>
+          <t>verified with caveat - the arithmetic closes; the note presents it as a reading — re-checked October 13, 2026, second pass: HFMA's figures match ($220.3 billion, $163.7 billion, $56.6 billion; 220.3 - 163.7 = 56.6); the double-subtraction stays THEIA Services' [I] reading.</t>
         </is>
       </c>
     </row>
@@ -14225,12 +14225,12 @@
       </c>
       <c r="M190" s="12" t="inlineStr">
         <is>
-          <t>TP-10 for the $891B; CE-38 for the $916.9B. The note draws no inference, and the ledger draws none UPDATED October 11, 2026: v17 states the comparison as a cannot-compare conclusion; the earlier 'for scale' wording ('no inference about ASPE's treatment of overlap is drawn') is not stated. The bases are at TP-13. Previous wording: 'For scale, CMS's overlap-adjusted combined estimate is $916.9B against ASPE's $891B; the windows and dollar bases differ, so no inference about ASPE's treatment of overlap is drawn' BLOCKED October 13, 2026 (verification_v4_log.md): ASPE's August 12, 2026 report could not be fetched: the proxy refused aspe.hhs.gov. (Paragon's comment CMS-2026-2476-0130 cites the report's URL but does not attach it.)</t>
+          <t>TP-10 for the $891B; CE-38 for the $916.9B. The note draws no inference, and the ledger draws none UPDATED October 11, 2026: v17 states the comparison as a cannot-compare conclusion; the earlier 'for scale' wording ('no inference about ASPE's treatment of overlap is drawn') is not stated. The bases are at TP-13. Previous wording: 'For scale, CMS's overlap-adjusted combined estimate is $916.9B against ASPE's $891B; the windows and dollar bases differ, so no inference about ASPE's treatment of overlap is drawn' VERIFIED October 13, 2026, second pass (verification_v4_log.md): ASPE, 'An Overview of State-Directed Payments and Medicaid Provider Taxes: History and Potential Effects of the Working Families and Tax Cut Legislation on Health Care Costs', Aug 12, 2026 (https://aspe.hhs.gov/reports/effects-working-families-tax-cut-legislation-health-care-costs), page text matched by script; the linked PDF is a September 2, 2026 version whose p. 11 carries the $891 billion passage. The ledger cites the title as 'Effects of the Working Families Tax Cut Legislation on Health Care Costs', which is the page's URL slug, not its title; v17 gives no title.</t>
         </is>
       </c>
       <c r="N190" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] ASPE, August 12, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: aspe.hhs.gov (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: ASPE's $891 billion and its 2025-2034 window match; the non-comparability is THEIA Services' [I] reading.</t>
         </is>
       </c>
     </row>
@@ -14513,12 +14513,12 @@
       </c>
       <c r="M194" s="12" t="inlineStr">
         <is>
-          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18. BLOCKED October 13, 2026 (verification_v4_log.md): GAO-24-106202 could not be fetched: the proxy refused www.gao.gov and files.gao.gov; govinfo's GAO collection does not carry it.</t>
+          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): gao.gov answered 'Access Denied' (Akamai, HTTP 403) for the product page and the PDF (https://www.gao.gov/assets/gao-24-106202.pdf). URL to open: https://www.gao.gov/products/gao-24-106202.</t>
         </is>
       </c>
       <c r="N194" s="12" t="inlineStr">
         <is>
-          <t>single-source — not re-read in the review or for this ledger — NEEDS VERIFICATION [DL3] GAO-24-106202, Table 4 is on the decision-log re-check list (sec. 2). blocked: www.gao.gov; files.gao.gov (re-checked October 13, 2026).</t>
+          <t>single-source — not re-read in the review or for this ledger — NEEDS VERIFICATION [DL3] GAO-24-106202, Table 4 is on the decision-log re-check list (sec. 2). blocked: www.gao.gov (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -15089,12 +15089,12 @@
       </c>
       <c r="M202" s="12" t="inlineStr">
         <is>
-          <t>The CMS limb is the net construction of Table 12 (CE-36). The distinction is v17's [I] reading; it keeps TP-21 and TP-37 from being read as support for a net-of-tax provider loss. Related: TP-17 (Texas Hospital Association paired figures). BLOCKED October 13, 2026 (verification_v4_log.md): The Texas Hospital Association's 2025 publication with paired gross and net figures could not be fetched: the proxy refused www.tha.org. THA's comment on CMS-2452-P (CMS-2026-2476-0109) is posted but is not the cited publication.</t>
+          <t>The CMS limb is the net construction of Table 12 (CE-36). The distinction is v17's [I] reading; it keeps TP-21 and TP-37 from being read as support for a net-of-tax provider loss. Related: TP-17 (Texas Hospital Association paired figures). VERIFIED October 13, 2026, second pass (verification_v4_log.md): Texas Hospital Association, 'Proposed Medicaid Cuts Would Have Catastrophic Impact On Texas' (PDF created April 2025; https://www.tha.org/wp-content/uploads/2025/04/2025_Medicaid_Proposed_Cuts_Reconciliation.pdf), matched by script: each provider-tax scenario gives a gross loss to Texas Medicaid and a net loss to hospitals.</t>
         </is>
       </c>
       <c r="N202" s="12" t="inlineStr">
         <is>
-          <t>verified as inference — NEEDS VERIFICATION [DL3] The Texas Hospital Association's paired gross and net figures (2025), which this note cites alongside CMS's netting (App. F), are on the decision-log re-check list. blocked: www.tha.org (re-checked October 13, 2026).</t>
+          <t>verified as inference — re-checked October 13, 2026, second pass: THA's paired gross and net figures (2025) match; the cap-test reading stays [I].</t>
         </is>
       </c>
     </row>
@@ -15305,12 +15305,12 @@
       </c>
       <c r="M205" s="12" t="inlineStr">
         <is>
-          <t>C4: 51 jurisdictions less the 14 with no hospital SDPs = 37 exactly UPDATED October 11, 2026: v17 words the count as 37 states 'including DC' that 'likely exceed the new caps' and tags it [E]. KFF's own wording is 'at least 37 states' with SDPs that 'could be reduced'; the note's 'likely exceed' is a paraphrase. The 51 less 14 arithmetic is unchanged. The KFF brief was not re-read this cycle (kff.org was unreachable in the verification files). Previous wording: 'KFF identifies 37 states with hospital SDPs likely affected by the new limits' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: 51 jurisdictions less the 14 with no hospital SDPs = 37 exactly UPDATED October 11, 2026: v17 words the count as 37 states 'including DC' that 'likely exceed the new caps' and tags it [E]. KFF's own wording is 'at least 37 states' with SDPs that 'could be reduced'; the note's 'likely exceed' is a paraphrase. The 51 less 14 arithmetic is unchanged. The KFF brief was not re-read this cycle (kff.org was unreachable in the verification files). Previous wording: 'KFF identifies 37 states with hospital SDPs likely affected by the new limits' VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), downloaded and matched by script: 'At least 37 states have Medicaid state directed payments for hospital services that could be reduced …'; 'SDPs with payments for hospital services in 37 states are likely affected by the limits'; DC is among the states (100% share in Louisiana and DC).</t>
         </is>
       </c>
       <c r="N205" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: KFF brief matches (at least 37 states; hospital SDPs in 37 states 'likely affected by the limits'; DC counted as a state).</t>
         </is>
       </c>
     </row>
@@ -15377,12 +15377,12 @@
       </c>
       <c r="M206" s="12" t="inlineStr">
         <is>
-          <t>Internal: the note's own group dollar column sums to $60.1B. V1 output independently confirms the $78.0B denominator UPDATED October 11, 2026: v17 splits the KFF bullet in two, states that the $60 billion excludes Minnesota and Missouri, says 'one year's' spending and restores 'about $93 billion' in all federal SDP spending (change map S6.1; decision log, 'Numbers vs ledger'). The Group A-D dollar column in the v17 table is the same $60.1 billion by construction (SE-05 to SE-08). The brief was not re-read this cycle. Previous wording: 'Approximately $60B in federal hospital SDP spending sits above the new limits, out of roughly $78B federal hospital SDP spending, within roughly $93B total federal SDP spending' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>Internal: the note's own group dollar column sums to $60.1B. V1 output independently confirms the $78.0B denominator UPDATED October 11, 2026: v17 splits the KFF bullet in two, states that the $60 billion excludes Minnesota and Missouri, says 'one year's' spending and restores 'about $93 billion' in all federal SDP spending (change map S6.1; decision log, 'Numbers vs ledger'). The Group A-D dollar column in the v17 table is the same $60.1 billion by construction (SE-05 to SE-08). The brief was not re-read this cycle. Previous wording: 'Approximately $60B in federal hospital SDP spending sits above the new limits, out of roughly $78B federal hospital SDP spending, within roughly $93B total federal SDP spending' VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/) and KFF's June 15, 2026 companion brief, matched by script. 60/0.77 = 77.9 and 60/0.64 = 93.8, consistent with the companion brief's $78.0 billion and $93 billion.</t>
         </is>
       </c>
       <c r="N206" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: KFF matches: $60 billion (one 12-month period, Minnesota and Missouri excluded) is 64% of federal SDP spending and 77% of federal hospital SDP spending; KFF's June 15, 2026 brief gives $93 billion and $78.0 billion.</t>
         </is>
       </c>
     </row>
@@ -15449,12 +15449,12 @@
       </c>
       <c r="M207" s="12" t="inlineStr">
         <is>
-          <t>C4: NH 0.0910; DC 1.0000; LA 0.9995. Count of shares at or above 0.70 = 27 exactly UPDATED October 11, 2026: v17 moves this bullet from sec. 6 to App. H (change map U31, U49) and words it 'at least 70 percent in 27 states'. The 9 percent (New Hampshire) and 100 percent (Louisiana and DC) endpoints are unchanged. C4 re-derivation stands. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: NH 0.0910; DC 1.0000; LA 0.9995. Count of shares at or above 0.70 = 27 exactly UPDATED October 11, 2026: v17 moves this bullet from sec. 6 to App. H (change map U31, U49) and words it 'at least 70 percent in 27 states'. The 9 percent (New Hampshire) and 100 percent (Louisiana and DC) endpoints are unchanged. C4 re-derivation stands. VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script.</t>
         </is>
       </c>
       <c r="N207" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: KFF brief matches (9% in New Hampshire to 100% in Louisiana and DC; at least 70% in 27 states).</t>
         </is>
       </c>
     </row>
@@ -15521,12 +15521,12 @@
       </c>
       <c r="M208" s="12" t="inlineStr">
         <is>
-          <t>C4: exactly 28 expansion states carry hospital_tax_above_3_5 = Yes. The ambulance and MCO counts are not checkable from the available outputs UPDATED October 11, 2026: v17 words the claim '31 expansion states have a non-exempt provider tax above 3.5 percent: 28 with hospital taxes, 10 with ambulance taxes and 6 with managed care organization taxes' and moves it to sec. 6. Counts unchanged. The 'non-exempt' qualifier corresponds to the statutory exemption for nursing facility and ICF/IID taxes (RM-29). BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: exactly 28 expansion states carry hospital_tax_above_3_5 = Yes. The ambulance and MCO counts are not checkable from the available outputs UPDATED October 11, 2026: v17 words the claim '31 expansion states have a non-exempt provider tax above 3.5 percent: 28 with hospital taxes, 10 with ambulance taxes and 6 with managed care organization taxes' and moves it to sec. 6. Counts unchanged. The 'non-exempt' qualifier corresponds to the statutory exemption for nursing facility and ICF/IID taxes (RM-29). VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, August 20, 2026 (https://www.kff.org/medicaid/5-questions-and-answers-about-medicaid-and-provider-taxes/; the old '5-key-facts' URL redirects there), Figure 2 note, matched by script. The ledger's 'KFF provider tax file, Aug 2026' is this brief.</t>
         </is>
       </c>
       <c r="N208" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified with caveat — re-checked October 13, 2026, second pass: KFF's August 20, 2026 provider-tax brief matches (31 expansion states; 28 hospital, 6 MCO, 10 ambulance).</t>
         </is>
       </c>
     </row>
@@ -15593,12 +15593,12 @@
       </c>
       <c r="M209" s="12" t="inlineStr">
         <is>
-          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N209" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -15665,12 +15665,12 @@
       </c>
       <c r="M210" s="12" t="inlineStr">
         <is>
-          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N210" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -15737,12 +15737,12 @@
       </c>
       <c r="M211" s="12" t="inlineStr">
         <is>
-          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N211" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -15809,12 +15809,12 @@
       </c>
       <c r="M212" s="12" t="inlineStr">
         <is>
-          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N212" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -15881,12 +15881,12 @@
       </c>
       <c r="M213" s="12" t="inlineStr">
         <is>
-          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure' CORRECTED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script: KFF also notes Colorado submitted the SDP on June 27, 2025 (about $378 million) and that CMS posted it after KFF's cut-off. The 14-state list and the other limbs rest on KFF's chart data, which is on datawrapper.dwcdn.net (refused by the network policy).</t>
         </is>
       </c>
       <c r="N213" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>corrected — source says: “Colorado also has an SDP that is above new limits, but CMS did not post the preprint publicly until after July 20, 2026.” (KFF, Aug 14, 2026, Figure 1 note). v17 must change Sec. 6 (see verification_v4_log.md). Base status was verified. Other limbs: NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy).</t>
         </is>
       </c>
     </row>
@@ -15953,12 +15953,12 @@
       </c>
       <c r="M214" s="12" t="inlineStr">
         <is>
-          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
         </is>
       </c>
       <c r="N214" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
         </is>
       </c>
     </row>
@@ -16025,12 +16025,12 @@
       </c>
       <c r="M215" s="12" t="inlineStr">
         <is>
-          <t>C4: every non-expansion row reads "N/A - not assessed (non-expansion state)" and carries an explicit note that the tier is not evidence of lower exposure UPDATED October 11, 2026: v17 tags the first limb [E] (KFF did not assess) and the second [I] ('not evidence'), and adds that the lower threshold does not reach non-expansion states. The earlier 'Group D's tax indicators read not assessed' wording is replaced by 'KFF did not assess'. Previous wording: 'Group D's tax indicators read "not assessed," which is an absence of assessment rather than evidence of an absence of taxes above the threshold' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: every non-expansion row reads "N/A - not assessed (non-expansion state)" and carries an explicit note that the tier is not evidence of lower exposure UPDATED October 11, 2026: v17 tags the first limb [E] (KFF did not assess) and the second [I] ('not evidence'), and adds that the lower threshold does not reach non-expansion states. The earlier 'Group D's tax indicators read not assessed' wording is replaced by 'KFF did not assess'. Previous wording: 'Group D's tax indicators read "not assessed," which is an absence of assessment rather than evidence of an absence of taxes above the threshold' CORRECTED October 13, 2026, second pass (verification_v4_log.md): KFF, August 20, 2026 (https://www.kff.org/medicaid/5-questions-and-answers-about-medicaid-and-provider-taxes/), matched by script: Figure 2 reports provider taxes by size for all responding states (47 with hospital taxes), and its note limits the 3.5 percent count to expansion states and names three non-responding states. So KFF's survey did cover non-expansion states; what it did not do is count their taxes against 3.5 percent.</t>
         </is>
       </c>
       <c r="N215" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>corrected — source says: “FL, KS, and MS did not respond to the 2025 survey.” (KFF, Aug 20, 2026, Figure 2 note). v17 must change Sec. 6 (see verification_v4_log.md). Base status was verified.</t>
         </is>
       </c>
     </row>
@@ -16097,12 +16097,12 @@
       </c>
       <c r="M216" s="12" t="inlineStr">
         <is>
-          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): Texas limb matches the brief's text ('Texas ($3.5 billion)', matched by script); the Tennessee, Georgia and South Carolina amounts are only in the Figure 4 chart data on datawrapper.dwcdn.net, refused by the network policy. URL to open: https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/D5jCd/.</t>
         </is>
       </c>
       <c r="N216" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -16169,12 +16169,12 @@
       </c>
       <c r="M217" s="12" t="inlineStr">
         <is>
-          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N217" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -16241,12 +16241,12 @@
       </c>
       <c r="M218" s="12" t="inlineStr">
         <is>
-          <t>C4: both INSUFFICIENT with a blank share. The C4 response states the point directly — "their blank is not a zero" — and distinguishes them from the 14 determined zeros UPDATED October 11, 2026: v17 states the exclusion and 'no KFF estimate' and no longer says the two states' SDPs are 'benchmarked to average commercial rates'; that limb is no longer a note claim. v17 tags the whole sentence [E], but 'belong in Group A' is THEIA Services' own grouping (SE-17); the C4 check (both INSUFFICIENT with a blank share) supports the 'no estimate' limb only. Previous wording: 'Minnesota and Missouri have hospital SDPs benchmarked to average commercial rates but no estimable above-limit figure, and are excluded from the $45.4B' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: both INSUFFICIENT with a blank share. The C4 response states the point directly — "their blank is not a zero" — and distinguishes them from the 14 determined zeros UPDATED October 11, 2026: v17 states the exclusion and 'no KFF estimate' and no longer says the two states' SDPs are 'benchmarked to average commercial rates'; that limb is no longer a note claim. v17 tags the whole sentence [E], but 'belong in Group A' is THEIA Services' own grouping (SE-17); the C4 check (both INSUFFICIENT with a blank share) supports the 'no estimate' limb only. Previous wording: 'Minnesota and Missouri have hospital SDPs benchmarked to average commercial rates but no estimable above-limit figure, and are excluded from the $45.4B' VERIFIED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script.</t>
         </is>
       </c>
       <c r="N218" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — re-checked October 13, 2026, second pass: KFF brief matches: Minnesota and Missouri are among the 37 but excluded from the dollar analysis for insufficient data; 'belong in Group A' stays THEIA Services' grouping (SE-17).</t>
         </is>
       </c>
     </row>
@@ -16385,12 +16385,12 @@
       </c>
       <c r="M220" s="12" t="inlineStr">
         <is>
-          <t>none located beyond KFF itself UPDATED October 11, 2026: CORRECTED. The previous wording had KFF's base-rate finding backwards: it said a high share above the limits partly reflects low base payment rates. The finding runs the other way: states with most SDP spending above the caps already have base rates at or near the caps, and low base rates leave more SDP spending under the caps. v17 states it that way. The first limb, 'dollars above the caps do not show which states face the largest proportional effects', replaces the earlier 'do not show proportional effects' (change map S6.2, NTC 6.14). The change map records v17's base-rate wording as 'kept as in v16' (S6.2). The correction was instructed by the note's author and matches v17's text; the KFF brief itself could not be re-read here. Previous wording: 'KFF's caveat governs the dollar column: a high share above limits partly reflects low base payment rates rather than unusually generous supplemental payments' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>none located beyond KFF itself UPDATED October 11, 2026: CORRECTED. The previous wording had KFF's base-rate finding backwards: it said a high share above the limits partly reflects low base payment rates. The finding runs the other way: states with most SDP spending above the caps already have base rates at or near the caps, and low base rates leave more SDP spending under the caps. v17 states it that way. The first limb, 'dollars above the caps do not show which states face the largest proportional effects', replaces the earlier 'do not show proportional effects' (change map S6.2, NTC 6.14). The change map records v17's base-rate wording as 'kept as in v16' (S6.2). The correction was instructed by the note's author and matches v17's text; the KFF brief itself could not be re-read here. Previous wording: 'KFF's caveat governs the dollar column: a high share above limits partly reflects low base payment rates rather than unusually generous supplemental payments' CORRECTED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script. Base-rate limb matches: states with lower base rates have more SDP spending below the limits, and where most SDP spending exceeds the limits base payments are at or near them. First limb as SE-24.</t>
         </is>
       </c>
       <c r="N220" s="12" t="inlineStr">
         <is>
-          <t>single-source — direction corrected to match v17; KFF brief not re-read — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>corrected — source says: “The dollar amount of SDP spending above new limits may not indicate which states could have the biggest proportional effects” (KFF, Aug 14, 2026). v17 must change Sec. 6 (see verification_v4_log.md). Base status was single-source — direction corrected to match v17; KFF brief not re-read.</t>
         </is>
       </c>
     </row>
@@ -16673,12 +16673,12 @@
       </c>
       <c r="M224" s="12" t="inlineStr">
         <is>
-          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
         </is>
       </c>
       <c r="N224" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -16961,12 +16961,12 @@
       </c>
       <c r="M228" s="12" t="inlineStr">
         <is>
-          <t>First limb of the sentence at SE-16, split out so the base-rate direction can be tracked separately. The KFF brief was not re-read this cycle. No corroborating source located beyond KFF itself. BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>First limb of the sentence at SE-16, split out so the base-rate direction can be tracked separately. The KFF brief was not re-read this cycle. No corroborating source located beyond KFF itself. CORRECTED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script. KFF hedges ('may not indicate', 'could have'); v17 states it flatly.</t>
         </is>
       </c>
       <c r="N228" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>corrected — source says: “The dollar amount of SDP spending above new limits may not indicate which states could have the biggest proportional effects” (KFF, Aug 14, 2026). v17 must change Sec. 6 (see verification_v4_log.md). Base status was single-source.</t>
         </is>
       </c>
     </row>
@@ -17609,12 +17609,12 @@
       </c>
       <c r="M237" s="12" t="inlineStr">
         <is>
-          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services' BLOCKED October 13, 2026 (verification_v4_log.md): GAO-23-105515 could not be fetched: the proxy refused www.gao.gov and files.gao.gov.</t>
+          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): gao.gov answered 'Access Denied' (Akamai, HTTP 403) for the product page and the PDF (https://www.gao.gov/assets/gao-23-105515.pdf). URL to open: https://www.gao.gov/products/gao-23-105515.</t>
         </is>
       </c>
       <c r="N237" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — NEEDS VERIFICATION [DL3] GAO-23-105515 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: www.gao.gov; files.gao.gov (re-checked October 13, 2026).</t>
+          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — NEEDS VERIFICATION [DL3] GAO-23-105515 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: www.gao.gov (site refused); re-checked October 13, 2026, second pass.</t>
         </is>
       </c>
     </row>
@@ -17681,12 +17681,12 @@
       </c>
       <c r="M238" s="12" t="inlineStr">
         <is>
-          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period' BLOCKED October 13, 2026 (verification_v4_log.md): Michelson, Cushing and Bucholz, 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics 179(2):208–209 (doi:10.1001/jamapediatrics.2024.5110; PMC11612914). PubMed has no abstract, the PubMed connector returned no full text, and the proxy refused jamanetwork.com, pmc.ncbi.nlm.nih.gov and europepmc.org.</t>
+          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): The PubMed connector was tried first and again returned no full text for PMC11612914 (abstract only: 'This cross-sectional study evaluates recent trends in pediatric inpatient capacity …'); jamanetwork.com answered a Cloudflare challenge; pmc.ncbi.nlm.nih.gov was refused by the network policy. URL to open: https://jamanetwork.com/journals/jamapediatrics/fullarticle/2826774; https://pmc.ncbi.nlm.nih.gov/articles/PMC11612914/. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
         </is>
       </c>
       <c r="N238" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: jamanetwork.com; pmc.ncbi.nlm.nih.gov (re-checked October 13, 2026).</t>
+          <t>single-source — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: jamanetwork.com (site refused); re-checked October 13, 2026, second pass. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
         </is>
       </c>
     </row>
@@ -18617,12 +18617,12 @@
       </c>
       <c r="M251" s="12" t="inlineStr">
         <is>
-          <t>Re-dated from Sept 5 to Sept 21, 2026 in the Sept 22 currency check; AV69 confirmed on reginfo.gov. See RM-10 UPDATED October 11, 2026: v17 states no OIRA review-list status for either RIN. Sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading ('Status as of [DATE]: White House review, CMS-2450, comment periods and counts, HFMA contact') has no text under it. The September 21, 2026 check is stale against the October 2026 draft and is not restated in the note. See RM-10. BLOCKED October 13, 2026 (verification_v4_log.md): reginfo.gov's EO 12866 review list could not be fetched: the proxy refused www.reginfo.gov.</t>
+          <t>Re-dated from Sept 5 to Sept 21, 2026 in the Sept 22 currency check; AV69 confirmed on reginfo.gov. See RM-10 UPDATED October 11, 2026: v17 states no OIRA review-list status for either RIN. Sec. 9 item 3 describes only what an arrival for review would signal, and the App. I heading ('Status as of [DATE]: White House review, CMS-2450, comment periods and counts, HFMA contact') has no text under it. The September 21, 2026 check is stale against the October 2026 draft and is not restated in the note. See RM-10. VERIFIED October 13, 2026, second pass (verification_v4_log.md): reginfo.gov, read October 13, 2026: the EO 12866 'rules under review' XML (RUNDATE 2026-10-13; https://www.reginfo.gov/public/do/XMLViewFileAction?f=EO_RULES_UNDER_REVIEW.xml) lists RIN 0938-AV70 (CMS-2450, received 05/12/2026) and neither 0938-AV69 nor 0938-AV93; this year's completed list shows OIRA concluded review of both proposed rules (AV69 on 2026-05-19, AV93 on 2026-07-21). Matched by script against the downloaded XML.</t>
         </is>
       </c>
       <c r="N251" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped (C-6) — perishable; no longer stated in the note — NEEDS VERIFICATION [DL3] reginfo.gov and the White House review status are on the decision-log re-check list (sec. 9 items 3-4; App. I); re-run the OIRA list check at the date the note fills in. blocked: www.reginfo.gov (re-checked October 13, 2026).</t>
+          <t>verified as scoped (C-6) — perishable; no longer stated in the note — re-checked October 13, 2026, second pass: OIRA's list of rules under review, run October 13, 2026, shows neither RIN (0938-AV69, 0938-AV93); the check can now be dated October 13, 2026.</t>
         </is>
       </c>
     </row>
@@ -20129,12 +20129,12 @@
       </c>
       <c r="M272" s="12" t="inlineStr">
         <is>
-          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down' BLOCKED October 13, 2026 (verification_v4_log.md): KFF's August 14, 2026 brief, state file and expansion tracker could not be fetched: the proxy refused www.kff.org and files.kff.org.</t>
+          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
         </is>
       </c>
       <c r="N272" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: www.kff.org; files.kff.org (re-checked October 13, 2026).</t>
+          <t>verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
         </is>
       </c>
     </row>
@@ -20201,12 +20201,12 @@
       </c>
       <c r="M273" s="12" t="inlineStr">
         <is>
-          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)' BLOCKED October 13, 2026 (verification_v4_log.md): Michelson, Cushing and Bucholz, 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics 179(2):208–209 (doi:10.1001/jamapediatrics.2024.5110; PMC11612914). PubMed has no abstract, the PubMed connector returned no full text, and the proxy refused jamanetwork.com, pmc.ncbi.nlm.nih.gov and europepmc.org.</t>
+          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): The PubMed connector was tried first and again returned no full text for PMC11612914 (abstract only: 'This cross-sectional study evaluates recent trends in pediatric inpatient capacity …'); jamanetwork.com answered a Cloudflare challenge; pmc.ncbi.nlm.nih.gov was refused by the network policy. URL to open: https://jamanetwork.com/journals/jamapediatrics/fullarticle/2826774; https://pmc.ncbi.nlm.nih.gov/articles/PMC11612914/. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
         </is>
       </c>
       <c r="N273" s="12" t="inlineStr">
         <is>
-          <t>single-source - one study (AC-10); caption only in v17 — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (sec. 8); the figure rests on AC-10. blocked: jamanetwork.com; pmc.ncbi.nlm.nih.gov (re-checked October 13, 2026).</t>
+          <t>single-source - one study (AC-10); caption only in v17 — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (sec. 8); the figure rests on AC-10. blocked: jamanetwork.com (site refused); re-checked October 13, 2026, second pass. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
         </is>
       </c>
     </row>
@@ -20506,7 +20506,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Flag at the end of the Status column: the item is on the decision log's re-check list or the change map's lists. [DL3] re-check list; [DL4] comment ID to verify; [CM] Federal Register pinpoint from the new-text check. Shaded orange. The base status stands. After the October 13, 2026 check, a flag that remains ends with 'blocked: &lt;host&gt;' or 'not found'.</t>
+          <t>Flag at the end of the Status column: the item is on the decision log's re-check list or the change map's lists. [DL3] re-check list; [DL4] comment ID to verify; [CM] Federal Register pinpoint from the new-text check. Shaded orange. The base status stands. After the October 13, 2026 check, a flag that remains ends with 'not found' or 'blocked: &lt;host&gt;', and after the second pass the host is followed by '(site refused)', '(login)' or '(network policy)'.</t>
         </is>
       </c>
     </row>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. All 91 flagged rows were checked, in order: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list, the unresolved row AC-14. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text, except four rows on one journal article read through the PubMed connector (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 34 rows match and lose the flag (25 upgraded, for example single-source to verified); 8 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 49 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. No row text other than the Cross-check and Status columns was changed. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
+          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. All 91 flagged rows were checked, in order: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list, the unresolved row AC-14. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text, except four rows on one journal article read through the PubMed connector (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 58 rows match and lose the flag (25 upgraded, for example single-source to verified); 12 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 21 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 1 rows with two tags were resolved for one tag only and keep the other tag's flag. No row text other than the Cross-check and Status columns was changed. A second pass the same day, after the network policy was opened, re-ran the 47 rows blocked in the first pass: 24 now match, 4 are corrected and 19 stay blocked (politico.com, fiercehealthcare.com, jamanetwork.com, gao.gov, medicaid.gov and cbo.gov refused at the site; datawrapper.dwcdn.net, which serves KFF's state-level chart data, was refused by the network policy); the figures above include it. A remaining flag now ends 'blocked: &lt;host&gt; (site refused)', '(login)' or '(network policy)'. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ledger v4 verification: third pass, part 1 (user-supplied copies, KFF chart data)
Re-runs the 19 rows still blocked after the second pass, plus SE-09's
remaining limbs. Sources: user-supplied copies of POLITICO (Sept 2, 2026),
GAO-24-106202, GAO-23-105515, the SDP preprint template and Michelson et
al. (JAMA Pediatrics), and KFF's Datawrapper chart data. Every quote is
script-matched. The attached files are not committed; only their file
names and the extracted quotes are recorded.

Results: 12 rows match. 7 are corrected: TP-30, SE-09, SE-10, SE-13,
SE-20, FG-06 and FG-07. SB-18 is partly checked, with its CBO limb
pending part 2. As instructed, RM-25 now cites the Texas Tribune and
reads "about two weeks". Adds 261011_Ledger_change_log.md and the log
section "Blocked rows, third pass (part 1)". Legend formulas stay live.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016jFZZ5qaUFnBNLfBGt45ve
</commit_message>
<xml_diff>
--- a/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
+++ b/review/ledger/261011_Evidence_Ledger_SectionA_v4.xlsx
@@ -2367,7 +2367,7 @@
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>CMS approvals or renewals of individual SDPs under current rules can bring financing effects forward before either rule is final; in September 2026, one state's SDP programs lapsed at the start of its fiscal year during a dispute over its provider tax calculation, and CMS authorized them about two and a half weeks later</t>
+          <t>CMS approvals or renewals of individual SDPs under current rules can bring financing effects forward before either rule is final; in September 2026, one state's SDP programs lapsed at the start of its fiscal year during a dispute over its provider tax calculation, and CMS authorized them about two weeks later</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -2377,12 +2377,12 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Texas Tribune, September 17, 2026; Fierce Healthcare, September 18, 2026 (as cited in note sec. 7, item 6); CMS preprint approvals on Medicaid.gov; state announcements</t>
+          <t>Texas Tribune, September 17, 2026; CMS preprint approvals on Medicaid.gov; state announcements</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Note sec. 9, item 5; Texas Tribune, September 17, 2026; Fierce Healthcare, September 18, 2026</t>
+          <t>Note sec. 9, item 5; Texas Tribune, September 17, 2026</t>
         </is>
       </c>
       <c r="G26" s="12" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="J26" s="12" t="inlineStr">
         <is>
-          <t>September 2026 (lapse at fiscal-year start; reauthorized about two and a half weeks later, dated September 18 at M-7)</t>
+          <t>September 2026 (lapse at fiscal-year start; reauthorized about two weeks later, September 17 per the Texas Tribune; M-7 dates it September 18)</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
-          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): Fierce Healthcare's September 18, 2026 article (https://www.fiercehealthcare.com/providers/cms-restores-12b-frozen-supplemental-medicaid-funds) answered a Cloudflare challenge. The Texas Tribune limb matches (https://www.texastribune.org/2026/09/17/texas-medicaid-hospitals-greg-abbott-federal-impasse/, matched by script): the halt began Sept. 1, the start of Texas's fiscal year, in a dispute over how Texas raises the taxes, and about $12 billion was restored on Sept. 17 (16 days, so 'about two and a half weeks' is closer to 'about two weeks'). URL to open: https://www.fiercehealthcare.com/providers/cms-restores-12b-frozen-supplemental-medicaid-funds. Texas Tribune limb matches.</t>
+          <t>Monitored at M-7. The state is not named in the note or the series UPDATED September 27, 2026: the note now cites the Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) for this reference case. It still does not name the state in its text. Neither article was re-read for this ledger; re-reading both would support an upgrade UPDATED October 11, 2026: Pointer moved to sec. 9 item 5. v17 words the lapse as 'during a dispute over its provider tax calculation'. The state is still not named in the note. Previous wording: 'CMS decisions on SDP preprint approvals and renewals under existing authority can bring financing effects forward before either rule is final; in September 2026, one state's directed payment programs lapsed at the start of its fiscal year pending a dispute over provider tax calculation, and were authorized about two and a half weeks later' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Texas Tribune, September 17, 2026 (https://www.texastribune.org/2026/09/17/texas-medicaid-hospitals-greg-abbott-federal-impasse/), downloaded in the second pass and matched by script again. As instructed, the Fierce Healthcare half was not checked; the Fierce citation was removed from the Primary source and Exact citation columns, and 'about two and a half weeks' became 'about two weeks' in the Claim and Time horizon columns (September 1 to September 17 is 16 days).</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
         <is>
-          <t>single-source — two outlets now cited in the note but neither re-read for this ledger; the dollar detail rests on the reference case at M-7 — NEEDS VERIFICATION [DL3] Texas Tribune (September 17, 2026) and Fierce Healthcare (September 18, 2026) are on the decision-log re-check list (sec. 9 item 5); neither was re-read for this ledger. blocked: www.fiercehealthcare.com (site refused); re-checked October 13, 2026, second pass. Texas Tribune limb matches.</t>
+          <t>single-source — Texas Tribune, September 17, 2026, re-read; the Fierce Healthcare citation was dropped — re-checked October 14, 2026, third pass: Texas Tribune matches (halt began Sept. 1, the start of the state's fiscal year; dispute over how Texas raises the taxes; nearly $12 billion restored, announced Thursday, Sept. 17); 16 days is 'about two weeks'. Fierce Healthcare citation dropped and 'about two and a half weeks' changed to 'about two weeks', as instructed on October 14, 2026.</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="M46" s="12" t="inlineStr">
         <is>
-          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): medicaid.gov answered 'Access Denied' (Akamai, HTTP 403) for the SDP guidance page and the preprint template. URL to open: https://www.medicaid.gov/medicaid/managed-care/downloads/sdp-4386c-preprint-template.pdf.</t>
+          <t>Not read for this ledger or in the verification files; named in the change map as 'U-5' (the preprint's financing fields) and carried as an open re-check. Supports NC-18. VERIFIED October 14, 2026, third pass (verification_v4_log.md): SDP preprint template (user-supplied copy: de2d1011-Section_438.6c_Preprint.pdf), Section VI 'Funding for the Non-Federal Share', matched by script: Q34 asks the state to 'Check all that apply' among general revenue, IGTs, provider taxes, donations and other; Q35's Table 4 'IGT Transferring Entities' has a column 'Total Amounts Transferred by This Entity'; Q36's Table 5 'Health Care-Related Provider Tax/Assessment(s)' asks for the tax's name, class, broad-based, uniform, 6% and hold-harmless tests, and has no dollar column. Caveat: the copy is the January 2021 version of the template; a later revision was not checked.</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>single-source — the preprint form was not read in the verification files — NEEDS VERIFICATION [DL3] SDP preprint, Section VI (financing fields) is on the decision-log re-check list (sec. 7 step 3). blocked: www.medicaid.gov (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified with caveat — the template read is the January 2021 version — re-checked October 14, 2026, third pass: Preprint Section VI matches (user-supplied copy: de2d1011-Section_438.6c_Preprint.pdf, January 2021 version): Q34 sources by checkbox; Table 4 IGT dollars by transferring entity; Table 5 provider taxes with no dollar column.</t>
         </is>
       </c>
     </row>
@@ -10049,12 +10049,12 @@
       </c>
       <c r="M132" s="12" t="inlineStr">
         <is>
-          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
+          <t>No independent derivation located (SB-11, C-4); single publisher UPDATED October 11, 2026: v17 refers to the article only, not to a companion newsletter, and states the mismatch-of-bases reading as [I]. Previous wording: 'The $681B figure is arithmetic published by POLITICO on Sept 2, 2026, in a news article and companion newsletter' VERIFIED October 14, 2026, third pass (verification_v4_log.md): POLITICO, September 2, 2026 (user-supplied copy: c0ecf7f8-260902_POLITICO_Report.docx; the copy carries no date line or byline, so the date is the one in the file name and the request). Matched by script: the three sentences the row reports, in order. The ledger's Quote column lower-cases the first word ('or as hospitals see it'); the article starts the sentence with 'Or'.</t>
         </is>
       </c>
       <c r="N132" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — single publisher, no corroborating outlet located — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified with caveat — single publisher, no corroborating outlet located — re-checked October 14, 2026, third pass: POLITICO's text matches ($340 billion through 2034; $756 billion federal and $265 billion state savings through 2035; 'as hospitals see it', $681 billion more than expected).</t>
         </is>
       </c>
     </row>
@@ -10121,12 +10121,12 @@
       </c>
       <c r="M133" s="12" t="inlineStr">
         <is>
-          <t>Internal: 756 + 265 − 340 = 681 exactly BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
+          <t>Internal: 756 + 265 − 340 = 681 exactly VERIFIED October 14, 2026, third pass (verification_v4_log.md): POLITICO, September 2, 2026 (user-supplied copy: c0ecf7f8-260902_POLITICO_Report.docx; the copy carries no date line or byline, so the date is the one in the file name and the request). Matched by script.</t>
         </is>
       </c>
       <c r="N133" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: POLITICO's construction matches ($340 billion through 2034; $756 billion and $265 billion through 2035); 756 + 265 - 340 = 681.</t>
         </is>
       </c>
     </row>
@@ -10193,12 +10193,12 @@
       </c>
       <c r="M134" s="12" t="inlineStr">
         <is>
-          <t>The note relies on this phrase to avoid attributing the figure to any hospital association BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge (HTTP 403, cf-mitigated: challenge); the Yahoo Finance syndicated copy was refused by the network policy (finance.yahoo.com). URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch).</t>
+          <t>The note relies on this phrase to avoid attributing the figure to any hospital association VERIFIED October 14, 2026, third pass (verification_v4_log.md): POLITICO, September 2, 2026 (user-supplied copy: c0ecf7f8-260902_POLITICO_Report.docx; the copy carries no date line or byline, so the date is the one in the file name and the request). Matched by script.</t>
         </is>
       </c>
       <c r="N134" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: POLITICO's framing matches ('Or as hospitals see it').</t>
         </is>
       </c>
     </row>
@@ -11273,12 +11273,12 @@
       </c>
       <c r="M149" s="12" t="inlineStr">
         <is>
-          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): politico.com answered a Cloudflare challenge and cbo.gov a JavaScript bot check (HTTP 403). The CBO files mentioned in the request were not among the session's uploads (only the ledger md and xlsx and the v17 docx are there), so CBO's July 21, 2025 Table 7 was not read. URL to open: https://www.politico.com/search?q=%22%24681+billion%22+hospitals (article of September 2, 2026, 'Hospitals say coming Trump administration rules are worse than GOP's Medicaid cuts'; exact URL not found: politico.com is closed to this session's search tool and refused the fetch); https://www.cbo.gov/publication/61570.</t>
+          <t>Internal: 340.5 rounds to 340. The article's framing ('hospitals expected to lose $340 billion through 2034', SB-02) names no source. The match is [FIRM]'s identification, not the article's attribution. Replaces SB-08 UPDATED October 11, 2026: v17 words the first limb as a plain [I] search result ('names no source') and drops the clause 'attributes it to hospitals' expectations'. Source moved from CRS R48633 to CBO directly. Previous wording: 'The $340B matches, to rounding, CBO's $340.5B outlay estimate for Sections 71115 and 71116; the article attributes it to hospitals' expectations and does not name a source' PARTLY CHECKED October 14, 2026, third pass (verification_v4_log.md): POLITICO, September 2, 2026 (user-supplied copy: c0ecf7f8-260902_POLITICO_Report.docx; the copy carries no date line or byline, so the date is the one in the file name and the request). Matched by script: 'Hospitals expected to lose $340 billion through 2034 after Congress passed the One Big, Beautiful Bill Act last year.' A search of the copy finds no 'CBO' and no 'Congressional Budget Office', so 'names no source' holds. CBO limb pending part 2.</t>
         </is>
       </c>
       <c r="N149" s="12" t="inlineStr">
         <is>
-          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). blocked: www.politico.com; www.cbo.gov (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified as scoped - the match is arithmetic; 'names no source' is a reading of one article — NEEDS VERIFICATION [DL3] POLITICO, September 2, 2026 is on the decision-log re-check list (secs. 5–6; App. H). partly checked, CBO limb pending part 2; blocked: www.cbo.gov (site refused); re-checked October 14, 2026, third pass: POLITICO limb matches (user-supplied copy: c0ecf7f8-260902_POLITICO_Report.docx): the article gives the $340 billion with no source and never names CBO.</t>
         </is>
       </c>
     </row>
@@ -14513,12 +14513,12 @@
       </c>
       <c r="M194" s="12" t="inlineStr">
         <is>
-          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): gao.gov answered 'Access Denied' (Akamai, HTTP 403) for the product page and the PDF (https://www.gao.gov/assets/gao-24-106202.pdf). URL to open: https://www.gao.gov/products/gao-24-106202.</t>
+          <t>Not read in the verification files or for this ledger. The change map lists GAO-24-106202 Table 4 as an existing citation 'still open' (U-5). Supports NC-18. CORRECTED October 14, 2026, third pass (verification_v4_log.md): GAO-24-106202 (user-supplied copy: 4ba29095-GAO-24-106202.pdf), matched by script. Table 4 gives, by state, one column 'Nonfederal share from providers and local governments', which note a defines as provider taxes and intergovernmental transfers together, for directed payments approved as of August 26, 2022. GAO treated the whole nonfederal share as state general funds for the 25 payments financed partly by providers or local governments, 'As such, the total amount of the nonfederal share from providers and local governments is undercounted.' So the 2022 date matches, but the table does not give dollars by source.</t>
         </is>
       </c>
       <c r="N194" s="12" t="inlineStr">
         <is>
-          <t>single-source — not re-read in the review or for this ledger — NEEDS VERIFICATION [DL3] GAO-24-106202, Table 4 is on the decision-log re-check list (sec. 2). blocked: www.gao.gov (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>corrected — source says: “since states do not provide information on the amount of funds from each source of the nonfederal share” (GAO-24-106202, December 2023, app. III, Table 4, pp. 44–46, note a and footnote 2; user-supplied copy: 4ba29095-GAO-24-106202.pdf). v17 must change Sec. 2 (see verification_v4_log.md). Base status was single-source — not re-read in the review or for this ledger; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -15593,12 +15593,12 @@
       </c>
       <c r="M209" s="12" t="inlineStr">
         <is>
-          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4: 28 expansion states with a hospital tax, less CO, CT, IN and VT which have no hospital SDPs, = 24 exactly UPDATED October 11, 2026: v17 has no footnote 5; the table's source line says 'THEIA Services' grouping from KFF's August 2026 state file and Medicaid expansion tracker; KFF does not use these groups. The dollar column sums KFF's estimates for each group.' The group is labelled 'Both rules' and the table adds a column on which parts of the two rules reach the group. Minnesota and Missouri belong in Group A but have no KFF estimate (SE-14), so the $45.4B excludes them. The 28 less 4 arithmetic is unchanged. Previous wording: 'Group A: 24 expansion states with affected hospital SDPs and a hospital tax above 3.5%; approximately $45.4B above limits' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. 28 expansion states have a hospital tax above 3.5% in the appendix table; CO, CT, IN and VT have no hospital SDPs on the map, leaving 24. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N209" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: KFF's chart data match: 24 expansion states with hospital SDPs likely affected and a hospital tax above 3.5% (Minnesota and Missouri included, no dollar estimate), $45.43 billion above the caps.</t>
         </is>
       </c>
     </row>
@@ -15665,12 +15665,12 @@
       </c>
       <c r="M210" s="12" t="inlineStr">
         <is>
-          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4: both expansion, both hospital tax No, both with measured shares (0.7209 and 0.5801) UPDATED October 11, 2026: v17 labels the group 'Cap plus lower threshold on non-hospital taxes' and says the lower threshold reaches ambulance or other taxes, not hospital taxes. The earlier ledger wording 'SDP cap plus a non-hospital tax class' is the same content. Previous wording: 'Group B: Washington and West Virginia; approximately $2.0B' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. Washington $1,391,768,801 and West Virginia $567,162,829 above the limits. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N210" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: KFF's chart data match: Washington and West Virginia have hospital SDPs likely affected, $1.96 billion above the caps, and only ambulance or other taxes above 3.5%.</t>
         </is>
       </c>
     </row>
@@ -15737,12 +15737,12 @@
       </c>
       <c r="M211" s="12" t="inlineStr">
         <is>
-          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4: all three expansion, hospital tax No, shares 1.0000 / 0.9649 / 0.8042 UPDATED October 11, 2026: v17 adds the qualifier 'other than nursing or intermediate care facility taxes', which are exempt from the lower threshold (RM-29). C4 shares are unchanged. The qualifier is not checkable from the C4 outputs. Previous wording: 'Group C: DC, Delaware and Hawaii; approximately $0.8B' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. DC $376,029,678, Delaware $175,574,794, Hawaii $247,941,877. The appendix table's note says nursing and intermediate care facility taxes are exempt, which checks v17's qualifier. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N211" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: KFF's chart data match: DC, Delaware and Hawaii have hospital SDPs likely affected, $0.80 billion above the caps, and no non-exempt tax above 3.5% (nursing and ICF taxes are exempt).</t>
         </is>
       </c>
     </row>
@@ -15809,12 +15809,12 @@
       </c>
       <c r="M212" s="12" t="inlineStr">
         <is>
-          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4: 10 non-expansion states less Alabama and Wyoming, both determined-zero on SDPs, = 8 exactly UPDATED October 11, 2026: v17 says the phase-down reaches Group D (RM-03: the phase-down applies in every state) and that the lower threshold does not (RM-08). The earlier measure line, 'threshold phase-down does not', used 'phase-down' for the tax threshold; see SE-18. Previous wording: 'Group D: 8 non-expansion states with affected SDPs (FL, GA, KS, MS, SC, TN, TX, WI); approximately $11.9B' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. The appendix table marks non-expansion states 'N/A, non-expansion state'. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N212" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>verified — re-checked October 14, 2026, third pass: KFF's chart data match: FL, GA, KS, MS, SC, TN, TX and WI are the eight non-expansion states with hospital SDPs likely affected, $11.91 billion above the caps; Alabama and Wyoming have no managed care.</t>
         </is>
       </c>
     </row>
@@ -15881,12 +15881,12 @@
       </c>
       <c r="M213" s="12" t="inlineStr">
         <is>
-          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure' CORRECTED October 13, 2026, second pass (verification_v4_log.md): KFF, Aug 14, 2026 brief (https://www.kff.org/medicaid/at-least-37-states-have-medicaid-state-directed-payments-for-hospital-services-that-could-be-reduced-by-the-2025-reconciliation-law-limits/), matched by script: KFF also notes Colorado submitted the SDP on June 27, 2025 (about $378 million) and that CMS posted it after KFF's cut-off. The 14-state list and the other limbs rest on KFF's chart data, which is on datawrapper.dwcdn.net (refused by the network policy).</t>
+          <t>C4: exactly 14 rows flagged "n/a (no SDPs)" or "n/a (no hospital SDPs)" — AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY. Groups A–E total 51, matching 50 states plus DC UPDATED October 11, 2026: v17 labels the group 'No identified hospital SDPs above the caps' and gives the dollar column as $0. The 14-state list and the 51-jurisdiction total are unchanged. Previous wording: 'Group E: 14 states with no identified hospital SDP exposure' CORRECTED October 14, 2026, third pass (verification_v4_log.md): Second-pass correction (Colorado) stands. Remaining limbs checked against KFF's chart data: Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. The 14 Group E states are exactly AL, AK, AR, CO, CT, ID, IN, ME, MD, MT, ND, SD, VT, WY, with no dollars above the limits in Figure 4. New: KFF's provider-tax appendix table (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv) lists Arkansas, an expansion state in Group E, with a non-exempt ambulance tax of 5.51%-6.0%, and KFF's map (https://datawrapper.dwcdn.net/m5vRC/2/dataset.csv) marks it 'AR*' with 'Affected tax(es): ambulance'. The lower threshold therefore reaches Arkansas as well as CO, CT, IN and VT. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N213" s="12" t="inlineStr">
         <is>
-          <t>corrected — source says: “Colorado also has an SDP that is above new limits, but CMS did not post the preprint publicly until after July 20, 2026.” (KFF, Aug 14, 2026, Figure 1 note). v17 must change Sec. 6 (see verification_v4_log.md). Base status was verified. Other limbs: NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy).</t>
+          <t>corrected — source says: “Colorado also has an SDP that is above new limits, but CMS did not post the preprint publicly until after July 20, 2026.” (KFF, Aug 14, 2026, Figure 1 note). v17 must change Sec. 6 (see verification_v4_log.md). Base status was verified; re-checked October 14, 2026, third pass. Also, KFF's provider-tax table says “Arkansas Yes Ambulance (5.51%-6.0%)” (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv): the lower threshold reaches Arkansas too.</t>
         </is>
       </c>
     </row>
@@ -15953,12 +15953,12 @@
       </c>
       <c r="M214" s="12" t="inlineStr">
         <is>
-          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
+          <t>C4: all four are expansion states with hospital_tax_above_3_5 = Yes and no hospital SDPs. This is the correction recorded at decision log B-8 UPDATED October 11, 2026: v17 replaces 'the phase-down reaches all four' with 'the lower threshold reaches' (the tax limit; 'phase-down' now means the SDP phase-down) and tags the sentence [I]. The same sentence adds that two Group E states carry KFF data-quality flags (SE-20). The reading rests on C4's hospital_tax_above_3_5 indicator. Previous wording: 'Group E is not a no-exposure group: Colorado, Connecticut, Indiana and Vermont are expansion states with a hospital tax above 3.5%, so the phase-down reaches all four' CORRECTED October 14, 2026, third pass (verification_v4_log.md): The four named states match the appendix table: Colorado, Connecticut and Vermont 'Hospital (5.51%-6.0%)', Indiana 'Hospital (3.51%-5.5%)', all expansion states without hospital SDPs on the Figure 1 map. But the list is incomplete: KFF's provider-tax appendix table (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv) lists Arkansas, an expansion state in Group E, with a non-exempt ambulance tax of 5.51%-6.0%, and KFF's map (https://datawrapper.dwcdn.net/m5vRC/2/dataset.csv) marks it 'AR*' with 'Affected tax(es): ambulance'. The lower threshold therefore reaches Arkansas as well as CO, CT, IN and VT. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N214" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
+          <t>corrected — source says: “Arkansas Yes Ambulance (5.51%-6.0%)” (KFF, Aug 20, 2026, provider-tax appendix table (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv)). v17 must change Sec. 6 (see verification_v4_log.md). Base status was verified; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -16097,12 +16097,12 @@
       </c>
       <c r="M216" s="12" t="inlineStr">
         <is>
-          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): Texas limb matches the brief's text ('Texas ($3.5 billion)', matched by script); the Tennessee, Georgia and South Carolina amounts are only in the Figure 4 chart data on datawrapper.dwcdn.net, refused by the network policy. URL to open: https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/D5jCd/.</t>
+          <t>Not re-derivable: C4 carries shares, not dollars. The relative ordering is consistent with C4's shares (TX 0.7058, TN 0.7581, GA 0.7608, SC 0.9195) UPDATED October 11, 2026: v17 moves the state dollars from sec. 6 to App. H (change map U31) and words them 'more than $1.6 billion each' (previously 'above'). Still not re-derivable from C4, which carries shares. Previous wording: 'Group D contains Texas at $3.5B above limits, and Tennessee, Georgia and South Carolina above $1.6B each' VERIFIED October 14, 2026, third pass (verification_v4_log.md): KFF Figure 4 data, matched by script; the brief's text gives 'Texas ($3.5 billion)'. Each of the three is above $1.6 billion. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N216" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>single-source — re-checked October 14, 2026, third pass: KFF's chart data match: Texas $3.48 billion; Georgia $2.17 billion, Tennessee $1.95 billion, South Carolina $1.65 billion above the limits.</t>
         </is>
       </c>
     </row>
@@ -16169,12 +16169,12 @@
       </c>
       <c r="M217" s="12" t="inlineStr">
         <is>
-          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before. BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4 deliverable reproduces this exactly: FL, KS, MS = INSUFFICIENT; GA, SC, TN, TX, WI = PARTIAL UPDATED October 11, 2026: v17 moves the flag list to App. H (change map T32) and keeps 'all eight states carry KFF data-quality flags' in sec. 6, tagged within the [I] sentence 'Group D's dollar figures are the least reliable'. KFF flags insufficient data in Florida, Kansas and Mississippi and partial data in Georgia, South Carolina, Tennessee, Texas and Wisconsin, as before. CORRECTED October 14, 2026, third pass (verification_v4_log.md): KFF's brief and its chart data (Figure 1, Figure 4 and the provider-tax table, with their notes) carry no INSUFFICIENT or PARTIAL label for any state; those labels come from the analyst's C4 file. KFF's Methods name the states whose missing payment rates it imputed: state-specific rates for Georgia, Kentucky, Louisiana, New Mexico, Nevada, New York, Pennsylvania and Washington; national rates for Arizona, California, Hawaii, Illinois, Texas and Wisconsin. So among Group D only Georgia, Texas and Wisconsin have imputed rates. Separately, the August 20, 2026 provider-tax brief says FL, KS and MS did not respond to the 2025 survey (SE-11). Searched by script for 'insufficient', 'partial' and 'data quality' in the brief and the chart pages: only Datawrapper's page code and the Minnesota and Missouri note. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N217" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>corrected — source says: “For the remaining states, KFF had complete payment rate information from the preprints.” (KFF, Aug 14, 2026, Methods). v17 must change Sec. 6 and App. H (see verification_v4_log.md). Base status was verified; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -16673,12 +16673,12 @@
       </c>
       <c r="M224" s="12" t="inlineStr">
         <is>
-          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/.</t>
+          <t>C4: AL and WY carry 'PARTIAL / DETERMINED ZERO' (SE-19). The inference that the zero partly reflects data limits is [FIRM]'s UPDATED October 11, 2026: v17 gives the flag detail in App. H, tags it [I], and in sec. 6 says only that 'two Group E states carry KFF data-quality flags'. The twelve-state count at SE-19 is no longer a note claim. Previous wording: 'Group E includes Alabama and Wyoming, whose records carry data-quality flags, so 'no identified exposure' partly reflects limited data there' CORRECTED October 14, 2026, third pass (verification_v4_log.md): KFF publishes no data-quality flag for Alabama or Wyoming (see SE-13); the 'PARTIAL / DETERMINED ZERO' labels are the analyst's C4 file. KFF's Figure 1 data mark both 'No managed care', and SDPs are directions to managed care plans, so the $0 reflects the absence of managed care, not limited data. Neither state is among those whose rates KFF imputed. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N224" s="12" t="inlineStr">
         <is>
-          <t>verified — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass.</t>
+          <t>corrected — source says: “states can implement SDPs that require MCOs to increase rates or set minimum rates for specified Medicaid services” (KFF, Aug 14, 2026; Figure 1 data list Alabama and Wyoming as 'No managed care' (https://datawrapper.dwcdn.net/ZdNkK/23/dataset.csv)). v17 must change Sec. 6 and App. H (see verification_v4_log.md). Base status was verified; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -17609,12 +17609,12 @@
       </c>
       <c r="M237" s="12" t="inlineStr">
         <is>
-          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): gao.gov answered 'Access Denied' (Akamai, HTTP 403) for the product page and the PDF (https://www.gao.gov/assets/gao-23-105515.pdf). URL to open: https://www.gao.gov/products/gao-23-105515.</t>
+          <t>GAO is synthesising published research rather than reporting an original count, and the note's verb was corrected to 'reported that research indicates' to match. The underlying studies were not retrieved. Data window ends 2018, seven years before either rule UPDATED October 11, 2026: v17 words the attribution 'GAO reported research showing' and the verb 'fell'; the attribution is unchanged in substance (GAO is synthesising published research, not reporting an original count). Previous wording: 'GAO reported that research indicates the number of rural hospitals providing obstetric services declined from 2004 through 2018, and that by 2018 more than half of rural counties had no hospital offering obstetric services' VERIFIED October 14, 2026, third pass (verification_v4_log.md): GAO-23-105515 (user-supplied copy: 313cff62-GAO-23-105515.pdf), Highlights page, matched by script: 'Research indicates that the number of rural hospitals providing obstetric services declined from 2004 through 2018, and more than half of rural counties did not have such services in 2018'. GAO adds 'according to the most recent data available'. v17's 'GAO reported research showing' and 'fell' carry the same meaning; the caveat (GAO reports others' research; window predates both rules) stands.</t>
         </is>
       </c>
       <c r="N237" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — NEEDS VERIFICATION [DL3] GAO-23-105515 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: www.gao.gov (site refused); re-checked October 13, 2026, second pass.</t>
+          <t>verified with caveat - GAO is reporting others' research, and the window predates both rules — re-checked October 14, 2026, third pass: GAO's Highlights match (user-supplied copy: 313cff62-GAO-23-105515.pdf): research indicates rural hospitals providing obstetric services declined 2004-2018, and more than half of rural counties had none in 2018.</t>
         </is>
       </c>
     </row>
@@ -17681,12 +17681,12 @@
       </c>
       <c r="M238" s="12" t="inlineStr">
         <is>
-          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): The PubMed connector was tried first and again returned no full text for PMC11612914 (abstract only: 'This cross-sectional study evaluates recent trends in pediatric inpatient capacity …'); jamanetwork.com answered a Cloudflare challenge; pmc.ncbi.nlm.nih.gov was refused by the network policy. URL to open: https://jamanetwork.com/journals/jamapediatrics/fullarticle/2826774; https://pmc.ncbi.nlm.nih.gov/articles/PMC11612914/. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
+          <t>Internal: the adult comparison is what makes the pediatric figures a claim about pediatric capacity specifically rather than about inpatient capacity generally. No corroborating source located, and the paper was not retrieved for this ledger. Data window ends 2022, three years before the reconciliation law UPDATED October 11, 2026: v17 words the attribution 'A national study found'; the Figure 7 caption says 'in one national study'. Figures unchanged. Previous wording: 'A national study of pediatric inpatient capacity found units down 29.9 percent and beds down 19.5 percent from 2008 to 2022, against a 4.4 percent decline in adult units over the same period' VERIFIED October 14, 2026, third pass (verification_v4_log.md): Michelson et al., 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics, published online December 2, 2024, 2025;179(2):208-209 (user-supplied copy: 2962057f-National_Trends_in_Pediatric_Inpatient_...trics___JAMA_Pediatrics___JAMA_Network.pdf), Results, matched by script. PMC was not needed: the attached copy was used. Adult beds fell 3.0%; v17 does not use the adult bed series.</t>
         </is>
       </c>
       <c r="N238" s="12" t="inlineStr">
         <is>
-          <t>single-source — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (change map 'Re-check list', sec. 8): no verification row covers it. blocked: jamanetwork.com (site refused); re-checked October 13, 2026, second pass. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
+          <t>single-source — one study, read in full — re-checked October 14, 2026, third pass: Michelson et al. match (user-supplied copy: 2962057f-National_Trends_in_Pediatric_Inpatient_...trics___JAMA_Pediatrics___JAMA_Network.pdf): pediatric units -29.9%, beds -19.5%, adult units -4.4%, 2008-2022.</t>
         </is>
       </c>
     </row>
@@ -20129,12 +20129,12 @@
       </c>
       <c r="M272" s="12" t="inlineStr">
         <is>
-          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): KFF's brief (kff.org, read) gives national totals only; the state-level figures behind the groups (which states are above the caps and by how much, data-quality flags, and which states have taxes above 3.5 percent) are in the brief's Datawrapper charts, and the network policy refused datawrapper.dwcdn.net. KFF's expansion tracker (read) lists 41 adopting states including DC and 10 not adopting. URL to open: https://datawrapper.dwcdn.net/ZdNkK/; https://datawrapper.dwcdn.net/UbS1f/; https://datawrapper.dwcdn.net/7EcOI/. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
+          <t>Counts at SE-05 to SE-10, SE-13, SE-19; dollar panel at SE-12; Group E note at SE-10. The 12 flagged states on the map (the 10 non-expansion states plus MN and MO) match SE-19 UPDATED October 11, 2026: v17 carries only the caption. The earlier title ('State Medicaid hospital financing exposure to two proposed CMS rules') and the 'data quality flag 12 states' layer are not in v17 (SE-19 is superseded); the map note that Colorado, Connecticut, Indiana and Vermont are reached by 'the phase-down' now reads 'the lower threshold' (SE-10). Counts at SE-05 to SE-10; the dollar panel at SE-12 (single-source); the group definitions are THEIA Services' (SE-17). The artwork was not supplied. Previous wording: 'Figure 6. "State Medicaid hospital financing exposure to two proposed CMS rules." Values: Group A 24 states; B 2; C 3; D 8; E 14; non-expansion states 10 (heavy boundary); data quality flag 12 states. Panel: Texas $3.5B above limits; Tennessee, Georgia and South Carolina above $1.6B each; CO, CT, IN, VT reached by the phase-down' CORRECTED October 14, 2026, third pass (verification_v4_log.md): Counts match KFF's chart data: Groups rebuilt by script (kffgroups.py) from the Figure 1 map (37 'Hospital SDPs likely affected'), the Figure 4 dollars, the provider-tax appendix table and KFF's expansion tracker (41 adopting jurisdictions including DC, 10 not adopting): A 24 ($45.43B; Minnesota and Missouri have no dollar estimate), B 2 ($1.96B), C 3 ($0.80B), D 8 ($11.91B), E 14 ($0); 51 in all, $60.1B. Non-expansion states: 10. Dollar panel matches (SE-12). But KFF's provider-tax appendix table (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv) lists Arkansas, an expansion state in Group E, with a non-exempt ambulance tax of 5.51%-6.0%, and KFF's map (https://datawrapper.dwcdn.net/m5vRC/2/dataset.csv) marks it 'AR*' with 'Affected tax(es): ambulance'. The lower threshold therefore reaches Arkansas as well as CO, CT, IN and VT. Colorado's SDP above the new limits (SE-09) also affects the Group E layer. Retrieval: each chart's base URL (https://datawrapper.dwcdn.net/&lt;id&gt;/) answers with a meta-refresh to its current version; the versioned page and its dataset.csv were downloaded with curl on October 14, 2026 and matched by script.</t>
         </is>
       </c>
       <c r="N272" s="12" t="inlineStr">
         <is>
-          <t>verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source — NEEDS VERIFICATION [DL3] KFF, August 14, 2026 (state file, expansion tracker, $155 billion) is on the decision-log re-check list (secs. 5–6; App. H); this row rests on it. blocked: datawrapper.dwcdn.net (network policy); re-checked October 13, 2026, second pass. Knock-on of SE-09: KFF says Colorado, a Group E state, has an SDP above the new limits.</t>
+          <t>corrected — source says: “Arkansas Yes Ambulance (5.51%-6.0%)” (KFF, Aug 20, 2026, provider-tax appendix table (https://datawrapper.dwcdn.net/q3dXL/7/dataset.csv)). v17 must change Figures (see verification_v4_log.md). Base status was verified with caveat — caption only in v17; artwork not supplied; dollar panel rests on SE-12, which is single-source; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -20201,12 +20201,12 @@
       </c>
       <c r="M273" s="12" t="inlineStr">
         <is>
-          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)' BLOCKED AGAIN October 13, 2026, second pass (verification_v4_log.md): The PubMed connector was tried first and again returned no full text for PMC11612914 (abstract only: 'This cross-sectional study evaluates recent trends in pediatric inpatient capacity …'); jamanetwork.com answered a Cloudflare challenge; pmc.ncbi.nlm.nih.gov was refused by the network policy. URL to open: https://jamanetwork.com/journals/jamapediatrics/fullarticle/2826774; https://pmc.ncbi.nlm.nih.gov/articles/PMC11612914/. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
+          <t>Internal: 100 − 29.9 = 70.1; 100 − 19.5 = 80.5; 100 − 4.4 = 95.6, matching AC-10. Single source, as the figure states UPDATED October 11, 2026: v17 carries only the caption, which now says 'units fell faster than adult units' where the earlier title said 'capacity fell faster than adult capacity'; the caption no longer claims pediatric beds against adult beds, consistent with the absence of an adult bed series. Values unchanged (AC-10); artwork not supplied. Previous wording: 'Figure 7. "Pediatric inpatient capacity fell faster than adult capacity" (caption adds "2008 to 2022"). Values: index 2008 = 100; 2022 pediatric units 70.1, pediatric beds 80.5, adult units 95.6 (no adult bed series in source)' CORRECTED October 14, 2026, third pass (verification_v4_log.md): Michelson et al., 'National Trends in Pediatric Inpatient Capacity', JAMA Pediatrics, published online December 2, 2024, 2025;179(2):208-209 (user-supplied copy: 2962057f-National_Trends_in_Pediatric_Inpatient_...trics___JAMA_Pediatrics___JAMA_Network.pdf), Results, matched by script. PMC was not needed: the attached copy was used. The three index values follow from the paper: 100 - 29.9 = 70.1, 100 - 19.5 = 80.5, 100 - 4.4 = 95.6. But the Claim column's '(no adult bed series in source)' differs from the paper, which reports adult beds falling 3.0%.</t>
         </is>
       </c>
       <c r="N273" s="12" t="inlineStr">
         <is>
-          <t>single-source - one study (AC-10); caption only in v17 — NEEDS VERIFICATION [DL3] Michelson et al., December 2024 is on the decision-log re-check list (sec. 8); the figure rests on AC-10. blocked: jamanetwork.com (site refused); re-checked October 13, 2026, second pass. pmc.ncbi.nlm.nih.gov also refused (network policy).</t>
+          <t>corrected — source says: “Adult inpatient units decreased from 4519 to 4318, declining 4.4% (95% CI, 0.4%-8.4%), and beds decreased from 405 908 to 393 802” (Michelson et al., JAMA Pediatrics, Dec 2, 2024, Results; user-supplied copy: 2962057f-National_Trends_in_Pediatric_Inpatient_...trics___JAMA_Pediatrics___JAMA_Network.pdf). v17 must change Figures (see verification_v4_log.md). Base status was single-source - one study (AC-10); caption only in v17; re-checked October 14, 2026, third pass.</t>
         </is>
       </c>
     </row>
@@ -20506,11 +20506,11 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Flag at the end of the Status column: the item is on the decision log's re-check list or the change map's lists. [DL3] re-check list; [DL4] comment ID to verify; [CM] Federal Register pinpoint from the new-text check. Shaded orange. The base status stands. After the October 13, 2026 check, a flag that remains ends with 'not found' or 'blocked: &lt;host&gt;', and after the second pass the host is followed by '(site refused)', '(login)' or '(network policy)'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="150" customHeight="1" s="10">
+          <t>Flag at the end of the Status column: the item is on the decision log's re-check list or the change map's lists. [DL3] re-check list; [DL4] comment ID to verify; [CM] Federal Register pinpoint from the new-text check. Shaded orange. The base status stands. After the October 13, 2026 check, a flag that remains ends with 'not found' or 'blocked: &lt;host&gt;', and after the second pass the host is followed by '(site refused)', '(login)' or '(network policy)'. After the October 14, 2026 third pass, 'partly checked' marks a row with one limb checked and another still pending; its flag stays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="230" customHeight="1" s="10">
       <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Coverage caveat</t>
@@ -20518,7 +20518,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Updated October 13, 2026. Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. All 91 flagged rows were checked, in order: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list, the unresolved row AC-14. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text, except four rows on one journal article read through the PubMed connector (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 58 rows match and lose the flag (25 upgraded, for example single-source to verified); 12 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 21 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 1 rows with two tags were resolved for one tag only and keep the other tag's flag. No row text other than the Cross-check and Status columns was changed. A second pass the same day, after the network policy was opened, re-ran the 47 rows blocked in the first pass: 24 now match, 4 are corrected and 19 stay blocked (politico.com, fiercehealthcare.com, jamanetwork.com, gao.gov, medicaid.gov and cbo.gov refused at the site; datawrapper.dwcdn.net, which serves KFF's state-level chart data, was refused by the network policy); the figures above include it. A remaining flag now ends 'blocked: &lt;host&gt; (site refused)', '(login)' or '(network policy)'. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
+          <t>Updated October 13, 2026, and on October 14, 2026 (third pass, part 1). Verification of the NEEDS VERIFICATION rows; details in verification_v4_log.md. All 91 flagged rows were checked, in order: [CM] Federal Register pinpoints, [DL4] comment IDs, [DL3] re-check list, the unresolved row AC-14. Each claim was compared with the primary source the row names, and every quotation and matched phrase was found by script in the downloaded text, except four rows on one journal article read through the PubMed connector (Federal Register and statute: govinfo.gov PDFs and HTML, with OCR for tables printed as images; comments: regulations.gov API and attachments). Outcome: 70 rows match and lose the flag (26 upgraded, for example single-source to verified); 18 differ and are marked corrected, with the source's wording (24 words or fewer), the pinpoint and what v17 must change; 3 keep the flag with 'blocked: &lt;host&gt;' or 'not found'. 1 row was checked in part only and keeps the flag for the rest (SB-18). No row text other than the Cross-check and Status columns was changed, except RM-25, whose Claim, Primary source, Exact citation and Time horizon were edited on October 14, 2026 as instructed (citation moved from Fierce Healthcare to the Texas Tribune, September 17, 2026; 'about two and a half weeks' changed to 'about two weeks'). A second pass on October 13, after the network policy was opened, re-ran the 47 rows blocked in the first pass: 24 now match, 4 are corrected and 19 stay blocked (politico.com, fiercehealthcare.com, jamanetwork.com, gao.gov, medicaid.gov and cbo.gov refused at the site; datawrapper.dwcdn.net, which serves KFF's state-level chart data, was refused by the network policy); the figures above include it. A remaining flag now ends 'blocked: &lt;host&gt; (site refused)', '(login)' or '(network policy)'. A third pass on October 14, 2026 (part 1 of 2) re-ran the 19 rows still blocked and SE-09's remaining limbs: copies the user supplied of the POLITICO article (September 2, 2026), GAO-24-106202, GAO-23-105515, the SDP preprint template and Michelson et al. (JAMA Pediatrics) were read and matched by script, and KFF's state-level chart data were downloaded from datawrapper.dwcdn.net; 12 now match, 7 are corrected, and SB-18 is partly checked, its CBO limb pending part 2; the figures above include it. The appendix title line now names THEIA Services instead of the [FIRM] placeholder.</t>
         </is>
       </c>
     </row>

</xml_diff>